<commit_message>
Added a new UI flow
</commit_message>
<xml_diff>
--- a/results/questions_answers.xlsx
+++ b/results/questions_answers.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C169"/>
+  <dimension ref="A1:C113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,12 +453,15 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ANTARES VISION.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company have a human rights policy or a code of conduct commiting to respect human rights?', 'context': [Document(id='bebc898a-2b45-453e-81c9-c8275f7216bf', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content='document.  \nLastly, specific methods have been adopted for checking the compliance of the behaviour of anyone acting on their own \nbehalf or within their work context, with the provisions of current legislation and with the rules of conduct established by the \npolicies and procedures adopted. \n \nHuman rights \n \nIn continuity with its values, the commitment defined in the Code of Ethics, AV Group adopted a specific Human Rights Policy'), Document(id='64506eca-5a57-410a-ad35-cfb7169ad920', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 48, 'page_label': '49'}, page_content="Sustainability report / NFR 2022 49 \n \n \nThe Human Rights policy of Antares Vision Group was drawn up starting from the identification of the potentially most \nvulnerable elements within its value chain, t o ensure full respect for the human rights of all individuals connected to the \nGroup's activities. The policy regulates behaviours and establishes the position of AV Group in relation to topics such as"), Document(id='5cb5e9ba-82dc-4639-8cfc-569ad2309e57', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="With the adoption of the Human Rights policy, which applies to all AV Group companies and provides for specific metho ds \nof implementation, employee training and monitoring, the Group intends to:  \n▪ strengthen its commitment to the protection of human rights in each country in which it operates,  \n▪ demonstrate the Group's awareness of the risks inherent in its business model, \n▪ promote the contents of the policy among its external stakeholders as well.")], 'answer': 'Antares Vision Group has both a Human Rights Policy and a Code of Ethics that commit to respecting human rights.'}</t>
+          <t>Question: Does the company have a human rights policy or a code of conduct committing to respect human rights?
+Answer: Yes
+Evidence: "Alerion’s exclusive focus on renewable energy implies that sustainability is strictly embedded in our business model."
+Location: Page 1, Section "Introduction"</t>
         </is>
       </c>
     </row>
@@ -470,19 +473,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company have a human rights policy or a code of conduct commiting to respect human rights?', 'context': [Document(id='c82bcb4f-0397-45f0-acbf-8ae562c05023', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 124, 'page_label': '123'}, page_content='ning the principles and standards of conduct required by all suppliers and business partners \nwith respect to the areas of business ethics, compliance, anti-corruption, human rights and \nworkers’ rights, diversity and inclusion, health, safety, the environment, etc.37.\nDuring the year, the mandatory acceptance of this Code was included in the qualification \nprocess for new suppliers, so that any new supplier signs up to it and its proactive imple -'), Document(id='67882b1c-f6ec-4a98-b1cf-143f28a4567a', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 124, 'page_label': '123'}, page_content='ciples of freedom and dignity of people and fundamental human rights, the exploitation of \nforced and child labor, as well as any form of personal discrimination. In support of this, since \n2019 all suppliers of hearing aids, whose contracts are subject to periodic renegotiation, are \nrequired to recognize and comply with the principles set forth in Amplifon’s Sustainability \nPolicy. In addition, at the start of 2022 a new Supplier Code of Conduct was adopted, defi-'), Document(id='a0026abd-c35d-47a4-a24f-0ab156e90b95', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 75, 'page_label': '74'}, page_content='WELL-BEING AND INTERNAL ENGAGEMENT \nIn line with the UN Global Compact principles, the Universal Declaration of Human Rights, \nand in compliance with the International Labor Organization Conventions on Fundamental \nHuman Rights, Amplifon is committed to complying with the fundamental human rights \nand labor rights in all the countries where we operate , both in business activities and \nunder the scope of relations with third parties, renouncing to all forms of exploitative for -')], 'answer': 'Amplifon: Yes, Amplifon commits to respecting human rights through its Sustainability Policy and has adopted a new Supplier Code of Conduct that aligns with international human rights standards.'}</t>
+          <t>Question: Does the company have a human rights policy or a code of conduct committing to respect human rights?
+Answer: Yes
+Evidence: "AV Group adopted a specific Human Rights Policy."
+Location: Sustainability report / NFR 2022, page 49</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Does the company have a human rights policy or a code of conduct commiting to respect human rights?</t>
+          <t>Is the human right policy approved by the highest governance body?</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -492,7 +498,10 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company have a human rights policy or a code of conduct commiting to respect human rights?', 'context': [Document(id='1603dfa0-95cf-4193-b970-a97988e35cc1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 1, 'page_label': '2'}, page_content='further in Europe, both in \nwind and solar sector. \n Alerion’s exclusive focus \non renewable energy \nimplies that sustainability \nis strictly embedded in our \nbusiness model. Our \noperations contribute \ndirectly to the reduction of \ngreenhouse gas (GHG) \nemissions and to the \npromotion of a system for \nsustainable territorial \ndevelopment. To this end, \nwe have in place a strong \nintegrated system for the \nassessment and \nmanagement of our'), Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='d92ded8b-d43e-4c82-bbff-33a71d9d335f', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 2, 'page_label': '3'}, page_content="In particular, over the next years, Alerion will focus its strategy on the acceleration of \ngrowth with an increasingly broad geographical diversification in Italy, Spain and \nRomania, and on technological diversification, through a plan of investments in the solar \nsector. \n2- GREEN BOND FRAMEWORK \nIn order to increase transparency of the Alerion Green Bond 20 21 - 2027, Alerion has \npublished the “Alerion 2021 Green Bond Framework” in line with ICMA's Green Bond")], 'answer': "Alerion's provided context does not mention a human rights policy or code of conduct committing to respect human rights. It focuses on their renewable energy strategy and green bond framework. Therefore, whether such a policy exists is not clear from the given information."}</t>
+          <t>Question: Is the human right policy approved by the highest governance body?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided text.
+Location: Not specified</t>
         </is>
       </c>
     </row>
@@ -509,82 +518,97 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>{'input': 'Is the human right policy approved by the highest governance body?', 'context': [Document(id='a5d4344c-bcff-442c-b0c1-8d73418a53a6', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="on 31 Jan uary 2023. This choice intends to reaffirm the importance of respect for human rights and strengthen the AV \nGroup's commitment to safeguarding them, in every country in which it operates. \n \nThe policy, available on the Antares Vision Group website  (Company Documents | Group Policies), has been developed in \naccordance with the main international human rights conventions, standards and recommendations (International Bill of"), Document(id='64506eca-5a57-410a-ad35-cfb7169ad920', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 48, 'page_label': '49'}, page_content="Sustainability report / NFR 2022 49 \n \n \nThe Human Rights policy of Antares Vision Group was drawn up starting from the identification of the potentially most \nvulnerable elements within its value chain, t o ensure full respect for the human rights of all individuals connected to the \nGroup's activities. The policy regulates behaviours and establishes the position of AV Group in relation to topics such as"), Document(id='bebc898a-2b45-453e-81c9-c8275f7216bf', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content='document.  \nLastly, specific methods have been adopted for checking the compliance of the behaviour of anyone acting on their own \nbehalf or within their work context, with the provisions of current legislation and with the rules of conduct established by the \npolicies and procedures adopted. \n \nHuman rights \n \nIn continuity with its values, the commitment defined in the Code of Ethics, AV Group adopted a specific Human Rights Policy')], 'answer': "Antares Vision Group's context, the document does not specify whether the human rights policy was approved by the highest governance body."}</t>
+          <t>Question: Is the human rights policy approved by the highest governance body?
+Answer: Yes
+Evidence: "The Human Rights policy of Antares Vision Group was drawn up starting from the identification of the potentially most vulnerable elements within its value chain..."
+Location: Sustainability report / NFR 2022, page 49</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Is the human right policy approved by the highest governance body?</t>
+          <t>Did the company involve critical stakeholders in the development of the Human Rights policy?</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>{'input': 'Is the human right policy approved by the highest governance body?', 'context': [Document(id='603f8281-6cc4-4632-8982-0fe5185df252', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 185, 'page_label': '184'}, page_content='section 4 “Board of Directors”\n2-11: Chair of the highest governance body p. 152; 153\n2-12: Role of the highest governance body\nin overseeing the management of impacts\nReport on Corporate Governance and \nownership structure at 31 December 2022, \nsection 4 “Board of Directors”\n2-13: Delegation of responsibilities for managing impacts\np. 30; Report on Corporate Governance \nand ownership structure at 31 December \n2022, section 4 “Board of Directors”\n2-14: Role of the highest governance body'), Document(id='06e99e70-ce08-469b-b3a3-9e2d601fdfcf', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='and management methods, as well as the GRI Standards reported are described.\nArea Principle Reference GRI Standards\nHuman Rights\n1. Business should support and \nrespect the protection of human rights \nproclaimed at an international level\n2. Businesses should ensure that they are \nnot complicit in violations of human rights\n• Well-being and internal engagement\n• Business ethics and fighting corruption\n• Procurement and Supply Chain \nmanagement\n• Note on methodology\n• GRI 2-23: Policy commitment'), Document(id='a0026abd-c35d-47a4-a24f-0ab156e90b95', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 75, 'page_label': '74'}, page_content='WELL-BEING AND INTERNAL ENGAGEMENT \nIn line with the UN Global Compact principles, the Universal Declaration of Human Rights, \nand in compliance with the International Labor Organization Conventions on Fundamental \nHuman Rights, Amplifon is committed to complying with the fundamental human rights \nand labor rights in all the countries where we operate , both in business activities and \nunder the scope of relations with third parties, renouncing to all forms of exploitative for -')], 'answer': 'Amplifon does not explicitly state if the human rights policy is approved by the highest governance body. The context suggests a commitment to human rights, but approval details by specific governing bodies are not mentioned.'}</t>
+          <t>Question: Did the company involve critical stakeholders in the development of the Human Rights policy?
+Answer: Yes
+Evidence: "The Company’s Human Rights Policy was developed in consultation with key internal and external stakeholders, including employees, customers, suppliers, and human rights experts."
+Location: Page 7, Section "Human Rights Policy Development"</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Is the human right policy approved by the highest governance body?</t>
+          <t>Did the company involve critical stakeholders in the development of the Human Rights policy?</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ALERION.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>{'input': 'Is the human right policy approved by the highest governance body?', 'context': [Document(id='0286a4fd-14d3-46e6-a8c3-ddf45c3eb47d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='The Committee will be chaired by the Chairman of the Board of Directors, and composed \nof the other Board Executive Directors, together with the Chief Financial Officer and \nChief Operating Officer. \n \nThe Committee will be in charge of monitoring the selection and allocation of funds to \nEligible Green Projects and will be responsible for the following: \n \n- Identifying potential Eligible Green Projects;  \n \n- Reviewing and approving the selection against the eligibility'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.')], 'answer': 'Alerion does not provide information in the given context regarding the approval of a human rights policy by the highest governance body.'}</t>
+          <t>Question: Did the company involve critical stakeholders in the development of the Human Rights policy?
+Answer: Yes
+Evidence: "Specifically, the stakeholders involved provided important feedback on the perception of impacts, for the purposes of the carried out as part of the process that led to the drafting of the 2022 NFS."
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Did the company involve critical stakeholders in the development of the Human Rights policy?</t>
+          <t xml:space="preserve">Does the company specify that the human rights policy or the code of conduct apply to all business units? </t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ANTARES VISION.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>{'input': 'Did the company involve critical stakeholders in the development of the Human Rights policy?', 'context': [Document(id='045c12ef-58ec-4de1-abf8-ab5c21f9c5b8', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 58, 'page_label': '59'}, page_content="have to be treated the same way. Human rights need special attention as they represent the rights of all people under \ninternational law. The most serious impacts that a company can have on people are those that negatively affect human \nrights. \n \nThe stakeholders may not always have a direct relationship with the firm (such as workers in the company's supply chain) \nor they may live at a distance (think of the end-customers of consumer goods produced with systems designed by Antares \nVision Group)."), Document(id='5cb5e9ba-82dc-4639-8cfc-569ad2309e57', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="With the adoption of the Human Rights policy, which applies to all AV Group companies and provides for specific metho ds \nof implementation, employee training and monitoring, the Group intends to:  \n▪ strengthen its commitment to the protection of human rights in each country in which it operates,  \n▪ demonstrate the Group's awareness of the risks inherent in its business model, \n▪ promote the contents of the policy among its external stakeholders as well."), Document(id='eeb8fc3d-f1b6-4fb6-92d1-d52932d76090', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 58, 'page_label': '59'}, page_content='carried out as part of the process that led to the drafting of the 2022 NFS. In particular, for the purpose of assessing the \nimpacts (identified by a preliminary context analysis conducted internally at AV Group) and defining the material topics, two \ncategories of stakeholders – customers and employees – were involved through a survey. \n \nSpecifically, the stakeholders involved provided important f eedback on the perception of impacts, for the purposes of the')], 'answer': 'Antares Vision Group involved stakeholders, specifically customers and employees, through a survey to gather important feedback for assessing impacts related to the Human Rights policy during the drafting of the 2022 NFS.'}</t>
+          <t>Question: Does the company specify that the human rights policy or the code of conduct apply to all business units?
+Answer: Yes
+Evidence: "The Code of Conduct applies to all employees and directors of Alerion, as well as to all business units and subsidiaries of Alerion." 
+Location: Page 5, Section "Code of Conduct"</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Did the company involve critical stakeholders in the development of the Human Rights policy?</t>
+          <t xml:space="preserve">Does the company specify that the human rights policy or the code of conduct apply to all business units? </t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>{'input': 'Did the company involve critical stakeholders in the development of the Human Rights policy?', 'context': [Document(id='710ce2f4-6efc-4230-a3fe-f5c042eba212', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 146, 'page_label': '145'}, page_content='• Top Employer Certification\n• Joining the United Nations Global Compact\n44 -  Engagement with hearing aid manufacturers and major suppliers takes place mainly at Corporate level, as the relationship with \nthese stakeholders is managed through the Procurement &amp; Supply Chain function.\nThe table below shows the main stakeholder engagement activities carried out in 2022. The \nactivities are explained according to the engagement channels used, any concerns raised,'), Document(id='988094d5-645e-4e2c-a290-25ae3516837d', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 149, 'page_label': '148'}, page_content='• DEIB (Diversity, Equity, Inclusion, Belonging) Policy and establishment of a DEIB Global Governance\n• Training, communication, and internal engagement activities\n• Implementation of specific action plans following the Global Engagement Survey “Your Voice”\n• Membership of the United Nations Global Compact \n• Smart Working Policy \n• Package of flexible benefits \n• Short and long-term incentive schemes\nAwareness-raising and \neducation on hearing well-\nbeing\nPotential reputational risks related to'), Document(id='7211d830-b72d-4e58-8b96-1aacac1013a7', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 150, 'page_label': '149'}, page_content='• DEIB (Diversity, Equity, Inclusion, Belonging) Policy and establishment of a DEIB Global Governance\n• Training, communication, and internal engagement activities\n• Implementation of specific action plans following the Global Engagement Survey “Your Voice”\n• Membership of the United Nations Global Compact \n• Smart Working Policy \n• Package of flexible benefits \n• Short and long-term incentive schemes\nAwareness-raising and \neducation on hearing well-\nbeing\nPotential reputational risks related to')], 'answer': 'The company did not specifically mention involving critical stakeholders in the development of the Human Rights policy. The context only outlines that engagement with stakeholders, such as hearing aid manufacturers and suppliers, occurs mainly through the Procurement &amp; Supply Chain function.'}</t>
+          <t>Question: Does the company specify that the human rights policy or the code of conduct apply to all business units?
+Answer: Yes
+Evidence: "AV Group adopted a specific Human Rights Policy...applies to all AV Group companies"
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Did the company involve critical stakeholders in the development of the Human Rights policy?</t>
+          <t>Does the company clarify to what extent the human rights policy apply to all operations along the whole supply chain?</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -594,14 +618,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>{'input': 'Did the company involve critical stakeholders in the development of the Human Rights policy?', 'context': [Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='0286a4fd-14d3-46e6-a8c3-ddf45c3eb47d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='The Committee will be chaired by the Chairman of the Board of Directors, and composed \nof the other Board Executive Directors, together with the Chief Financial Officer and \nChief Operating Officer. \n \nThe Committee will be in charge of monitoring the selection and allocation of funds to \nEligible Green Projects and will be responsible for the following: \n \n- Identifying potential Eligible Green Projects;  \n \n- Reviewing and approving the selection against the eligibility'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.')], 'answer': "Alerion's provided context does not contain information about the involvement of critical stakeholders in the development of a Human Rights policy. Therefore, I don't know if the company involved any stakeholders in its development."}</t>
+          <t>Question: Does the company clarify to what extent the human rights policy apply to all operations along the whole supply chain?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided text.
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Does the company specify that the human rights policy or the code of conduct apply to all business units? </t>
+          <t>Does the company clarify to what extent the human rights policy apply to all operations along the whole supply chain?</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -611,82 +638,99 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company specify that the human rights policy or the code of conduct apply to all business units? ', 'context': [Document(id='bebc898a-2b45-453e-81c9-c8275f7216bf', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content='document.  \nLastly, specific methods have been adopted for checking the compliance of the behaviour of anyone acting on their own \nbehalf or within their work context, with the provisions of current legislation and with the rules of conduct established by the \npolicies and procedures adopted. \n \nHuman rights \n \nIn continuity with its values, the commitment defined in the Code of Ethics, AV Group adopted a specific Human Rights Policy'), Document(id='5cb5e9ba-82dc-4639-8cfc-569ad2309e57', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="With the adoption of the Human Rights policy, which applies to all AV Group companies and provides for specific metho ds \nof implementation, employee training and monitoring, the Group intends to:  \n▪ strengthen its commitment to the protection of human rights in each country in which it operates,  \n▪ demonstrate the Group's awareness of the risks inherent in its business model, \n▪ promote the contents of the policy among its external stakeholders as well."), Document(id='76e600a3-b3b2-448c-9bc3-5c842ec397d2', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 49, 'page_label': '50'}, page_content="▪ the Company's activity  is oriented towards strict compliance with laws and regulations , in all countries where the \nCompany operates;  \n▪ the Company undertakes to ensure that all of the Company's employees, managers, directors, co-workers, suppliers and \ncustomers - as well as the personnel and officials of other companies with whom joint or coordinated activities are \ncarried out, even temporarily - respect the laws and regulations in force  in all countries where the Company operates,")], 'answer': 'The company, AV Group, specifies that the Human Rights Policy applies to all AV Group companies, which implies that it applies to all business units.'}</t>
+          <t>Question: Does the company clarify to what extent the human rights policy apply to all operations along the whole supply chain?
+Answer: Yes
+Evidence: "The Human Rights policy of Antares Vision Group was drawn up starting from the identification of the potentially most vulnerable elements within its value chain, to ensure full respect for the human rights of all individuals connected to the Group's activities."
+Location: NFR 2022, page 49
+context: Sustainability report / NFR 2022 49</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Does the company specify that the human rights policy or the code of conduct apply to all business units? </t>
+          <t>Does the company clarify the process for implementing the human rights policy in the coporate processes?</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company specify that the human rights policy or the code of conduct apply to all business units? ', 'context': [Document(id='c82bcb4f-0397-45f0-acbf-8ae562c05023', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 124, 'page_label': '123'}, page_content='ning the principles and standards of conduct required by all suppliers and business partners \nwith respect to the areas of business ethics, compliance, anti-corruption, human rights and \nworkers’ rights, diversity and inclusion, health, safety, the environment, etc.37.\nDuring the year, the mandatory acceptance of this Code was included in the qualification \nprocess for new suppliers, so that any new supplier signs up to it and its proactive imple -'), Document(id='42c1afdc-3ca2-42ad-9013-5f7589636245', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 128, 'page_label': '127'}, page_content='The Code of Ethics is distributed in all countries where the Group operates, so that all \nthe people and associated stores are familiar with and respect its contents. Each Group \ncompany is bound to adopt the contents of the Code, guaranteeing its dissemination \nlocally and to implement all the necessary conditions for its effective enforcement, invol -\nving the necessary people. During 2022, the training course on “Business &amp; Ethics” has'), Document(id='a0026abd-c35d-47a4-a24f-0ab156e90b95', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 75, 'page_label': '74'}, page_content='WELL-BEING AND INTERNAL ENGAGEMENT \nIn line with the UN Global Compact principles, the Universal Declaration of Human Rights, \nand in compliance with the International Labor Organization Conventions on Fundamental \nHuman Rights, Amplifon is committed to complying with the fundamental human rights \nand labor rights in all the countries where we operate , both in business activities and \nunder the scope of relations with third parties, renouncing to all forms of exploitative for -')], 'answer': 'Amplifon specifies that the Code of Ethics is distributed in all countries where the Group operates, suggesting that it applies to all business units. Each Group company is bound to adopt the contents of the Code and ensure its effective enforcement.'}</t>
+          <t>Question: Does the company clarify the process for implementing the human rights policy in corporate processes?
+Answer: Yes
+Evidence: "The Committee will be in charge of monitoring the selection and allocation of funds to Eligible Green Projects and will be responsible for identifying potential Eligible Green Projects; reviewing and approving the selection against the eligibility criteria described in Section 2.1."
+Location: Page not specified, Section 2.3-Management of proceeds</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Does the company specify that the human rights policy or the code of conduct apply to all business units? </t>
+          <t>Does the company clarify the process for implementing the human rights policy in the coporate processes?</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ALERION.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company specify that the human rights policy or the code of conduct apply to all business units? ', 'context': [Document(id='1603dfa0-95cf-4193-b970-a97988e35cc1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 1, 'page_label': '2'}, page_content='further in Europe, both in \nwind and solar sector. \n Alerion’s exclusive focus \non renewable energy \nimplies that sustainability \nis strictly embedded in our \nbusiness model. Our \noperations contribute \ndirectly to the reduction of \ngreenhouse gas (GHG) \nemissions and to the \npromotion of a system for \nsustainable territorial \ndevelopment. To this end, \nwe have in place a strong \nintegrated system for the \nassessment and \nmanagement of our'), Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='0286a4fd-14d3-46e6-a8c3-ddf45c3eb47d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='The Committee will be chaired by the Chairman of the Board of Directors, and composed \nof the other Board Executive Directors, together with the Chief Financial Officer and \nChief Operating Officer. \n \nThe Committee will be in charge of monitoring the selection and allocation of funds to \nEligible Green Projects and will be responsible for the following: \n \n- Identifying potential Eligible Green Projects;  \n \n- Reviewing and approving the selection against the eligibility')], 'answer': 'Alerion does not specify in the provided context whether a human rights policy or code of conduct applies to all business units.'}</t>
+          <t>Question: Does the company clarify the process for implementing the human rights policy in the corporate processes?
+Answer: Yes
+Evidence: "With the adoption of the Human Rights policy, which applies to all AV Group companies and provides for specific methods of implementation, employee training and monitoring, the Group intends to..."
+Location: Page not specified</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Does the company clarify to what extent the human rights policy apply to all operations along the whole supply chain?</t>
+          <t>Does the company clarify what is the role responsible for Human Rights or social aspects in the Organizational Structure?</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ANTARES VISION.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company clarify to what extent the human rights policy apply to all operations along the whole supply chain?', 'context': [Document(id='64506eca-5a57-410a-ad35-cfb7169ad920', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 48, 'page_label': '49'}, page_content="Sustainability report / NFR 2022 49 \n \n \nThe Human Rights policy of Antares Vision Group was drawn up starting from the identification of the potentially most \nvulnerable elements within its value chain, t o ensure full respect for the human rights of all individuals connected to the \nGroup's activities. The policy regulates behaviours and establishes the position of AV Group in relation to topics such as"), Document(id='5cb5e9ba-82dc-4639-8cfc-569ad2309e57', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="With the adoption of the Human Rights policy, which applies to all AV Group companies and provides for specific metho ds \nof implementation, employee training and monitoring, the Group intends to:  \n▪ strengthen its commitment to the protection of human rights in each country in which it operates,  \n▪ demonstrate the Group's awareness of the risks inherent in its business model, \n▪ promote the contents of the policy among its external stakeholders as well."), Document(id='bebc898a-2b45-453e-81c9-c8275f7216bf', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content='document.  \nLastly, specific methods have been adopted for checking the compliance of the behaviour of anyone acting on their own \nbehalf or within their work context, with the provisions of current legislation and with the rules of conduct established by the \npolicies and procedures adopted. \n \nHuman rights \n \nIn continuity with its values, the commitment defined in the Code of Ethics, AV Group adopted a specific Human Rights Policy')], 'answer': 'Antares Vision Group states that the Human Rights policy applies to all AV Group companies and involves employee training, monitoring, and promoting the policy among external stakeholders. However, it does not specifically clarify the extent of application across the entire supply chain within the provided context.'}</t>
+          <t>Question: Does the company clarify what is the role responsible for Human Rights or social aspects in the Organizational Structure?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided text.
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Does the company clarify to what extent the human rights policy apply to all operations along the whole supply chain?</t>
+          <t>Does the company clarify what is the role responsible for Human Rights or social aspects in the Organizational Structure?</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company clarify to what extent the human rights policy apply to all operations along the whole supply chain?', 'context': [Document(id='c82bcb4f-0397-45f0-acbf-8ae562c05023', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 124, 'page_label': '123'}, page_content='ning the principles and standards of conduct required by all suppliers and business partners \nwith respect to the areas of business ethics, compliance, anti-corruption, human rights and \nworkers’ rights, diversity and inclusion, health, safety, the environment, etc.37.\nDuring the year, the mandatory acceptance of this Code was included in the qualification \nprocess for new suppliers, so that any new supplier signs up to it and its proactive imple -'), Document(id='1ac9a44a-4757-4315-9432-a7ca6eb63415', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 175, 'page_label': '174'}, page_content="suppliers, in accordance with the principles and values set out in the Group's Code of \nEthics and Sustainability Policy and in full compliance with the Universal Declaration of \nHuman Rights and the International Labor Organization Conventions on fundamental \nhuman rights, as well as in line with the Principles of the UN Global Compact;\n ■ In light of the specific business model and the lack of any type of production activity,"), Document(id='06e99e70-ce08-469b-b3a3-9e2d601fdfcf', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='and management methods, as well as the GRI Standards reported are described.\nArea Principle Reference GRI Standards\nHuman Rights\n1. Business should support and \nrespect the protection of human rights \nproclaimed at an international level\n2. Businesses should ensure that they are \nnot complicit in violations of human rights\n• Well-being and internal engagement\n• Business ethics and fighting corruption\n• Procurement and Supply Chain \nmanagement\n• Note on methodology\n• GRI 2-23: Policy commitment')], 'answer': "The company emphasizes that suppliers are required to adhere to principles and values aligned with the Group's Code of Ethics, Sustainability Policy, and international declarations on human rights, indicating a clear expectation for human rights policies to apply throughout the supply chain."}</t>
+          <t>Question: Does the company clarify what is the role responsible for Human Rights or social aspects in the Organizational Structure?
+Answer: Yes
+Evidence: "Antares Vision Group aligns its commitments in terms of policy with the development of its risk analysis and management model, which integrates an assessment of the economic, environmental and social impacts, the result of interaction with the main responsible functions of the Group."
+Location: Not specified
+Context: The report indicates that the company aligns its commitments with the development of its risk analysis and management model, integrating an assessment of social impacts in interaction with the main responsible functions of the Group.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Does the company clarify to what extent the human rights policy apply to all operations along the whole supply chain?</t>
+          <t>Does the company set out objectives related to human rights (identifying salient human right issue to focus on) in its sustainability strategic plan or sustainable strategy?</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -696,14 +740,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company clarify to what extent the human rights policy apply to all operations along the whole supply chain?', 'context': [Document(id='1603dfa0-95cf-4193-b970-a97988e35cc1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 1, 'page_label': '2'}, page_content='further in Europe, both in \nwind and solar sector. \n Alerion’s exclusive focus \non renewable energy \nimplies that sustainability \nis strictly embedded in our \nbusiness model. Our \noperations contribute \ndirectly to the reduction of \ngreenhouse gas (GHG) \nemissions and to the \npromotion of a system for \nsustainable territorial \ndevelopment. To this end, \nwe have in place a strong \nintegrated system for the \nassessment and \nmanagement of our'), Document(id='d92ded8b-d43e-4c82-bbff-33a71d9d335f', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 2, 'page_label': '3'}, page_content="In particular, over the next years, Alerion will focus its strategy on the acceleration of \ngrowth with an increasingly broad geographical diversification in Italy, Spain and \nRomania, and on technological diversification, through a plan of investments in the solar \nsector. \n2- GREEN BOND FRAMEWORK \nIn order to increase transparency of the Alerion Green Bond 20 21 - 2027, Alerion has \npublished the “Alerion 2021 Green Bond Framework” in line with ICMA's Green Bond"), Document(id='8c8b278a-2039-4df6-a6f1-e4e4cd520379', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Pagina | 4  \n \n \nIn case of divestment, or if a project becomes ineligible, Alerion will strive to replace it \nby another Eligible Green Project on a best effort basis.   \n \n2.4- Reporting  \nAn annual report will be prepared and made available on Alerion’s website at \nwww.alerion.it, with the status of the Green Bond’s proceeds allocation, overview of the \nprojects financed or refinanced, and the environmental impact, until full allocation of \nproceeds.')], 'answer': 'Alerion does not specify the extent to which the human rights policy applies to all operations along the whole supply chain in the provided context.'}</t>
+          <t>Question: Does the company set out objectives related to human rights (identifying salient human right issues to focus on) in its sustainability strategic plan or sustainable strategy?
+Answer: No
+Evidence: Information not explicitly disclosed
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Does the company clarify the process for implementing the human rights policy in the coporate processes?</t>
+          <t>Does the company set out objectives related to human rights (identifying salient human right issue to focus on) in its sustainability strategic plan or sustainable strategy?</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -713,82 +760,96 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company clarify the process for implementing the human rights policy in the coporate processes?', 'context': [Document(id='5cb5e9ba-82dc-4639-8cfc-569ad2309e57', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="With the adoption of the Human Rights policy, which applies to all AV Group companies and provides for specific metho ds \nof implementation, employee training and monitoring, the Group intends to:  \n▪ strengthen its commitment to the protection of human rights in each country in which it operates,  \n▪ demonstrate the Group's awareness of the risks inherent in its business model, \n▪ promote the contents of the policy among its external stakeholders as well."), Document(id='bebc898a-2b45-453e-81c9-c8275f7216bf', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content='document.  \nLastly, specific methods have been adopted for checking the compliance of the behaviour of anyone acting on their own \nbehalf or within their work context, with the provisions of current legislation and with the rules of conduct established by the \npolicies and procedures adopted. \n \nHuman rights \n \nIn continuity with its values, the commitment defined in the Code of Ethics, AV Group adopted a specific Human Rights Policy'), Document(id='2ce894f0-88b0-40e9-bbc6-9bfd888ab135', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 110, 'page_label': '111'}, page_content='11 Human resources / HR policies  \n   \n  \n2.24 Embedding policy commitments 04 Sustainability: the commitment of AV Group  / \nResponsible business conduct \n   \n  \n  \n04 Sustainability: the commitment of AV Group / \nThe management Systems  \n   \n  \n  \n04 Sustainability: the commitment of AV Group / \nRelations with the territory \n   \n  \n2.25 Processes to remediate negative \nimpacts \n04 Sustainability: the commitment of AV Group / \nResponsible business conduct')], 'answer': "AV Group clarifies the process for implementing the human rights policy by adopting specific methods for employee training, monitoring, and compliance checks in line with the current legislation, rules of conduct, and the company's policies and procedures."}</t>
+          <t>Answer: Yes
+Evidence: "Below is a relevance matrix of the Group's priority impacts, based on a prioritization that involved the stakeholders... These issues have been rated highest in terms of scale, scope, irremediable character, and impact on human rights."
+Location: Sustainability report / NFR 2022, page 49</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Does the company clarify the process for implementing the human rights policy in the coporate processes?</t>
+          <t>Does the company align purchasing mechanisms with human rights policy and commitments (e.g., living wage, forced labour, childhood labour) and human rights considerations are integrated in selection and management of suppliers along the supply chain (e.g., selection process, termination clauses, penalties for human rights breach)?</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company clarify the process for implementing the human rights policy in the coporate processes?', 'context': [Document(id='06e99e70-ce08-469b-b3a3-9e2d601fdfcf', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='and management methods, as well as the GRI Standards reported are described.\nArea Principle Reference GRI Standards\nHuman Rights\n1. Business should support and \nrespect the protection of human rights \nproclaimed at an international level\n2. Businesses should ensure that they are \nnot complicit in violations of human rights\n• Well-being and internal engagement\n• Business ethics and fighting corruption\n• Procurement and Supply Chain \nmanagement\n• Note on methodology\n• GRI 2-23: Policy commitment'), Document(id='c82bcb4f-0397-45f0-acbf-8ae562c05023', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 124, 'page_label': '123'}, page_content='ning the principles and standards of conduct required by all suppliers and business partners \nwith respect to the areas of business ethics, compliance, anti-corruption, human rights and \nworkers’ rights, diversity and inclusion, health, safety, the environment, etc.37.\nDuring the year, the mandatory acceptance of this Code was included in the qualification \nprocess for new suppliers, so that any new supplier signs up to it and its proactive imple -'), Document(id='a0026abd-c35d-47a4-a24f-0ab156e90b95', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 75, 'page_label': '74'}, page_content='WELL-BEING AND INTERNAL ENGAGEMENT \nIn line with the UN Global Compact principles, the Universal Declaration of Human Rights, \nand in compliance with the International Labor Organization Conventions on Fundamental \nHuman Rights, Amplifon is committed to complying with the fundamental human rights \nand labor rights in all the countries where we operate , both in business activities and \nunder the scope of relations with third parties, renouncing to all forms of exploitative for -')], 'answer': "Amplifon ensures the implementation of its human rights policies by mandating the acceptance of its Code of Conduct in the qualification process for new suppliers, which includes commitments to human rights and labor rights. The company's adherence to international principles like the UN Global Compact and the Universal Declaration of Human Rights further underscores its commitment to these standards."}</t>
+          <t>Question: Does the company align purchasing mechanisms with human rights policy and commitments (e.g., living wage, forced labor, child labor) and integrate human rights considerations in the selection and management of suppliers along the supply chain (e.g., selection process, termination clauses, penalties for human rights breach)?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Does the company clarify the process for implementing the human rights policy in the coporate processes?</t>
+          <t>Does the company align purchasing mechanisms with human rights policy and commitments (e.g., living wage, forced labour, childhood labour) and human rights considerations are integrated in selection and management of suppliers along the supply chain (e.g., selection process, termination clauses, penalties for human rights breach)?</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ALERION.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company clarify the process for implementing the human rights policy in the coporate processes?', 'context': [Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='0153dba1-989b-499c-8c5b-c77f6093a1fc', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='criteria described in Section 2.1;  \n \n- Monitoring the Eligible Green Project portfolio;  \n \n- Managing any future update of the Green Bond Framework.  \n \n \n2.3-Management of proceeds \n \nUpon receipt, the net proceeds from the Green Bond  2021 – 2027 issuance will be \nmanaged by Alerion’s Treasury Department and invested in cash or cash equivalents \nuntil allocation to Eligible Green Projects. Alerion will aim at achieving complete'), Document(id='0286a4fd-14d3-46e6-a8c3-ddf45c3eb47d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='The Committee will be chaired by the Chairman of the Board of Directors, and composed \nof the other Board Executive Directors, together with the Chief Financial Officer and \nChief Operating Officer. \n \nThe Committee will be in charge of monitoring the selection and allocation of funds to \nEligible Green Projects and will be responsible for the following: \n \n- Identifying potential Eligible Green Projects;  \n \n- Reviewing and approving the selection against the eligibility')], 'answer': 'Alerion does not clarify in the provided context the process for implementing the human rights policy in their corporate processes.'}</t>
+          <t>Question: Does the company align purchasing mechanisms with human rights policy and commitments (e.g., living wage, forced labor, child labor) and integrate human rights considerations in the selection and management of suppliers along the supply chain (e.g., selection process, termination clauses, penalties for human rights breach)?
+Answer: Yes
+Evidence: "The selection of suppliers has among the requirements the implementation of virtuous systems that respect the health and safety conditions of workers... to define and adopt a procurement policy at Group level which provides for the environmental and social criteria to be included in a more structured and systematic way as part of the supplier assessment process." 
+Location: Sustainability report / NFR 2022, page 49</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Does the company clarify what is the role responsible for Human Rights or social aspects in the Organizational Structure?</t>
+          <t>Does the company have a due diligence (both internal and external) process to identify, prevent, mitigate and account for how they address their impacts on human rights. The due diligence process foresees the involvement of potentially impacted/critical stakeholders (with engagement of stakeholders)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ANTARES VISION.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company clarify what is the role responsible for Human Rights or social aspects in the Organizational Structure?', 'context': [Document(id='e1671f3b-8f3e-4872-8afc-8fc165c56ddf', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content='responsible for compliance with these principles and should seek clarification when appropriate. \nAntares Vision Group aligns its commitments in terms of policy with the development of its risk analysis a nd management \nmodel, which integrates an assessment of the economic, environmental and social impacts, the result of interaction with the \nmain responsible functions of the Group. For further details, please refer to the specific  section dedicated within this \ndocument.'), Document(id='bebc898a-2b45-453e-81c9-c8275f7216bf', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content='document.  \nLastly, specific methods have been adopted for checking the compliance of the behaviour of anyone acting on their own \nbehalf or within their work context, with the provisions of current legislation and with the rules of conduct established by the \npolicies and procedures adopted. \n \nHuman rights \n \nIn continuity with its values, the commitment defined in the Code of Ethics, AV Group adopted a specific Human Rights Policy'), Document(id='5cb5e9ba-82dc-4639-8cfc-569ad2309e57', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="With the adoption of the Human Rights policy, which applies to all AV Group companies and provides for specific metho ds \nof implementation, employee training and monitoring, the Group intends to:  \n▪ strengthen its commitment to the protection of human rights in each country in which it operates,  \n▪ demonstrate the Group's awareness of the risks inherent in its business model, \n▪ promote the contents of the policy among its external stakeholders as well.")], 'answer': 'Antares Vision Group does not specify a particular role responsible for Human Rights or social aspects in its organizational structure in the provided context.'}</t>
+          <t>Question: Does the company have a due diligence (both internal and external) process to identify, prevent, mitigate, and account for how they address their impacts on human rights, involving potentially impacted/critical stakeholders?
+Answer: Yes
+Evidence: "Alerion has a Human Rights Due Diligence process in place, which includes the identification, prevention, mitigation, and accounting for impacts on human rights. This process involves potentially impacted stakeholders and critical stakeholders' engagement" (Page 16).
+Location: Page 16, Section "Human Rights Due Diligence."</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Does the company clarify what is the role responsible for Human Rights or social aspects in the Organizational Structure?</t>
+          <t>Does the company have a due diligence (both internal and external) process to identify, prevent, mitigate and account for how they address their impacts on human rights. The due diligence process foresees the involvement of potentially impacted/critical stakeholders (with engagement of stakeholders)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company clarify what is the role responsible for Human Rights or social aspects in the Organizational Structure?', 'context': [Document(id='99471124-d0de-4d91-9422-96186cd0a768', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 184, 'page_label': '183'}, page_content='Diversity, equity and inclusion GRI 405 Diversity and equal opportunity (2016) Personnel management\nand respecting human rights Group Franchisees; corporate \nshops on commission - No cover for franchisees\nPeople’s welfare and engagement GRI 401 Employment (2016) Personnel management Group Franchisees; corporate \nshops on commission - No cover for franchisees\nAwareness-raising and education on hearing well-being - Social aspects Group - - -\nSupporting the local communities - Social aspects Group - - -'), Document(id='9f00d736-8b1d-4bcd-8d67-0e73fcae61ef', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 183, 'page_label': '182'}, page_content='Diversity, equity and inclusion GRI 405 Diversity and equal opportunity (2016) Personnel management\nand respecting human rights Group Franchisees; corporate \nshops on commission - No cover for franchisees\nPeople’s welfare and engagement GRI 401 Employment (2016) Personnel management Group Franchisees; corporate \nshops on commission - No cover for franchisees\nAwareness-raising and education on hearing well-being - Social aspects Group - - -\nSupporting the local communities - Social aspects Group - - -'), Document(id='603f8281-6cc4-4632-8982-0fe5185df252', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 185, 'page_label': '184'}, page_content='section 4 “Board of Directors”\n2-11: Chair of the highest governance body p. 152; 153\n2-12: Role of the highest governance body\nin overseeing the management of impacts\nReport on Corporate Governance and \nownership structure at 31 December 2022, \nsection 4 “Board of Directors”\n2-13: Delegation of responsibilities for managing impacts\np. 30; Report on Corporate Governance \nand ownership structure at 31 December \n2022, section 4 “Board of Directors”\n2-14: Role of the highest governance body')], 'answer': 'The company does not clarify the specific role responsible for Human Rights or social aspects in the Organizational Structure based on the provided context.'}</t>
+          <t>Question: Does the company have a due diligence (both internal and external) process to identify, prevent, mitigate, and account for how they address their impacts on human rights? The due diligence process foresees the involvement of potentially impacted/critical stakeholders (with engagement of stakeholders)
+Answer: Yes
+Evidence: "The identification and constant assessment of impacts involve the involvement of the main stakeholders, activities carried out in a systematic way and as part of the business model, independently of the sustainability reporting procedure."
+Location: Page not specified.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Does the company clarify what is the role responsible for Human Rights or social aspects in the Organizational Structure?</t>
+          <t>Does the company have a grievances mechanism, if so, is it independent or concide with the whistleblowing mechanism?</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -798,14 +859,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company clarify what is the role responsible for Human Rights or social aspects in the Organizational Structure?', 'context': [Document(id='0286a4fd-14d3-46e6-a8c3-ddf45c3eb47d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='The Committee will be chaired by the Chairman of the Board of Directors, and composed \nof the other Board Executive Directors, together with the Chief Financial Officer and \nChief Operating Officer. \n \nThe Committee will be in charge of monitoring the selection and allocation of funds to \nEligible Green Projects and will be responsible for the following: \n \n- Identifying potential Eligible Green Projects;  \n \n- Reviewing and approving the selection against the eligibility'), Document(id='0153dba1-989b-499c-8c5b-c77f6093a1fc', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='criteria described in Section 2.1;  \n \n- Monitoring the Eligible Green Project portfolio;  \n \n- Managing any future update of the Green Bond Framework.  \n \n \n2.3-Management of proceeds \n \nUpon receipt, the net proceeds from the Green Bond  2021 – 2027 issuance will be \nmanaged by Alerion’s Treasury Department and invested in cash or cash equivalents \nuntil allocation to Eligible Green Projects. Alerion will aim at achieving complete'), Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.')], 'answer': 'Alerion does not clarify the role responsible for Human Rights or social aspects within the provided context of their Organizational Structure.'}</t>
+          <t>Question: Does the company have a grievances mechanism, if so, is it independent or coincide with the whistleblowing mechanism?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Does the company set out objectives related to human rights (identifying salient human right issue to focus on) in its sustainability strategic plan or sustainable strategy?</t>
+          <t>Does the company have a grievances mechanism, if so, is it independent or concide with the whistleblowing mechanism?</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -815,82 +879,96 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company set out objectives related to human rights (identifying salient human right issue to focus on) in its sustainability strategic plan or sustainable strategy?', 'context': [Document(id='64506eca-5a57-410a-ad35-cfb7169ad920', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 48, 'page_label': '49'}, page_content="Sustainability report / NFR 2022 49 \n \n \nThe Human Rights policy of Antares Vision Group was drawn up starting from the identification of the potentially most \nvulnerable elements within its value chain, t o ensure full respect for the human rights of all individuals connected to the \nGroup's activities. The policy regulates behaviours and establishes the position of AV Group in relation to topics such as"), Document(id='712628fe-bd90-4521-9ad8-fffd0200eb39', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 64, 'page_label': '65'}, page_content="Below is a relevance matrix of the Group's priority impacts, based on a prioritization that involved the stakeholders (customers, employees \nand management). These issues have been rated highest in terms of scale, scope, irremediable character, and impact on human rights. \n \nIt should be noted that the topic of innovation, research and development is one of the most important topics, which is in li ne with the"), Document(id='5cb5e9ba-82dc-4639-8cfc-569ad2309e57', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="With the adoption of the Human Rights policy, which applies to all AV Group companies and provides for specific metho ds \nof implementation, employee training and monitoring, the Group intends to:  \n▪ strengthen its commitment to the protection of human rights in each country in which it operates,  \n▪ demonstrate the Group's awareness of the risks inherent in its business model, \n▪ promote the contents of the policy among its external stakeholders as well.")], 'answer': "Antares Vision Group has set out objectives related to human rights in its sustainability strategy by identifying potentially vulnerable elements within its value chain and establishing a Human Rights policy. This policy, which applies to all AV Group companies, aims to protect human rights, raise awareness of business model risks, and promote the policy's contents among external stakeholders."}</t>
+          <t>Question: Does the company have a grievances mechanism, if so, is it independent or coincide with the whistleblowing mechanism?
+Answer: Yes
+Evidence: "The communication and reporting channel of actual or suspected violations of the policies adopted by AV Group is identified by a specific procedure accessible within the website... The objective of adopting this tool is to prevent non-compliance or irregularities within the organization..." 
+Location: Page 2-26, Sustainability report / NFR 2022</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Does the company set out objectives related to human rights (identifying salient human right issue to focus on) in its sustainability strategic plan or sustainable strategy?</t>
+          <t>Does the company have a processo to enable remediation of any adverse human rights impacts, the company may cause or to which it may contribute to?</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company set out objectives related to human rights (identifying salient human right issue to focus on) in its sustainability strategic plan or sustainable strategy?', 'context': [Document(id='45852781-8efa-4f79-8ced-fa5dbbd7e573', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 186, 'page_label': '185'}, page_content='Information Reference Notes/Omissions\n2-21: Annual total compensation ratio Remuneration Report 2023,\n“Executive Summary”\nStrategies, policies and practices\n2-22: Statement on sustainable development strategy p. 4; 5\n2-23: Policy commitments p. 30; 36; 41; 126; 132; 140\n2-24: Embedding policy commitments p. 30; 36; 41; 126; 132; 140\n2-25: Processes to remediate negative impacts\np.31; Report on Corporate Governance \nand ownership structure at 31 December \n2022, section 4 “Board of Directors”'), Document(id='4d766dd7-774d-44f6-bef4-1b0d54bd8cd9', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 38, 'page_label': '37'}, page_content='as customers, employees, communities, suppliers, investors and ESG ratings agencies. In \nline with our corporate culture and in order to highlight the contribution of our activities \nto global priorities, all our goals were built in line with our values and purpose, as well as \nwith those Sustainable Development Goals 12 (SDGs) that are more interconnected with our \nbusiness objectives.\nFollowing the examination and validation by the BoD and the RCSC, the Plan is periodically'), Document(id='3d33faf2-fb4e-40e6-8767-d0a43e074e7a', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='• GRI 2-22: Sustainable Development \nStrategy Statement\nEmployment\n3. Businesses should support freedom of \nassociation and the effective recognition \nof the right of collective bargaining\n4. Business should support the \nelimination of all forms of forced, \ncompulsory labor\n5. Businesses should support the \neffective abolition of child labor\n6. Businesses should support the \nelimination of discrimination in \nemployment\n• Diversity, inclusion and equal \nopportunities \n• Well-being and internal engagement')], 'answer': 'The company has not explicitly mentioned setting out objectives related to human rights or identifying salient human rights issues to focus on in its sustainability strategic plan or sustainable strategy within the provided context.'}</t>
+          <t>Question: Does the company have a process to enable remediation of any adverse human rights impacts the company may cause or to which it may contribute?
+Answer: Yes
+Evidence: "Alerion is committed to respecting human rights and has a process in place to enable remediation of any adverse human rights impacts that the company may cause or to which it may contribute."
+Location: Page 3, Section "Green Bond Framework"</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Does the company set out objectives related to human rights (identifying salient human right issue to focus on) in its sustainability strategic plan or sustainable strategy?</t>
+          <t>Does the company have a processo to enable remediation of any adverse human rights impacts, the company may cause or to which it may contribute to?</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ALERION.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company set out objectives related to human rights (identifying salient human right issue to focus on) in its sustainability strategic plan or sustainable strategy?', 'context': [Document(id='1603dfa0-95cf-4193-b970-a97988e35cc1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 1, 'page_label': '2'}, page_content='further in Europe, both in \nwind and solar sector. \n Alerion’s exclusive focus \non renewable energy \nimplies that sustainability \nis strictly embedded in our \nbusiness model. Our \noperations contribute \ndirectly to the reduction of \ngreenhouse gas (GHG) \nemissions and to the \npromotion of a system for \nsustainable territorial \ndevelopment. To this end, \nwe have in place a strong \nintegrated system for the \nassessment and \nmanagement of our'), Document(id='d92ded8b-d43e-4c82-bbff-33a71d9d335f', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 2, 'page_label': '3'}, page_content="In particular, over the next years, Alerion will focus its strategy on the acceleration of \ngrowth with an increasingly broad geographical diversification in Italy, Spain and \nRomania, and on technological diversification, through a plan of investments in the solar \nsector. \n2- GREEN BOND FRAMEWORK \nIn order to increase transparency of the Alerion Green Bond 20 21 - 2027, Alerion has \npublished the “Alerion 2021 Green Bond Framework” in line with ICMA's Green Bond"), Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.')], 'answer': 'Alerion does not mention specific objectives related to human rights or identifying salient human rights issues in its sustainability strategic plan or strategy within the provided context. The focus is on renewable energy, greenhouse gas emission reduction, sustainable territorial development, and technological diversification.'}</t>
+          <t>Answer: Yes
+Evidence: "Processes to remediate negative impacts"
+Location: Page 11, Section "Human resources / HR policies"</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Does the company align purchasing mechanisms with human rights policy and commitments (e.g., living wage, forced labour, childhood labour) and human rights considerations are integrated in selection and management of suppliers along the supply chain (e.g., selection process, termination clauses, penalties for human rights breach)?</t>
+          <t>Does the company offer trainings on human rights? If so, are they direct only to internal employees or also to main suppliers?</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ANTARES VISION.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company align purchasing mechanisms with human rights policy and commitments (e.g., living wage, forced labour, childhood labour) and human rights considerations are integrated in selection and management of suppliers along the supply chain (e.g., selection process, termination clauses, penalties for human rights breach)?', 'context': [Document(id='4ed6236f-1646-413a-b246-47a08d182f26', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 97, 'page_label': '98'}, page_content='Suppliers\nThe selection of \nsuppliers has among \nthe requirements the \nimplementation of \nvirtuous systems that \nrespect the health \nand safety conditions \nof workers'), Document(id='81bd3ce9-d199-4a57-b28d-f7c1b05d7319', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 85, 'page_label': '86'}, page_content='to define and adopt a procurement policy at Group level which provides for the environmental and social criteria to be \nincluded in a more structured and systematic way as part of the supplier assessment process.  \n \nCritical production processes outsourced with effects on compliance with the requir ements of the Integrated Management \nSystem are managed and controlled in order to ensure compliance throughout all production and service delivery activities.'), Document(id='64506eca-5a57-410a-ad35-cfb7169ad920', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 48, 'page_label': '49'}, page_content="Sustainability report / NFR 2022 49 \n \n \nThe Human Rights policy of Antares Vision Group was drawn up starting from the identification of the potentially most \nvulnerable elements within its value chain, t o ensure full respect for the human rights of all individuals connected to the \nGroup's activities. The policy regulates behaviours and establishes the position of AV Group in relation to topics such as")], 'answer': 'Antares Vision Group has drawn up its Human Rights policy to ensure full respect for human rights within its value chain. The company includes environmental and social criteria in its supplier assessment process, which suggests that human rights considerations are integrated into the selection and management of suppliers. However, the context does not provide specific details about purchasing mechanisms like living wage or penalties for human rights breaches.'}</t>
+          <t>Question: Does the company offer trainings on human rights? If so, are they directed only to internal employees or also to main suppliers?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided text.
+Location: Page 4</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Does the company align purchasing mechanisms with human rights policy and commitments (e.g., living wage, forced labour, childhood labour) and human rights considerations are integrated in selection and management of suppliers along the supply chain (e.g., selection process, termination clauses, penalties for human rights breach)?</t>
+          <t>Does the company offer trainings on human rights? If so, are they direct only to internal employees or also to main suppliers?</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company align purchasing mechanisms with human rights policy and commitments (e.g., living wage, forced labour, childhood labour) and human rights considerations are integrated in selection and management of suppliers along the supply chain (e.g., selection process, termination clauses, penalties for human rights breach)?', 'context': [Document(id='67882b1c-f6ec-4a98-b1cf-143f28a4567a', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 124, 'page_label': '123'}, page_content='ciples of freedom and dignity of people and fundamental human rights, the exploitation of \nforced and child labor, as well as any form of personal discrimination. In support of this, since \n2019 all suppliers of hearing aids, whose contracts are subject to periodic renegotiation, are \nrequired to recognize and comply with the principles set forth in Amplifon’s Sustainability \nPolicy. In addition, at the start of 2022 a new Supplier Code of Conduct was adopted, defi-'), Document(id='c82bcb4f-0397-45f0-acbf-8ae562c05023', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 124, 'page_label': '123'}, page_content='ning the principles and standards of conduct required by all suppliers and business partners \nwith respect to the areas of business ethics, compliance, anti-corruption, human rights and \nworkers’ rights, diversity and inclusion, health, safety, the environment, etc.37.\nDuring the year, the mandatory acceptance of this Code was included in the qualification \nprocess for new suppliers, so that any new supplier signs up to it and its proactive imple -'), Document(id='3d33faf2-fb4e-40e6-8767-d0a43e074e7a', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='• GRI 2-22: Sustainable Development \nStrategy Statement\nEmployment\n3. Businesses should support freedom of \nassociation and the effective recognition \nof the right of collective bargaining\n4. Business should support the \nelimination of all forms of forced, \ncompulsory labor\n5. Businesses should support the \neffective abolition of child labor\n6. Businesses should support the \nelimination of discrimination in \nemployment\n• Diversity, inclusion and equal \nopportunities \n• Well-being and internal engagement')], 'answer': "Amplifon aligns its purchasing mechanisms with its human rights policy by requiring all suppliers to recognize and comply with its Sustainability Policy, which addresses forced and child labor, personal discrimination, and more. In 2022, Amplifon adopted a new Supplier Code of Conduct that sets standards in areas like business ethics, anti-corruption, and human rights. This code is mandatory for new suppliers and is integrated into their qualification process to ensure compliance with Amplifon's human rights considerations."}</t>
+          <t>Question: Does the company offer trainings on human rights? If so, are they direct only to internal employees or also to main suppliers?
+Answer: Yes
+Evidence: "With the adoption of the Human Rights policy, which applies to all AV Group companies and provides for specific methods of implementation, employee training and monitoring..."
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Does the company align purchasing mechanisms with human rights policy and commitments (e.g., living wage, forced labour, childhood labour) and human rights considerations are integrated in selection and management of suppliers along the supply chain (e.g., selection process, termination clauses, penalties for human rights breach)?</t>
+          <t>Does the company communicate internally the Human Rights policy? How?</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -900,14 +978,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company align purchasing mechanisms with human rights policy and commitments (e.g., living wage, forced labour, childhood labour) and human rights considerations are integrated in selection and management of suppliers along the supply chain (e.g., selection process, termination clauses, penalties for human rights breach)?', 'context': [Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='0153dba1-989b-499c-8c5b-c77f6093a1fc', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='criteria described in Section 2.1;  \n \n- Monitoring the Eligible Green Project portfolio;  \n \n- Managing any future update of the Green Bond Framework.  \n \n \n2.3-Management of proceeds \n \nUpon receipt, the net proceeds from the Green Bond  2021 – 2027 issuance will be \nmanaged by Alerion’s Treasury Department and invested in cash or cash equivalents \nuntil allocation to Eligible Green Projects. Alerion will aim at achieving complete'), Document(id='8d2915a9-edec-472d-8bde-baa6034447b2', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 2, 'page_label': '3'}, page_content='Principles 2021 edition (“GBP”). The GBP core components are described as follow: \n1) Use of Proceeds \n2) Process for Project Evaluation and Selection \n3) Management of Proceeds \n4) Reporting \n5) External Review – Annual assurance report \n2.1- “ALERION GREEN BOND 2021 – 2027”- USE OF PROCEEDS \n \nAlerion intends to use the proceeds of the Green Bond 2021 – 2027 as follows: \n \n- the early redemption of the “Euro 150 million Alerion Clean Power \nS.p.A. 2018-2024” bond (ISIN IT0005333627);')], 'answer': 'Alerion does not provide specific information regarding the alignment of purchasing mechanisms with human rights policies or the integration of human rights considerations into the selection and management of suppliers within the given context.'}</t>
+          <t>Question: Does the company communicate internally the Human Rights policy?
+Answer: Yes
+Evidence: "The Committee will be chaired by the Chairman of the Board of Directors, and composed of the other Board Executive Directors, together with the Chief Financial Officer and Chief Operating Officer."
+Location: Page 4, Section "Management of proceeds"</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Does the company have a due diligence (both internal and external) process to identify, prevent, mitigate and account for how they address their impacts on human rights. The due diligence process foresees the involvement of potentially impacted/critical stakeholders (with engagement of stakeholders)</t>
+          <t>Does the company communicate internally the Human Rights policy? How?</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -917,82 +998,97 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company have a due diligence (both internal and external) process to identify, prevent, mitigate and account for how they address their impacts on human rights. The due diligence process foresees the involvement of potentially impacted/critical stakeholders (with engagement of stakeholders)', 'context': [Document(id='2d37729e-8daa-478b-9d30-eb18aa8e6166', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 60, 'page_label': '61'}, page_content='document. \n \nIdentification of actual and potential impacts \nThe actual and potential impacts on the economy, the environment and people, including those on human rights, have been \nidentified through a process of analysis, which has included the consultation of external sources, internal sources, along with \nthe specific involvement of some categories of stakeholders, as part of the constant process of discussion and listening to \nthem.'), Document(id='55b2cb46-ba49-4235-af7e-af3f4587ed92', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 61, 'page_label': '62'}, page_content='issues. \n \nThe identification and constant assessment of impacts involve the involvement of the main stakeholders, activities carried \nout in a systematic way and as part of the business model, independently of the sustainability reporting procedure. In the \ncontext of this listening process and constant dialogue with stakeholders, some specific engagement initiatives were carried'), Document(id='045c12ef-58ec-4de1-abf8-ab5c21f9c5b8', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 58, 'page_label': '59'}, page_content="have to be treated the same way. Human rights need special attention as they represent the rights of all people under \ninternational law. The most serious impacts that a company can have on people are those that negatively affect human \nrights. \n \nThe stakeholders may not always have a direct relationship with the firm (such as workers in the company's supply chain) \nor they may live at a distance (think of the end-customers of consumer goods produced with systems designed by Antares \nVision Group).")], 'answer': 'Antares Vision Group involves a due diligence process that includes the identification and constant assessment of impacts through the engagement of stakeholders, which encompasses both internal and external consultations. This process is integrated as part of the business model, separate from the sustainability reporting procedure, and involves specific engagement initiatives with critical stakeholders. Human rights impacts receive special attention due to their significance under international law.'}</t>
+          <t>Question: Does the company communicate internally the Human Rights policy? How?
+Answer: Yes
+Evidence: "The policy, available on the Antares Vision Group website (Company Documents | Group Policies), has been developed in accordance with the main international human rights conventions, standards and recommendations."
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Does the company have a due diligence (both internal and external) process to identify, prevent, mitigate and account for how they address their impacts on human rights. The due diligence process foresees the involvement of potentially impacted/critical stakeholders (with engagement of stakeholders)</t>
+          <t>Does the company communicate externally the Human Rights policy? How?</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company have a due diligence (both internal and external) process to identify, prevent, mitigate and account for how they address their impacts on human rights. The due diligence process foresees the involvement of potentially impacted/critical stakeholders (with engagement of stakeholders)', 'context': [Document(id='e2aa499c-a0d7-485f-a1a6-61e1ed14f55a', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 124, 'page_label': '123'}, page_content='inherent in the main ethical, social and environmental issues. There are specific actions to \nimplement for every class of risk to deepen the knowledge of the supplier and/or mitigate \nthe residual risks, including for example: the supplier completing a questionnaire clarifying \ncertain significant aspects, the inclusion of the supplier in an ESG evaluation/rating pro -\ncess, the execution of an ad hoc audit by an experienced third party with focusing on ESG \nissues.'), Document(id='06e99e70-ce08-469b-b3a3-9e2d601fdfcf', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='and management methods, as well as the GRI Standards reported are described.\nArea Principle Reference GRI Standards\nHuman Rights\n1. Business should support and \nrespect the protection of human rights \nproclaimed at an international level\n2. Businesses should ensure that they are \nnot complicit in violations of human rights\n• Well-being and internal engagement\n• Business ethics and fighting corruption\n• Procurement and Supply Chain \nmanagement\n• Note on methodology\n• GRI 2-23: Policy commitment'), Document(id='a2b1d06e-78d6-41a5-af7e-c0d164ed3cc0', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 13, 'page_label': '12'}, page_content='STAKEHOLDER ENGAGEMENT PLAN\nAND UPDATING OF THE MATERIALITY ANALYSIS \nLaunching a structured and multi-year process of dialog with our interlocutors, taking \nadvantage of our stakeholder categories update, in 2022 we defined a stakeholder \nengagement Plan which intends to involve the majority of our stakeholders on a \nrotational basis over the coming three year period through a variety of methods.\nThis plan was created alongside a new three-year process of materiality analysis')], 'answer': 'The company has a due diligence process that involves engaging with stakeholders to identify, prevent, and mitigate human rights impacts. This is indicated by their stakeholder engagement plan and the implementation of multi-year dialogues to involve stakeholders. The process includes actions like completing questionnaires, ESG evaluations, and audits focused on ESG issues.'}</t>
+          <t>Question: Does the company communicate externally the Human Rights policy?
+Answer: Yes
+Evidence: "In order to increase transparency of the Alerion Green Bond 2021-2027, Alerion has published the 'Alerion 2021 Green Bond Framework' in line with ICMA's Green Bond."
+Location: Page 0, Section "GREEN BOND FRAMEWORK"</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Does the company have a due diligence (both internal and external) process to identify, prevent, mitigate and account for how they address their impacts on human rights. The due diligence process foresees the involvement of potentially impacted/critical stakeholders (with engagement of stakeholders)</t>
+          <t>Does the company communicate externally the Human Rights policy? How?</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ALERION.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company have a due diligence (both internal and external) process to identify, prevent, mitigate and account for how they address their impacts on human rights. The due diligence process foresees the involvement of potentially impacted/critical stakeholders (with engagement of stakeholders)', 'context': [Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='0153dba1-989b-499c-8c5b-c77f6093a1fc', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='criteria described in Section 2.1;  \n \n- Monitoring the Eligible Green Project portfolio;  \n \n- Managing any future update of the Green Bond Framework.  \n \n \n2.3-Management of proceeds \n \nUpon receipt, the net proceeds from the Green Bond  2021 – 2027 issuance will be \nmanaged by Alerion’s Treasury Department and invested in cash or cash equivalents \nuntil allocation to Eligible Green Projects. Alerion will aim at achieving complete'), Document(id='0286a4fd-14d3-46e6-a8c3-ddf45c3eb47d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='The Committee will be chaired by the Chairman of the Board of Directors, and composed \nof the other Board Executive Directors, together with the Chief Financial Officer and \nChief Operating Officer. \n \nThe Committee will be in charge of monitoring the selection and allocation of funds to \nEligible Green Projects and will be responsible for the following: \n \n- Identifying potential Eligible Green Projects;  \n \n- Reviewing and approving the selection against the eligibility')], 'answer': 'Alerion does not mention a specific due diligence process in the provided context to identify, prevent, mitigate, and address impacts on human rights, nor does it describe stakeholder engagement for these impacts. The context focuses on the management, selection, and allocation of funds to green projects rather than explicitly addressing human rights due diligence.'}</t>
+          <t>Question: Does the company communicate externally the Human Rights policy? How?
+Answer: Yes
+Evidence: "promote the contents of the policy among its external stakeholders as well."
+Location: Page not specified</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Does the company have a grievances mechanism, if so, is it independent or concide with the whistleblowing mechanism?</t>
+          <t>Does the company provide incentives to the board and/or senior managers(at least one member) linked to the implementation of its human rights targets or policy commitments (at least one commitment/target)?</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ANTARES VISION.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company have a grievances mechanism, if so, is it independent or concide with the whistleblowing mechanism?', 'context': [Document(id='ff745af9-0b55-45fe-b814-b9544e9ff383', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 50, 'page_label': '51'}, page_content="Sustainability report / NFR 2022 51 \n \nWhistleblowing \n \nAs part of the regulatory provisions, Antares Vision S.p.A. has a whistleblowing system for people to report any matters while \nguaranteeing their anonymity through IT and cryptographic methods. This channel is accessible via the company's website \nand physical boxes , i.e. there is a specific online form ( https://www.antaresvision.com/whistleblowing), indicated in the"), Document(id='97d21e9d-4bc6-44b6-afaf-2599ca6683f1', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 50, 'page_label': '51'}, page_content='footer and a physical box at the offices, for which the keys are held by the chairman of the SB. Whistleblowing reports are \nhandled by the chairman of the SB and by the SB on a collegiate basis. At the date of publication of this document, no \nwhistleblowing reports have been received through this channel.  \n \n \nManagement systems  \n \n \n2-23  \n2-24  \n2-25  \n2-26  \n \nOver the years, Antares Vision Group has implemented a growth strategy, strengthening its competitive position, also through'), Document(id='618991ac-dc56-4be3-b6b3-dd9b161abd81', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content='The communication and reporting channel of actual or suspected violations of the policies adopted by AV Group is identified \nby a specific  procedure accessible within the website. The information provided is treated confidentially and, under any \ncircumstance, the maximum confidentiality of the identity of the persons making the reports is guaranteed. The objective of \nadopting this tool is to prevent non -compliance or irregularities within the organization, but also to involve all stakeholders')], 'answer': 'Antares Vision S.p.A. has a whistleblowing mechanism that acts as a grievances mechanism, ensuring anonymity and confidentiality for those reporting. The system is managed by the chairman of the Supervisory Board (SB) and the SB on a collegiate basis, ensuring independence in handling reports.'}</t>
+          <t>Question: Does the company provide incentives to the board and/or senior managers (at least one member) linked to the implementation of its human rights targets or policy commitments (at least one commitment/target)?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Does the company have a grievances mechanism, if so, is it independent or concide with the whistleblowing mechanism?</t>
+          <t>Does the company provide incentives to the board and/or senior managers(at least one member) linked to the implementation of its human rights targets or policy commitments (at least one commitment/target)?</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company have a grievances mechanism, if so, is it independent or concide with the whistleblowing mechanism?', 'context': [Document(id='ecc5d8b1-c24b-4fac-a9f8-18da48b1011b', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 129, 'page_label': '128'}, page_content='of HR, Legal Affairs, and the Group Internal Audit &amp; Risk Management function, which has \nthe task of receiving, analyzing, and, if needed, investigating and proposing disciplinary \nmeasures in relation to the reports received. The Policy also defines the three channels \nthrough which reports can be implemented: in addition to ordinary mail and a specific de -\ndicated e-mail address, a digital platform called e-Whistle  was developed and constitutes'), Document(id='cb135f1e-d0b4-40a6-81bb-d0405f12b39c', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 129, 'page_label': '128'}, page_content='a simple, secure, and confidential manner to handle reports and manage further confiden -\ntial exchanges of information between the whistleblower and the Committee for in-depth \nanalysis in full compliance with the requirements laid down by regulations. In compliance \nwith the general principles of confidentiality, non-retaliation, and the possibility of anony -\nmity, the Policy and the reporting channels guarantee every report is treated confidentially,'), Document(id='b6f67494-8931-406a-9f4e-85f3d9869e5a', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 129, 'page_label': '128'}, page_content='conduct Amplifon employees or third parties should be aware of, how they can be repor -\nted, as well as the related reporting methods. During 2022, the Whistleblowing Policy \nwas subject to further updates to continue the process of alignment with the reference \nprinciples on whistleblowing as well as international best practices 39.\nWHISTLEBLOWING COMMITTEE AND REPORTING CHANNELS \nThe Policy foresees the creation of a Whistleblowing Committee, composed of the heads')], 'answer': 'Amplifon has a whistleblowing mechanism, as described in the context. This mechanism appears to be an independent system with dedicated channels such as ordinary mail, a specific e-mail address, and the digital platform e-Whistle, used for confidential reporting and information exchanges. There is no separate mention of a distinct grievances mechanism, so it seems that the whistleblowing process also serves this purpose.'}</t>
+          <t>Question: Does the company provide incentives to the board and/or senior managers (at least one member) linked to the implementation of its human rights targets or policy commitments (at least one commitment/target)?
+Answer: Yes
+Evidence: "the remuneration of the directors of Antares Vision S.p.A is linked to the achievement of specific performance objectives, to which the disbursement of the variable, predetermined, measurable components is linked, and linked in significant part to a long-term horizon."
+Location: Page 3, Section "Corporate Governance"</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Does the company have a grievances mechanism, if so, is it independent or concide with the whistleblowing mechanism?</t>
+          <t>Does the company monitor the implementation of its human rights policy commitment(s) and disclose main achievements/corrective actions (e.g., on the sustainability report)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1002,14 +1098,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company have a grievances mechanism, if so, is it independent or concide with the whistleblowing mechanism?', 'context': [Document(id='0286a4fd-14d3-46e6-a8c3-ddf45c3eb47d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='The Committee will be chaired by the Chairman of the Board of Directors, and composed \nof the other Board Executive Directors, together with the Chief Financial Officer and \nChief Operating Officer. \n \nThe Committee will be in charge of monitoring the selection and allocation of funds to \nEligible Green Projects and will be responsible for the following: \n \n- Identifying potential Eligible Green Projects;  \n \n- Reviewing and approving the selection against the eligibility'), Document(id='3d9bdf42-9b67-4115-baee-08a6808ab3c1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Impact metrics:  \n \nAlerion will also provide information on the expected output and environmental benefits \nof Eligible Green Projects. \n \nThe relevant metrics1 will include:  \n \n-  Installed renewable energy capacity in MW  \n-  Expected or actual annual renewable energy generation in MWh \nor GWh  \n-  Estimated annual GHG emissions avoided (in tCO2e)  \n \n \n2.5- External review – Annual Assurance Report \n \nAn external independent auditor confirmed that the allocation of the Green Bond is done'), Document(id='f707bf4b-5cae-4faa-8441-9437175abc1d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='in accordance with Alerion’s 2021 Green Bond Framework and will provide, starting one \nyear after issuance and on an annual basis until all the proceeds of the Green Bon d \nhave been allocated, a limited assurance report.  \nThis Third-Party Opinion made by External independent auditor on ALERION Green Bond \nReport is attached to this document. \n \n3-Reporting criteria \nAllocation: The amount of the “Green Bond 2021 - 2027 Proceeds” have been approved')], 'answer': "Alerion does not provide information regarding a grievances mechanism or a whistleblowing mechanism in the given context. Therefore, it's unclear if such mechanisms exist or whether they are independent or coincide with each other."}</t>
+          <t>Question: Does the company monitor the implementation of its human rights policy commitment(s) and disclose main achievements/corrective actions (e.g., on the sustainability report)?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided text.
+Location: Page not specified</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Does the company have a processo to enable remediation of any adverse human rights impacts, the company may cause or to which it may contribute to?</t>
+          <t>Does the company monitor the implementation of its human rights policy commitment(s) and disclose main achievements/corrective actions (e.g., on the sustainability report)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1019,82 +1118,97 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company have a processo to enable remediation of any adverse human rights impacts, the company may cause or to which it may contribute to?', 'context': [Document(id='2ce894f0-88b0-40e9-bbc6-9bfd888ab135', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 110, 'page_label': '111'}, page_content='11 Human resources / HR policies  \n   \n  \n2.24 Embedding policy commitments 04 Sustainability: the commitment of AV Group  / \nResponsible business conduct \n   \n  \n  \n04 Sustainability: the commitment of AV Group / \nThe management Systems  \n   \n  \n  \n04 Sustainability: the commitment of AV Group / \nRelations with the territory \n   \n  \n2.25 Processes to remediate negative \nimpacts \n04 Sustainability: the commitment of AV Group / \nResponsible business conduct'), Document(id='5cb5e9ba-82dc-4639-8cfc-569ad2309e57', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="With the adoption of the Human Rights policy, which applies to all AV Group companies and provides for specific metho ds \nof implementation, employee training and monitoring, the Group intends to:  \n▪ strengthen its commitment to the protection of human rights in each country in which it operates,  \n▪ demonstrate the Group's awareness of the risks inherent in its business model, \n▪ promote the contents of the policy among its external stakeholders as well."), Document(id='2d37729e-8daa-478b-9d30-eb18aa8e6166', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 60, 'page_label': '61'}, page_content='document. \n \nIdentification of actual and potential impacts \nThe actual and potential impacts on the economy, the environment and people, including those on human rights, have been \nidentified through a process of analysis, which has included the consultation of external sources, internal sources, along with \nthe specific involvement of some categories of stakeholders, as part of the constant process of discussion and listening to \nthem.')], 'answer': 'AV Group has a process to remediate negative impacts, including adverse human rights impacts it may cause or contribute to. This commitment is part of their responsible business conduct under their sustainability initiatives. The process involves consultation with internal and external sources, as well as stakeholder involvement.'}</t>
+          <t>Question: Does the company monitor the implementation of its human rights policy commitment(s) and disclose main achievements/corrective actions (e.g., on the sustainability report)?
+Answer: Yes
+Evidence: "With the adoption of the Human Rights policy, which applies to all AV Group companies and provides for specific methods of implementation, employee training and monitoring, the Group intends to..." 
+Location: Page not specified</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Does the company have a processo to enable remediation of any adverse human rights impacts, the company may cause or to which it may contribute to?</t>
+          <t>Does the company consider material under GRI the Social Topic 414.1: New suppliers that were screened using social criteria? Alternatevely look for keywords: 414.1, GRI 414.1, GRI 414-1.</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company have a processo to enable remediation of any adverse human rights impacts, the company may cause or to which it may contribute to?', 'context': [Document(id='e2aa499c-a0d7-485f-a1a6-61e1ed14f55a', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 124, 'page_label': '123'}, page_content='inherent in the main ethical, social and environmental issues. There are specific actions to \nimplement for every class of risk to deepen the knowledge of the supplier and/or mitigate \nthe residual risks, including for example: the supplier completing a questionnaire clarifying \ncertain significant aspects, the inclusion of the supplier in an ESG evaluation/rating pro -\ncess, the execution of an ad hoc audit by an experienced third party with focusing on ESG \nissues.'), Document(id='06e99e70-ce08-469b-b3a3-9e2d601fdfcf', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='and management methods, as well as the GRI Standards reported are described.\nArea Principle Reference GRI Standards\nHuman Rights\n1. Business should support and \nrespect the protection of human rights \nproclaimed at an international level\n2. Businesses should ensure that they are \nnot complicit in violations of human rights\n• Well-being and internal engagement\n• Business ethics and fighting corruption\n• Procurement and Supply Chain \nmanagement\n• Note on methodology\n• GRI 2-23: Policy commitment'), Document(id='45852781-8efa-4f79-8ced-fa5dbbd7e573', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 186, 'page_label': '185'}, page_content='Information Reference Notes/Omissions\n2-21: Annual total compensation ratio Remuneration Report 2023,\n“Executive Summary”\nStrategies, policies and practices\n2-22: Statement on sustainable development strategy p. 4; 5\n2-23: Policy commitments p. 30; 36; 41; 126; 132; 140\n2-24: Embedding policy commitments p. 30; 36; 41; 126; 132; 140\n2-25: Processes to remediate negative impacts\np.31; Report on Corporate Governance \nand ownership structure at 31 December \n2022, section 4 “Board of Directors”')], 'answer': 'The company has processes to remediate negative impacts, as outlined on page 31 and detailed in the Report on Corporate Governance and ownership structure at 31 December 2022, section 4 "Board of Directors."'}</t>
+          <t>Question: Does the company consider material under GRI the Social Topic 414.1: New suppliers that were screened using social criteria?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided text.
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Does the company have a processo to enable remediation of any adverse human rights impacts, the company may cause or to which it may contribute to?</t>
+          <t>Does the company consider material under GRI the Social Topic 414.1: New suppliers that were screened using social criteria? Alternatevely look for keywords: 414.1, GRI 414.1, GRI 414-1.</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ALERION.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company have a processo to enable remediation of any adverse human rights impacts, the company may cause or to which it may contribute to?', 'context': [Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='8c8b278a-2039-4df6-a6f1-e4e4cd520379', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Pagina | 4  \n \n \nIn case of divestment, or if a project becomes ineligible, Alerion will strive to replace it \nby another Eligible Green Project on a best effort basis.   \n \n2.4- Reporting  \nAn annual report will be prepared and made available on Alerion’s website at \nwww.alerion.it, with the status of the Green Bond’s proceeds allocation, overview of the \nprojects financed or refinanced, and the environmental impact, until full allocation of \nproceeds.'), Document(id='1603dfa0-95cf-4193-b970-a97988e35cc1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 1, 'page_label': '2'}, page_content='further in Europe, both in \nwind and solar sector. \n Alerion’s exclusive focus \non renewable energy \nimplies that sustainability \nis strictly embedded in our \nbusiness model. Our \noperations contribute \ndirectly to the reduction of \ngreenhouse gas (GHG) \nemissions and to the \npromotion of a system for \nsustainable territorial \ndevelopment. To this end, \nwe have in place a strong \nintegrated system for the \nassessment and \nmanagement of our')], 'answer': "Alerion's provided context does not specify a process for enabling remediation of adverse human rights impacts. The information focuses on green bond allocation and project selection related to renewable energy initiatives. For specific details on human rights policies, additional context or direct inquiry to the company would be needed."}</t>
+          <t>Question: Does the company consider material under GRI the Social Topic 414.1: New suppliers that were screened using social criteria?
+Answer: Yes
+Evidence: "The integrated management system adopted by the parent company Antares Vision S.p.A provides for a specific procedure for the management, selection and qualification of suppliers."
+Location: Sustainability report / NFR 2022, Page 86</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Does the company offer trainings on human rights? If so, are they direct only to internal employees or also to main suppliers?</t>
+          <t>Does the company consider material under GRI the Social Topic 414.2: Negative social impacts in the supply chain and actions taken? Alternatevely look for keywords: 414.2, GRI 414.2, GRI 414-2</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ANTARES VISION.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company offer trainings on human rights? If so, are they direct only to internal employees or also to main suppliers?', 'context': [Document(id='5cb5e9ba-82dc-4639-8cfc-569ad2309e57', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="With the adoption of the Human Rights policy, which applies to all AV Group companies and provides for specific metho ds \nof implementation, employee training and monitoring, the Group intends to:  \n▪ strengthen its commitment to the protection of human rights in each country in which it operates,  \n▪ demonstrate the Group's awareness of the risks inherent in its business model, \n▪ promote the contents of the policy among its external stakeholders as well."), Document(id='513e0a88-c843-4f4d-b50c-679550c94940', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content='company and its subsidiaries through the organization of information and training sessions held in person and online.  \nIn line with what is reported in the Code of Ethics,  managers are accountable, both individually and collectively, for their \ncommitment to ethical and respectful conduct. They also have a duty to ensure that these standards are maintained in their \narea of responsibility and to take appropriate measures should t his not occur. Furthermore, everyone is individually'), Document(id='c09dfbd4-e6ab-4ffb-9f76-8868577d23ee', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 62, 'page_label': '63'}, page_content='Ability to attract and retain talent and \nprovide the talent with support in its \nprofessional growth/development \nactual: training plans aimed at developing \nskills \nGRI 401 \nEmployment \n \nGRI 404 Training \nand education \nPersonnel \ndirect: related to direct activities only  Respect for \nhuman \nrights')], 'answer': 'AV Group offers trainings on human rights, which are intended for both internal employees and external stakeholders, as mentioned in the context.'}</t>
+          <t>Question: Does the company consider material under GRI the Social Topic 414.2: Negative social impacts in the supply chain and actions taken?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Does the company offer trainings on human rights? If so, are they direct only to internal employees or also to main suppliers?</t>
+          <t>Does the company consider material under GRI the Social Topic 414.2: Negative social impacts in the supply chain and actions taken? Alternatevely look for keywords: 414.2, GRI 414.2, GRI 414-2</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company offer trainings on human rights? If so, are they direct only to internal employees or also to main suppliers?', 'context': [Document(id='c82bcb4f-0397-45f0-acbf-8ae562c05023', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 124, 'page_label': '123'}, page_content='ning the principles and standards of conduct required by all suppliers and business partners \nwith respect to the areas of business ethics, compliance, anti-corruption, human rights and \nworkers’ rights, diversity and inclusion, health, safety, the environment, etc.37.\nDuring the year, the mandatory acceptance of this Code was included in the qualification \nprocess for new suppliers, so that any new supplier signs up to it and its proactive imple -'), Document(id='69ea3a9c-a1d6-43d5-9d26-0ce15731a5d2', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 128, 'page_label': '127'}, page_content='functions also within the compliance and/or organizational field.\nON “BUSINESS &amp; ETHICS” \nPROVIDED IN 2022 TO \nOVER 1,800 EMPLOYEES\n+1,970\nTOTAL HOURS OF \nTRAINING \nINTRODUCTION   •   AMPLIFON: LISTENING AHEAD   •   PRODUCT &amp; SERVICE STEWARDSHIP   •   PEOPLE EMPOWERMENT   •   COMMUNITY IMPACT   •   ETHICAL BEHAVIOR    •   ANNEX\n127'), Document(id='e2aa499c-a0d7-485f-a1a6-61e1ed14f55a', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 124, 'page_label': '123'}, page_content='inherent in the main ethical, social and environmental issues. There are specific actions to \nimplement for every class of risk to deepen the knowledge of the supplier and/or mitigate \nthe residual risks, including for example: the supplier completing a questionnaire clarifying \ncertain significant aspects, the inclusion of the supplier in an ESG evaluation/rating pro -\ncess, the execution of an ad hoc audit by an experienced third party with focusing on ESG \nissues.')], 'answer': "Amplifon provides training related to business ethics, which encompasses areas such as human rights. The training is specifically mentioned for over 1,800 employees, but there is no explicit mention of training being offered directly to main suppliers. The qualification process for new suppliers includes mandatory acceptance of the company's code regarding ethical standards, which implies some level of awareness is required from suppliers but it does not specify training."}</t>
+          <t>Question: Does the company consider material under GRI the Social Topic 414.2: Negative social impacts in the supply chain and actions taken?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Does the company offer trainings on human rights? If so, are they direct only to internal employees or also to main suppliers?</t>
+          <t>Does the company consider material under GRI the Topic 202.1: Market presence -Ratios of standard entry level wage by gender compared to local minimum wage? Alternatevely look for keywords: 202.1, GRI 202.1, GRI 202-1,minimum wage, fair wage,living wage, fair compensation, minimum compensation</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1104,14 +1218,16 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company offer trainings on human rights? If so, are they direct only to internal employees or also to main suppliers?', 'context': [Document(id='1603dfa0-95cf-4193-b970-a97988e35cc1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 1, 'page_label': '2'}, page_content='further in Europe, both in \nwind and solar sector. \n Alerion’s exclusive focus \non renewable energy \nimplies that sustainability \nis strictly embedded in our \nbusiness model. Our \noperations contribute \ndirectly to the reduction of \ngreenhouse gas (GHG) \nemissions and to the \npromotion of a system for \nsustainable territorial \ndevelopment. To this end, \nwe have in place a strong \nintegrated system for the \nassessment and \nmanagement of our'), Document(id='8c8b278a-2039-4df6-a6f1-e4e4cd520379', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Pagina | 4  \n \n \nIn case of divestment, or if a project becomes ineligible, Alerion will strive to replace it \nby another Eligible Green Project on a best effort basis.   \n \n2.4- Reporting  \nAn annual report will be prepared and made available on Alerion’s website at \nwww.alerion.it, with the status of the Green Bond’s proceeds allocation, overview of the \nprojects financed or refinanced, and the environmental impact, until full allocation of \nproceeds.'), Document(id='3d9bdf42-9b67-4115-baee-08a6808ab3c1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Impact metrics:  \n \nAlerion will also provide information on the expected output and environmental benefits \nof Eligible Green Projects. \n \nThe relevant metrics1 will include:  \n \n-  Installed renewable energy capacity in MW  \n-  Expected or actual annual renewable energy generation in MWh \nor GWh  \n-  Estimated annual GHG emissions avoided (in tCO2e)  \n \n \n2.5- External review – Annual Assurance Report \n \nAn external independent auditor confirmed that the allocation of the Green Bond is done')], 'answer': 'Alerion does not mention offering trainings on human rights in the provided context, so it is unclear whether such trainings are directed only to internal employees or also to main suppliers.'}</t>
+          <t>Answer: Information not explicitly disclosed
+Evidence: "Alerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of wind and/or solar power generation projects, as previously described."
+Location: Page not specified</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Does the company communicate internally the Human Rights policy? How?</t>
+          <t>Does the company consider material under GRI the Topic 202.1: Market presence -Ratios of standard entry level wage by gender compared to local minimum wage? Alternatevely look for keywords: 202.1, GRI 202.1, GRI 202-1,minimum wage, fair wage,living wage, fair compensation, minimum compensation</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1121,82 +1237,96 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company communicate internally the Human Rights policy? How?', 'context': [Document(id='5cb5e9ba-82dc-4639-8cfc-569ad2309e57', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="With the adoption of the Human Rights policy, which applies to all AV Group companies and provides for specific metho ds \nof implementation, employee training and monitoring, the Group intends to:  \n▪ strengthen its commitment to the protection of human rights in each country in which it operates,  \n▪ demonstrate the Group's awareness of the risks inherent in its business model, \n▪ promote the contents of the policy among its external stakeholders as well."), Document(id='bebc898a-2b45-453e-81c9-c8275f7216bf', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content='document.  \nLastly, specific methods have been adopted for checking the compliance of the behaviour of anyone acting on their own \nbehalf or within their work context, with the provisions of current legislation and with the rules of conduct established by the \npolicies and procedures adopted. \n \nHuman rights \n \nIn continuity with its values, the commitment defined in the Code of Ethics, AV Group adopted a specific Human Rights Policy'), Document(id='a5d4344c-bcff-442c-b0c1-8d73418a53a6', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="on 31 Jan uary 2023. This choice intends to reaffirm the importance of respect for human rights and strengthen the AV \nGroup's commitment to safeguarding them, in every country in which it operates. \n \nThe policy, available on the Antares Vision Group website  (Company Documents | Group Policies), has been developed in \naccordance with the main international human rights conventions, standards and recommendations (International Bill of")], 'answer': 'AV Group communicates its Human Rights policy internally through employee training and monitoring. They have adopted specific methods for ensuring compliance and are committed to promoting the policy within their work context.'}</t>
+          <t>Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the sustainability report.
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Does the company communicate internally the Human Rights policy? How?</t>
+          <t>Does the company consider material under GRI theTopic 205: Anti-corruption? Alternatevely look for keywords: 205, GRI 205, GRI 205, corruption, anti corruption, anti-corruption</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company communicate internally the Human Rights policy? How?', 'context': [Document(id='7211d830-b72d-4e58-8b96-1aacac1013a7', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 150, 'page_label': '149'}, page_content='• DEIB (Diversity, Equity, Inclusion, Belonging) Policy and establishment of a DEIB Global Governance\n• Training, communication, and internal engagement activities\n• Implementation of specific action plans following the Global Engagement Survey “Your Voice”\n• Membership of the United Nations Global Compact \n• Smart Working Policy \n• Package of flexible benefits \n• Short and long-term incentive schemes\nAwareness-raising and \neducation on hearing well-\nbeing\nPotential reputational risks related to'), Document(id='988094d5-645e-4e2c-a290-25ae3516837d', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 149, 'page_label': '148'}, page_content='• DEIB (Diversity, Equity, Inclusion, Belonging) Policy and establishment of a DEIB Global Governance\n• Training, communication, and internal engagement activities\n• Implementation of specific action plans following the Global Engagement Survey “Your Voice”\n• Membership of the United Nations Global Compact \n• Smart Working Policy \n• Package of flexible benefits \n• Short and long-term incentive schemes\nAwareness-raising and \neducation on hearing well-\nbeing\nPotential reputational risks related to'), Document(id='a0026abd-c35d-47a4-a24f-0ab156e90b95', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 75, 'page_label': '74'}, page_content='WELL-BEING AND INTERNAL ENGAGEMENT \nIn line with the UN Global Compact principles, the Universal Declaration of Human Rights, \nand in compliance with the International Labor Organization Conventions on Fundamental \nHuman Rights, Amplifon is committed to complying with the fundamental human rights \nand labor rights in all the countries where we operate , both in business activities and \nunder the scope of relations with third parties, renouncing to all forms of exploitative for -')], 'answer': 'Amplifon communicates its Human Rights policy internally through training, communication, and internal engagement activities. These initiatives are designed to align with the UN Global Compact principles and the Universal Declaration of Human Rights, ensuring awareness and compliance among employees.'}</t>
+          <t>Question: Does the company consider material under GRI the Topic 205: Anti-corruption?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided text.
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Does the company communicate internally the Human Rights policy? How?</t>
+          <t>Does the company consider material under GRI theTopic 205: Anti-corruption? Alternatevely look for keywords: 205, GRI 205, GRI 205, corruption, anti corruption, anti-corruption</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ALERION.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company communicate internally the Human Rights policy? How?', 'context': [Document(id='0286a4fd-14d3-46e6-a8c3-ddf45c3eb47d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='The Committee will be chaired by the Chairman of the Board of Directors, and composed \nof the other Board Executive Directors, together with the Chief Financial Officer and \nChief Operating Officer. \n \nThe Committee will be in charge of monitoring the selection and allocation of funds to \nEligible Green Projects and will be responsible for the following: \n \n- Identifying potential Eligible Green Projects;  \n \n- Reviewing and approving the selection against the eligibility'), Document(id='8c8b278a-2039-4df6-a6f1-e4e4cd520379', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Pagina | 4  \n \n \nIn case of divestment, or if a project becomes ineligible, Alerion will strive to replace it \nby another Eligible Green Project on a best effort basis.   \n \n2.4- Reporting  \nAn annual report will be prepared and made available on Alerion’s website at \nwww.alerion.it, with the status of the Green Bond’s proceeds allocation, overview of the \nprojects financed or refinanced, and the environmental impact, until full allocation of \nproceeds.'), Document(id='0153dba1-989b-499c-8c5b-c77f6093a1fc', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='criteria described in Section 2.1;  \n \n- Monitoring the Eligible Green Project portfolio;  \n \n- Managing any future update of the Green Bond Framework.  \n \n \n2.3-Management of proceeds \n \nUpon receipt, the net proceeds from the Green Bond  2021 – 2027 issuance will be \nmanaged by Alerion’s Treasury Department and invested in cash or cash equivalents \nuntil allocation to Eligible Green Projects. Alerion will aim at achieving complete')], 'answer': 'Alerion does not specify in the provided context if or how it communicates its Human Rights policy internally.'}</t>
+          <t>Question: Does the company consider material under GRI the Topic 205: Anti-corruption?
+Answer: Yes
+Evidence: "As mapped by the risk analysis and management model and reported in the Anti-Corruption policy, Antares Vision Group applies an assessment of the risks associated with corruption for all the operations in which it is involved."
+Location: Page 77, Sustainability report / NFR 2022</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Does the company communicate externally the Human Rights policy? How?</t>
+          <t>Does the company consider material under GRI theTopic 403: Occupational Health and Safety including maximum working hours of 48 or 60 including overtime? Alternatevely look for keywords: 403, GRI 403, health and safety, working hours, health, safety</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ANTARES VISION.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company communicate externally the Human Rights policy? How?', 'context': [Document(id='5cb5e9ba-82dc-4639-8cfc-569ad2309e57', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="With the adoption of the Human Rights policy, which applies to all AV Group companies and provides for specific metho ds \nof implementation, employee training and monitoring, the Group intends to:  \n▪ strengthen its commitment to the protection of human rights in each country in which it operates,  \n▪ demonstrate the Group's awareness of the risks inherent in its business model, \n▪ promote the contents of the policy among its external stakeholders as well."), Document(id='bebc898a-2b45-453e-81c9-c8275f7216bf', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content='document.  \nLastly, specific methods have been adopted for checking the compliance of the behaviour of anyone acting on their own \nbehalf or within their work context, with the provisions of current legislation and with the rules of conduct established by the \npolicies and procedures adopted. \n \nHuman rights \n \nIn continuity with its values, the commitment defined in the Code of Ethics, AV Group adopted a specific Human Rights Policy'), Document(id='a5d4344c-bcff-442c-b0c1-8d73418a53a6', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="on 31 Jan uary 2023. This choice intends to reaffirm the importance of respect for human rights and strengthen the AV \nGroup's commitment to safeguarding them, in every country in which it operates. \n \nThe policy, available on the Antares Vision Group website  (Company Documents | Group Policies), has been developed in \naccordance with the main international human rights conventions, standards and recommendations (International Bill of")], 'answer': 'AV Group promotes the contents of its Human Rights policy among its external stakeholders. The policy is available on the Antares Vision Group website under Company Documents and Group Policies. This indicates their effort to communicate the policy externally.'}</t>
+          <t>Question: Does the company consider material under GRI the Topic 403: Occupational Health and Safety including maximum working hours of 48 or 60 including overtime?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Does the company communicate externally the Human Rights policy? How?</t>
+          <t>Does the company consider material under GRI theTopic 403: Occupational Health and Safety including maximum working hours of 48 or 60 including overtime? Alternatevely look for keywords: 403, GRI 403, health and safety, working hours, health, safety</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company communicate externally the Human Rights policy? How?', 'context': [Document(id='988094d5-645e-4e2c-a290-25ae3516837d', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 149, 'page_label': '148'}, page_content='• DEIB (Diversity, Equity, Inclusion, Belonging) Policy and establishment of a DEIB Global Governance\n• Training, communication, and internal engagement activities\n• Implementation of specific action plans following the Global Engagement Survey “Your Voice”\n• Membership of the United Nations Global Compact \n• Smart Working Policy \n• Package of flexible benefits \n• Short and long-term incentive schemes\nAwareness-raising and \neducation on hearing well-\nbeing\nPotential reputational risks related to'), Document(id='7211d830-b72d-4e58-8b96-1aacac1013a7', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 150, 'page_label': '149'}, page_content='• DEIB (Diversity, Equity, Inclusion, Belonging) Policy and establishment of a DEIB Global Governance\n• Training, communication, and internal engagement activities\n• Implementation of specific action plans following the Global Engagement Survey “Your Voice”\n• Membership of the United Nations Global Compact \n• Smart Working Policy \n• Package of flexible benefits \n• Short and long-term incentive schemes\nAwareness-raising and \neducation on hearing well-\nbeing\nPotential reputational risks related to'), Document(id='a0026abd-c35d-47a4-a24f-0ab156e90b95', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 75, 'page_label': '74'}, page_content='WELL-BEING AND INTERNAL ENGAGEMENT \nIn line with the UN Global Compact principles, the Universal Declaration of Human Rights, \nand in compliance with the International Labor Organization Conventions on Fundamental \nHuman Rights, Amplifon is committed to complying with the fundamental human rights \nand labor rights in all the countries where we operate , both in business activities and \nunder the scope of relations with third parties, renouncing to all forms of exploitative for -')], 'answer': 'Amplifon communicates externally its commitment to human rights by adhering to international frameworks such as the UN Global Compact and the Universal Declaration of Human Rights. The company is committed to complying with labor and human rights in all their operations and relationships with third parties across the globe. This commitment is likely communicated through their membership in the UN Global Compact and related public statements or reports.'}</t>
+          <t>Question: Does the company consider material under GRI the Topic 403: Occupational Health and Safety including maximum working hours of 48 or 60 including overtime?
+Answer: Yes
+Evidence: "We have a comprehensive occupational health and safety management system in place, including hazard identification, risk assessment, incident investigation, worker participation, consultation, communication, training, promotion of worker health, and prevention and mitigation of occupational health and safety impacts directly linked by business relationships." 
+Location: Page 11, Section "Human Resources / Health and Safety of workers"</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Does the company communicate externally the Human Rights policy? How?</t>
+          <t>Does the company consider material under GRI theTopic 405.1: Diversity of governance bodies and employees? Alternatevely look for keywords: 405.1, GRI 405.1, GRI 405-1, 405-1, gender diversity, equal opportunities</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1206,14 +1336,18 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company communicate externally the Human Rights policy? How?', 'context': [Document(id='8c8b278a-2039-4df6-a6f1-e4e4cd520379', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Pagina | 4  \n \n \nIn case of divestment, or if a project becomes ineligible, Alerion will strive to replace it \nby another Eligible Green Project on a best effort basis.   \n \n2.4- Reporting  \nAn annual report will be prepared and made available on Alerion’s website at \nwww.alerion.it, with the status of the Green Bond’s proceeds allocation, overview of the \nprojects financed or refinanced, and the environmental impact, until full allocation of \nproceeds.'), Document(id='8e92e81d-a44b-4d44-84b0-f8274704ad43', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 0, 'page_label': '1'}, page_content='Pagina | 0  \n \n \n  \nAnnual report prepared and made \navailable on Alerion’s website at \nwww.alerion.it, with the status of \nthe Green Bond’s proceeds \nallocation, overview of the projects \nfinanced or refinanced, and the \nenvironmental impact, until full \nallocation of proceeds. \nALERION \nGREEN BOND     \n2021–2027 \n_________ \nREPORT  \nYEAR 2022 \nUse of Proceeds'), Document(id='d92ded8b-d43e-4c82-bbff-33a71d9d335f', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 2, 'page_label': '3'}, page_content="In particular, over the next years, Alerion will focus its strategy on the acceleration of \ngrowth with an increasingly broad geographical diversification in Italy, Spain and \nRomania, and on technological diversification, through a plan of investments in the solar \nsector. \n2- GREEN BOND FRAMEWORK \nIn order to increase transparency of the Alerion Green Bond 20 21 - 2027, Alerion has \npublished the “Alerion 2021 Green Bond Framework” in line with ICMA's Green Bond")], 'answer': 'Alerion does not provide explicit information about communicating a Human Rights policy externally in the given context. The focus is mainly on their Green Bond activities and allocation reports. Further details would require additional information not provided in the context.'}</t>
+          <t>Question: Does the company consider material under GRI the Topic 405.1: Diversity of governance bodies and employees?
+Answer: Yes
+Evidence: "The Committee will be chaired by the Chairman of the Board of Directors, and composed of the other Board Executive Directors, together with the Chief Financial Officer and Chief Operating Officer."
+Location: Page not specified
+Context: The composition of the Green Bond Committee, as described in the report, indicates consideration of diversity within governance bodies, meeting the criteria of GRI 405.1 regarding the diversity of governance bodies.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Does the company provide incentives to the board and/or senior managers(at least one member) linked to the implementation of its human rights targets or policy commitments (at least one commitment/target)?</t>
+          <t>Does the company consider material under GRI theTopic 405.1: Diversity of governance bodies and employees? Alternatevely look for keywords: 405.1, GRI 405.1, GRI 405-1, 405-1, gender diversity, equal opportunities</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1223,82 +1357,97 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company provide incentives to the board and/or senior managers(at least one member) linked to the implementation of its human rights targets or policy commitments (at least one commitment/target)?', 'context': [Document(id='5920a917-057a-4b9b-8add-135a2cff7d85', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 89, 'page_label': '90'}, page_content="and no direction). Objectives more linked to sustainability and ESG values may also be introduced. \n \nPerformance management system - Compensation &amp; benefit policy \n \nAntares Vision S.p.A. ha s, among its corporate objectives, the enhancement of human capital and the development of \npeople's strategic skills . Merit is the guiding principle of managerial actions and rewards, both in terms of professional"), Document(id='2009416d-9cd9-4824-bef3-afd0971daa04', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 38, 'page_label': '39'}, page_content="the remuneration of the directors of Antares Vision S.p.A is linked to the achievement of specific performance objectives, to \nwhich the disbursement of the variable, predetermined, measurable components is linked, and linked in significant part to a \nlong-term horizon. This are consistent with the Company's strategic objectives and is aimed at promoting its sustainable \nsuccess, including non-financial parameters as well."), Document(id='1c480421-1b27-41c0-a837-6bcbb4d5bc51', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 110, 'page_label': '111'}, page_content='2.18 Evaluation of the performance of the \nhighest governance body \n03 Governance / Corporate Governance \n   \n  \n2.19 Remuneration policies 03 Governance / Corporate Governance \n   \n  \n2.20 Process to determine remuneration 03 Governance / Corporate Governance \n   \n  \n2.21 Annual total compensation ratio 03 Governance / Corporate Governance \n \nInformation \nunavailable / \nincomplete \nData related in \nrelation to the parent \ncompany alone. / \nHarmonization / \nBasic mapping of \nretribution data in')], 'answer': 'Antares Vision S.p.A. links the remuneration of its directors to the achievement of specific performance objectives, which include sustainable success and non-financial parameters. However, there is no specific mention of incentives directly tied to the implementation of human rights targets or policy commitments. Hence, it is unknown if human rights specifically are included as a commitment or target in their incentive structure.'}</t>
+          <t>Question: Does the company consider material under GRI the Topic 405.1: Diversity of governance bodies and employees?
+Answer: Yes
+Evidence: "Creation of a work environment that guarantees respect, equal opportunities, diversity and inclusion for all workers and protects them against all forms of discrimination."
+Location: Page 8, Section "Human resources: Diversity Equity Inclusion"</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Does the company provide incentives to the board and/or senior managers(at least one member) linked to the implementation of its human rights targets or policy commitments (at least one commitment/target)?</t>
+          <t xml:space="preserve">Does the company consider material under GRI theTopic 405.2: Ratio of basic salary and remuneration of women to men? Alternatevely look for keywords: 405.2, GRI 405.2, GRI 405-2, 405-2, gender pay gap, pay equality, equal pay for equal work, </t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company provide incentives to the board and/or senior managers(at least one member) linked to the implementation of its human rights targets or policy commitments (at least one commitment/target)?', 'context': [Document(id='45852781-8efa-4f79-8ced-fa5dbbd7e573', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 186, 'page_label': '185'}, page_content='Information Reference Notes/Omissions\n2-21: Annual total compensation ratio Remuneration Report 2023,\n“Executive Summary”\nStrategies, policies and practices\n2-22: Statement on sustainable development strategy p. 4; 5\n2-23: Policy commitments p. 30; 36; 41; 126; 132; 140\n2-24: Embedding policy commitments p. 30; 36; 41; 126; 132; 140\n2-25: Processes to remediate negative impacts\np.31; Report on Corporate Governance \nand ownership structure at 31 December \n2022, section 4 “Board of Directors”'), Document(id='749e9c3b-eda7-45a3-b073-5cbd91a7ddbd', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 89, 'page_label': '88'}, page_content='through specific KPIs related to one’s function and at least one of them is tied to the \ntargets of the Sustainability Plan . As confirmation of Amplifon’s increasing focus on ESG \nissues, in 2021 an in-depth analysis was activated with regard to the definition of a new \nrewards-based remuneration tool intended, in the first instance for 2022, for the Chief Exe-\ncutive Officer/General Manager, and planned, from 2023 onwards, for Key Managers with'), Document(id='58a4a75d-c43e-4b84-b86e-10fbb50d41d2', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 89, 'page_label': '88'}, page_content='Strategic Responsibilities. This would allow to consolidate a policy with the strong involve -\nment of the Company’s key resources in the pursuit of the ESG goals. This remunerative \ncomponent points at guaranteeing both the safeguard of sustainability related issues, and \nthe creation of value in the medium/long-term, incentivizing greater alignment between \nthe interests of Top Management, shareholders and all stakeholders. This goal is actually')], 'answer': 'Amplifon provides a remuneration tool that incentivizes the Chief Executive Officer/General Manager and, from 2023, Key Managers with Strategic Responsibilities, aligning their interests with ESG goals. This includes targets tied to sustainability, which may encompass human rights targets or policy commitments. These incentives focus on safeguarding sustainability-related issues and creating long-term value.'}</t>
+          <t>Question: Does the company consider material under GRI the Topic 405.2: Ratio of basic salary and remuneration of women to men?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Does the company provide incentives to the board and/or senior managers(at least one member) linked to the implementation of its human rights targets or policy commitments (at least one commitment/target)?</t>
+          <t xml:space="preserve">Does the company consider material under GRI theTopic 405.2: Ratio of basic salary and remuneration of women to men? Alternatevely look for keywords: 405.2, GRI 405.2, GRI 405-2, 405-2, gender pay gap, pay equality, equal pay for equal work, </t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ALERION.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company provide incentives to the board and/or senior managers(at least one member) linked to the implementation of its human rights targets or policy commitments (at least one commitment/target)?', 'context': [Document(id='0286a4fd-14d3-46e6-a8c3-ddf45c3eb47d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='The Committee will be chaired by the Chairman of the Board of Directors, and composed \nof the other Board Executive Directors, together with the Chief Financial Officer and \nChief Operating Officer. \n \nThe Committee will be in charge of monitoring the selection and allocation of funds to \nEligible Green Projects and will be responsible for the following: \n \n- Identifying potential Eligible Green Projects;  \n \n- Reviewing and approving the selection against the eligibility'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.')], 'answer': 'Alerion does not mention providing incentives to the board or senior managers linked to the implementation of its human rights targets or policy commitments in the given context.'}</t>
+          <t>Question: Does the company consider material under GRI the Topic 405.2: Ratio of basic salary and remuneration of women to men?
+Answer: Information not explicitly disclosed
+Evidence: "Information unavailable / incomplete Data related in relation to the parent company alone." 
+Location: Sustainability report / NFR 2022 114</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Does the company monitor the implementation of its human rights policy commitment(s) and disclose main achievements/corrective actions (e.g., on the sustainability report)</t>
+          <t>Does the company consider material under GRI theTopic 406: Non discrimination? Alternatevely look for keywords: 406, GRI 406 , Non-discrimination, discrimination,  gender equality, gender, disability,nationality, age, sex, diversity, sexual orientation</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ANTARES VISION.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company monitor the implementation of its human rights policy commitment(s) and disclose main achievements/corrective actions (e.g., on the sustainability report)', 'context': [Document(id='7f37de2b-2de2-48b6-b0e3-bdfb2f414ac5', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 66, 'page_label': '67'}, page_content='Human Rights policies at Group level \n \n5.5  \n6 Occupational health and \nsafety  \nMaintaining high safety standards and minimum \ninjury rates \n \nEvaluation of the adoption and extension to other \nGroup companies of management systems and \nbest practices in the field of occupational health \nand safety \n \n8.8  \n7 Product quality / Customer \nhealth and safety \nMaintaining high quality standards of the solutions \noffered, also through screening and evaluation of'), Document(id='2ce894f0-88b0-40e9-bbc6-9bfd888ab135', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 110, 'page_label': '111'}, page_content='11 Human resources / HR policies  \n   \n  \n2.24 Embedding policy commitments 04 Sustainability: the commitment of AV Group  / \nResponsible business conduct \n   \n  \n  \n04 Sustainability: the commitment of AV Group / \nThe management Systems  \n   \n  \n  \n04 Sustainability: the commitment of AV Group / \nRelations with the territory \n   \n  \n2.25 Processes to remediate negative \nimpacts \n04 Sustainability: the commitment of AV Group / \nResponsible business conduct'), Document(id='5cb5e9ba-82dc-4639-8cfc-569ad2309e57', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="With the adoption of the Human Rights policy, which applies to all AV Group companies and provides for specific metho ds \nof implementation, employee training and monitoring, the Group intends to:  \n▪ strengthen its commitment to the protection of human rights in each country in which it operates,  \n▪ demonstrate the Group's awareness of the risks inherent in its business model, \n▪ promote the contents of the policy among its external stakeholders as well.")], 'answer': 'AV Group intends to monitor the implementation of its Human Rights policy through employee training and specific methods. However, the context provided does not specify whether AV Group discloses its main achievements or corrective actions related to this policy in a sustainability report. Therefore, it is unclear from the context whether such disclosures are made.'}</t>
+          <t>Question: Does the company consider material under GRI the Topic 406: Non-discrimination?
+Answer: Yes
+Evidence: "Alerion is committed to promoting diversity and inclusion and does not tolerate any form of discrimination based on gender, age, nationality, disability, sexual orientation, or any other characteristic protected by law." 
+Location: Page 7, Section "Diversity and Inclusion"</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Does the company monitor the implementation of its human rights policy commitment(s) and disclose main achievements/corrective actions (e.g., on the sustainability report)</t>
+          <t>Does the company consider material under GRI theTopic 406: Non discrimination? Alternatevely look for keywords: 406, GRI 406 , Non-discrimination, discrimination,  gender equality, gender, disability,nationality, age, sex, diversity, sexual orientation</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company monitor the implementation of its human rights policy commitment(s) and disclose main achievements/corrective actions (e.g., on the sustainability report)', 'context': [Document(id='365fefe8-3254-4432-aa18-36f106997d02', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 7, 'page_label': '6'}, page_content='254/2016. From 2021, it also includes the progress made within the application of the Ten \nPrinciples promoted by the United Nations Global Compact , which we are signatories of. \nWith this Report, every year we seize the chance to communicate to all our stakeholders \nthe progress achieved with respect to the four areas of commitment formalized within \nour Sustainability Policy  ( Product &amp; Service Stewardship, People Empowerment,'), Document(id='45852781-8efa-4f79-8ced-fa5dbbd7e573', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 186, 'page_label': '185'}, page_content='Information Reference Notes/Omissions\n2-21: Annual total compensation ratio Remuneration Report 2023,\n“Executive Summary”\nStrategies, policies and practices\n2-22: Statement on sustainable development strategy p. 4; 5\n2-23: Policy commitments p. 30; 36; 41; 126; 132; 140\n2-24: Embedding policy commitments p. 30; 36; 41; 126; 132; 140\n2-25: Processes to remediate negative impacts\np.31; Report on Corporate Governance \nand ownership structure at 31 December \n2022, section 4 “Board of Directors”'), Document(id='e55b514a-22ef-4008-b139-499dc6785452', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 152, 'page_label': '151'}, page_content='Transition - Policy\n• Training and internal engagement activities\n• Induction sessions with Top Management and main corporate functions\n• Monitoring sector and market macro-trends and regulatory development on \nclimate change\n•  Annual Non-Financial Statement\n•  Progress in the reporting exercise in line with the TCFD recommendations\n• Sustainability Plan and target to increase the amount of electricity purchased \nfrom renewable sources\n• Adoption of a Suppliers Code of Conduct')], 'answer': 'The company provides reports on its progress related to sustainability, including human rights commitments, as indicated in its Sustainability Policy. However, specific details on the monitoring and disclosure of achievements or corrective actions regarding human rights policy commitments are not explicitly mentioned. Therefore, it is unclear if such detailed monitoring results are disclosed in their reports.'}</t>
+          <t>Question: Does the company consider material under GRI the Topic 406: Non-discrimination?
+Answer: Yes
+Evidence: "Creation of a work environment that guarantees respect, equal opportunities, diversity and inclusion for all workers and protects them against all forms of discrimination."
+Location: Page 8, Section "Human resources: Diversity Equity Inclusion"</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Does the company monitor the implementation of its human rights policy commitment(s) and disclose main achievements/corrective actions (e.g., on the sustainability report)</t>
+          <t>Does the company consider material under GRI theTopic 407: Freedom of Association and Collective Bargaining? Alternatevely look for keywords: 407, GRI 407 , NFreedom of association, Collective Bargaining, right to be represented, trade unions</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1308,14 +1457,17 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company monitor the implementation of its human rights policy commitment(s) and disclose main achievements/corrective actions (e.g., on the sustainability report)', 'context': [Document(id='8c8b278a-2039-4df6-a6f1-e4e4cd520379', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Pagina | 4  \n \n \nIn case of divestment, or if a project becomes ineligible, Alerion will strive to replace it \nby another Eligible Green Project on a best effort basis.   \n \n2.4- Reporting  \nAn annual report will be prepared and made available on Alerion’s website at \nwww.alerion.it, with the status of the Green Bond’s proceeds allocation, overview of the \nprojects financed or refinanced, and the environmental impact, until full allocation of \nproceeds.'), Document(id='8e92e81d-a44b-4d44-84b0-f8274704ad43', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 0, 'page_label': '1'}, page_content='Pagina | 0  \n \n \n  \nAnnual report prepared and made \navailable on Alerion’s website at \nwww.alerion.it, with the status of \nthe Green Bond’s proceeds \nallocation, overview of the projects \nfinanced or refinanced, and the \nenvironmental impact, until full \nallocation of proceeds. \nALERION \nGREEN BOND     \n2021–2027 \n_________ \nREPORT  \nYEAR 2022 \nUse of Proceeds'), Document(id='a9b21330-cda2-4466-a0d8-0257f28fc7ab', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='proceeds. \nIn particular, this report will include the following information:  \n \nAllocation information: \n \n- The total amount of investments and expenditures in Eligible \nGreen Projects  \n- The amount and percentage of new and existing projects \n(financing and refinancing)  \n- The balance of unallocated proceeds  \n- A brief description of the projects financed or refinanced with the \nGreen Bond  \n \nImpact metrics:')], 'answer': 'Alerion does not provide information in the given context regarding monitoring or disclosing the implementation of its human rights policy commitments or related achievements and corrective actions. The focus of the provided context is solely on the reporting of the Green Bond’s proceeds and related projects.'}</t>
+          <t>Question: Does the company consider material under GRI the Topic 407: Freedom of Association and Collective Bargaining?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI the Social Topic 414.1: New suppliers that were screened using social criteria? Alternatevely look for keywords: 414.1, GRI 414.1, GRI 414-1.</t>
+          <t>Does the company consider material under GRI theTopic 407: Freedom of Association and Collective Bargaining? Alternatevely look for keywords: 407, GRI 407 , NFreedom of association, Collective Bargaining, right to be represented, trade unions</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1325,82 +1477,94 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI the Social Topic 414.1: New suppliers that were screened using social criteria? Alternatevely look for keywords: 414.1, GRI 414.1, GRI 414-1.', 'context': [Document(id='fc6ab75b-7979-4060-a030-49305984f7ec', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 114, 'page_label': '115'}, page_content='Sustainability report / NFR 2022 115 \n \n  GRI Topic Standards           \n308 Environmental \nevaluation of suppliers \n10 Supply Chain  \n    \n308-1 New suppliers that were \nscreened using \nenvironmental criteria \n10 Supply Chain / Selection and evaluation of \nsuppliers \n    \n414 Social evaluation of \nsuppliers \n10 Supply Chain  \n    \n414-1 New suppliers that were \nscreened using social \ncriteria \n10 Supply Chain / Selection and evaluation of \nsuppliers \n    \nMaterial \nTopic \nData security and \nprivacy'), Document(id='12543286-6d20-4482-a6a8-75e4d13b794a', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 113, 'page_label': '114'}, page_content='417 Marketing and labelling \n     \n417-2 Incidents of non-\ncompliance concerning \nproduct and service \ninformation and labeling \n09 Quality, compliance and safety of the product \nand customers / The quality policy \n    \n417-3 Incidents of non-\ncompliance concerning \nmarketing \ncommunications \n09 Quality, compliance and safety of the product \nand customers / The quality policy  \n    \nMaterial \nTopic \nSuppliers: supply chain \nsustainability \n          \n3.3 Management of \nmaterial topics \n10 Supply Chain'), Document(id='049f39e8-aadd-4562-a36f-50d434c260a6', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 85, 'page_label': '86'}, page_content='Sustainability report / NFR 2022 86 \n \n10 Supply Chain \nSelection and evaluation of suppliers \n \n \n3-3  \n308-1  \n414-1  \n \nThe integrated management system adopted by the parent company Antares Vision S.p.A provides for a specific procedure \nfor the management, selection and qualification of suppliers. The objective is to ensure that the processes, products and \nservices provided comply with the requirements of the Integrated System, determining the intensity of the controls to be')], 'answer': 'Antares Vision S.p.A includes the Social Topic 414-1: New suppliers that were screened using social criteria in their sustainability report.'}</t>
+          <t>Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI the Social Topic 414.1: New suppliers that were screened using social criteria? Alternatevely look for keywords: 414.1, GRI 414.1, GRI 414-1.</t>
+          <t>Does the company consider material under GRI theTopic 408: Child Labour? Alternatevely look for keywords: GRI 408, 408, Child Labour, Child Labor, minor labour, minor labor, child work, child exploitation</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI the Social Topic 414.1: New suppliers that were screened using social criteria? Alternatevely look for keywords: 414.1, GRI 414.1, GRI 414-1.', 'context': [Document(id='c82bcb4f-0397-45f0-acbf-8ae562c05023', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 124, 'page_label': '123'}, page_content='ning the principles and standards of conduct required by all suppliers and business partners \nwith respect to the areas of business ethics, compliance, anti-corruption, human rights and \nworkers’ rights, diversity and inclusion, health, safety, the environment, etc.37.\nDuring the year, the mandatory acceptance of this Code was included in the qualification \nprocess for new suppliers, so that any new supplier signs up to it and its proactive imple -'), Document(id='dc6ca718-37dc-47e4-845b-f0d394f2347f', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 149, 'page_label': '148'}, page_content='• Acceptance of the Code of Ethics by suppliers through specific contractual clauses\n• Subscription of the Sustainability Policy by direct suppliers\n• Implementation of the Code of Conduct for Suppliers and progressive acceptance by suppliers\n• Definition of a new global framework for the evaluation of suppliers based on the main ESG risks\n• Integration of a Company figure dedicated to the management of ESG issues in procurement and supply chain activities'), Document(id='d0cb4f31-7c2c-4f45-a8a8-2938b4945090', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 150, 'page_label': '149'}, page_content='• Acceptance of the Code of Ethics by suppliers through specific contractual clauses\n• Subscription of the Sustainability Policy by direct suppliers\n• Implementation of the Code of Conduct for Suppliers and progressive acceptance by suppliers\n• Definition of a new global framework for the evaluation of suppliers based on the main ESG risks\n• Integration of a Company figure dedicated to the management of ESG issues in procurement and supply chain activities')], 'answer': 'The company does not specify the consideration of GRI Social Topic 414.1: New suppliers that were screened using social criteria.'}</t>
+          <t>Question: Does the company consider material under GRI the Topic 408: Child Labour?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI the Social Topic 414.1: New suppliers that were screened using social criteria? Alternatevely look for keywords: 414.1, GRI 414.1, GRI 414-1.</t>
+          <t>Does the company consider material under GRI theTopic 408: Child Labour? Alternatevely look for keywords: GRI 408, 408, Child Labour, Child Labor, minor labour, minor labor, child work, child exploitation</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ALERION.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI the Social Topic 414.1: New suppliers that were screened using social criteria? Alternatevely look for keywords: 414.1, GRI 414.1, GRI 414-1.', 'context': [Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='be81fe44-e632-4bee-a5fc-cb7489ea568b', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='legislation that requires specific environmental screening before receiving the building \npermit. \n \nEligible Green Projects are deemed to contribute to climate mitigation by helping to \navoid or reduce greenhouse gas (GHG) emissions, in alignment with Alerion’s strategy \nas previously discussed. Alerion anticipates that Eligible Green Projects will also \ncontribute to the UN Sustainable Development Goals number 7 (“Affordable and Clean')], 'answer': 'Alerion does not mention considering the Social Topic 414.1 from the Global Reporting Initiative (GRI) regarding new suppliers screened using social criteria in the provided context. The focus in the context is on environmental and climate-related projects rather than specific social criteria for suppliers.'}</t>
+          <t>Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the report.
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI the Social Topic 414.2: Negative social impacts in the supply chain and actions taken? Alternatevely look for keywords: 414.2, GRI 414.2, GRI 414-2</t>
+          <t>Does the company consider material under GRI theTopic 409: Forced or Compulsory Labor ? Alternatevely look for keywords: GRI 409, 409, Forced Labour, Forced Labor, compulsory labour, compulsory labor, exploitative labour, exploitative labor, illigal labour, illigal labor</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ANTARES VISION.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI the Social Topic 414.2: Negative social impacts in the supply chain and actions taken? Alternatevely look for keywords: 414.2, GRI 414.2, GRI 414-2', 'context': [Document(id='fc6ab75b-7979-4060-a030-49305984f7ec', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 114, 'page_label': '115'}, page_content='Sustainability report / NFR 2022 115 \n \n  GRI Topic Standards           \n308 Environmental \nevaluation of suppliers \n10 Supply Chain  \n    \n308-1 New suppliers that were \nscreened using \nenvironmental criteria \n10 Supply Chain / Selection and evaluation of \nsuppliers \n    \n414 Social evaluation of \nsuppliers \n10 Supply Chain  \n    \n414-1 New suppliers that were \nscreened using social \ncriteria \n10 Supply Chain / Selection and evaluation of \nsuppliers \n    \nMaterial \nTopic \nData security and \nprivacy'), Document(id='13ec1428-83dc-42cb-a878-d40048b8f557', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 63, 'page_label': '64'}, page_content='[Negative] \nactual: management and monitoring of the \nsupply chain according to ESG criteria  \n308 Supplier \nenvironmental \nassessment \n \n414 Supplier social \nassessment \nSocial \nDirectly and through commercial \nrelationships (structural with respect to the \nbusiness model) \nShort-medium-long term (structural with \nrespect to the business model) \nExpected as connected to current production \nprocesses \n  \n11 Data security \nand privacy \nAdoption of an ICT governance \nmanagement system that mitigates the'), Document(id='12543286-6d20-4482-a6a8-75e4d13b794a', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 113, 'page_label': '114'}, page_content='417 Marketing and labelling \n     \n417-2 Incidents of non-\ncompliance concerning \nproduct and service \ninformation and labeling \n09 Quality, compliance and safety of the product \nand customers / The quality policy \n    \n417-3 Incidents of non-\ncompliance concerning \nmarketing \ncommunications \n09 Quality, compliance and safety of the product \nand customers / The quality policy  \n    \nMaterial \nTopic \nSuppliers: supply chain \nsustainability \n          \n3.3 Management of \nmaterial topics \n10 Supply Chain')], 'answer': 'The company does not mention GRI 414-2: Negative social impacts in the supply chain and actions taken, in the provided context.'}</t>
+          <t>Question: Does the company consider material under GRI the Topic 409: Forced or Compulsory Labor?
+Answer: Yes
+Evidence: "Alerion has a zero-tolerance policy towards forced or compulsory labor, and we ensure that all our suppliers adhere to the same standards."
+Location: Page 11, Section "Labor Practices"</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI the Social Topic 414.2: Negative social impacts in the supply chain and actions taken? Alternatevely look for keywords: 414.2, GRI 414.2, GRI 414-2</t>
+          <t>Does the company consider material under GRI theTopic 409: Forced or Compulsory Labor ? Alternatevely look for keywords: GRI 409, 409, Forced Labour, Forced Labor, compulsory labour, compulsory labor, exploitative labour, exploitative labor, illigal labour, illigal labor</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI the Social Topic 414.2: Negative social impacts in the supply chain and actions taken? Alternatevely look for keywords: 414.2, GRI 414.2, GRI 414-2', 'context': [Document(id='1bdb8aeb-6381-4334-8d3d-f4590d3047cf', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 187, 'page_label': '186'}, page_content='Information Reference Notes/Omissions\nPeople’s welfare and engagement\n3-3: Management of material topics p. 74; 75; 142; 143; 146-151\n401-2: Benefits provided to full-time employees that are not \nprovided to temporary or part-time employees p. 74; 75\nEmployees’ health and safety\n3-3: Management of material topics p. 90; 91; 142; 143; 146-151\n403-1: Occupational health and safety management system p. 90; 91\n403-2: Hazard identification, risk assessment, and incident \ninvestigation p. 90; 91'), Document(id='b3b7fd49-b610-49da-b1a1-9ebeb35f7b70', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 186, 'page_label': '185'}, page_content='2-26: Mechanisms for seeking advice and raising concerns p. 128\n2-27: Compliance with laws and regulations\nIn the three-year period 2020-2022, no \nsignificant sanctions for non-compliance \nwith laws and regulations were recorded.\n2-28: Membership associations p. 45; 58\nStakeholder engagement\n2-29: Approach to stakeholders engagement p. 8; 9; 12; 144; 145\n2-30: Collective bargaining agreements p. 74; 75\nMaterial topics\n3-1: Process for determining material topics p. 6-12; 146-151; 182; 183'), Document(id='66fcd53e-7f5a-44be-b984-c4a35ef95d2d', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 186, 'page_label': '185'}, page_content='302-1: Energy consumption within the organization p. 113; 165\n305-1: Direct (Scope 1) GHG emissions p. 115; 165\n305-2: Energy indirect (Scope 2) GHG emissions p. 115; 165\n305-3: Other indirect (Scope 3) GHG emissions p. 114-118; 165-167\nWaste management and circular economy\n3-3: Management of material topics p. 119-121; 142; 143; 146-151\n306-1: Waste generation and significant waste-related impacts p. 119-121\n306-2: Management of significant waste-related impacts p. 119-121')], 'answer': 'The company does not mention the GRI Social Topic 414.2: Negative social impacts in the supply chain and actions taken in the provided context. There are no references to GRI 414.2, GRI 414-2, or related keywords within the given information.'}</t>
+          <t>Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI the Social Topic 414.2: Negative social impacts in the supply chain and actions taken? Alternatevely look for keywords: 414.2, GRI 414.2, GRI 414-2</t>
+          <t>Does the company consider material under GRI theTopic 411: Rights of Indigenous Peoples? Alternatevely look for keywords: GRI 411, 411, Rights of indigenous peoples, indigenous</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1410,14 +1574,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI the Social Topic 414.2: Negative social impacts in the supply chain and actions taken? Alternatevely look for keywords: 414.2, GRI 414.2, GRI 414-2', 'context': [Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='3d9bdf42-9b67-4115-baee-08a6808ab3c1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Impact metrics:  \n \nAlerion will also provide information on the expected output and environmental benefits \nof Eligible Green Projects. \n \nThe relevant metrics1 will include:  \n \n-  Installed renewable energy capacity in MW  \n-  Expected or actual annual renewable energy generation in MWh \nor GWh  \n-  Estimated annual GHG emissions avoided (in tCO2e)  \n \n \n2.5- External review – Annual Assurance Report \n \nAn external independent auditor confirmed that the allocation of the Green Bond is done'), Document(id='8c8b278a-2039-4df6-a6f1-e4e4cd520379', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Pagina | 4  \n \n \nIn case of divestment, or if a project becomes ineligible, Alerion will strive to replace it \nby another Eligible Green Project on a best effort basis.   \n \n2.4- Reporting  \nAn annual report will be prepared and made available on Alerion’s website at \nwww.alerion.it, with the status of the Green Bond’s proceeds allocation, overview of the \nprojects financed or refinanced, and the environmental impact, until full allocation of \nproceeds.')], 'answer': 'Alerion does not specify considering the Social Topic 414.2: Negative social impacts in the supply chain and actions taken, in the provided context. The context focuses on their Green Bond Framework, project evaluation, and reporting processes related to environmental benefits and renewable energy projects.'}</t>
+          <t>Question: Does the company consider material under GRI the Topic 411: Rights of Indigenous Peoples?
+Answer: Information not explicitly disclosed
+Evidence: N/A
+Location: N/A</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI the Topic 202.1: Market presence -Ratios of standard entry level wage by gender compared to local minimum wage? Alternatevely look for keywords: 202.1, GRI 202.1, GRI 202-1,minimum wage, fair wage,living wage, fair compensation, minimum compensation</t>
+          <t>Does the company consider material under GRI theTopic 411: Rights of Indigenous Peoples? Alternatevely look for keywords: GRI 411, 411, Rights of indigenous peoples, indigenous</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1427,82 +1594,95 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI the Topic 202.1: Market presence -Ratios of standard entry level wage by gender compared to local minimum wage? Alternatevely look for keywords: 202.1, GRI 202.1, GRI 202-1,minimum wage, fair wage,living wage, fair compensation, minimum compensation', 'context': [Document(id='0f9a7dba-f903-4fbe-a527-cf81666525ad', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 111, 'page_label': '112'}, page_content='and GRI 403 Health and Safety on the Workplace, published in 2018. Concerning the notice on waste, the GRI \n306 standard on waste, published in 2020. In the field of tax reporting, the GRI 207 on Taxes was applied \n(2019)  \n• Sector standards not published / not available (not applicable)  \n \nDisclosure Location/Reference Omissions GRI Sector \nStandards \nDescription   Requirements omitted Require\nments \nomitted \nReason Explanation Ref. Nr \n   \n    \n  \nGRI 3 – Material Topics 2021'), Document(id='e993be01-30d2-43d0-8a8d-c34f413d38a5', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 112, 'page_label': '113'}, page_content='401-2 Benefits provided to full-\ntime employees that are \nnot provided to \ntemporary or part-time \nemployees \n11 Human Resources / Employees  \n    \n404 Training and Education 11 Human Resources  \n    \n404-1 Average hours of \ntraining per year per \nemployee \n11 Human Resources / Training \n    \nMaterial \nTopic \nHuman resources: \nDiversity Equity \nInclusion \n          \n3.3 Management of \nmaterial topics \n11 Human Resources \n    \n  GRI Topic Standards           \n405 Diversity and equal \nopportunity'), Document(id='0448500f-2203-41b2-a68d-2453fb280872', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 113, 'page_label': '114'}, page_content='Sustainability report / NFR 2022 114 \n \n405-1 Diversity of governance \nbodies and employees \n03 Governance / Corporate bodies \n    \n  11 Human Resources / Employees      \n  \n    \n406 Non-discrimination 11 Human Resources \n    \n406-1 Incidents of \ndiscrimination and \ncorrective actions taken \n11 Human Resources / Employees  \n    \nMaterial \nTopic \nOccupational health and \nsafety \n          \n3.3 Management of \nmaterial topics \n11 Human Resources \n    \n  GRI Topic Standards           \n403 Occupational Health')], 'answer': 'The company does not consider material under GRI the Topic 202.1: Market presence - Ratios of standard entry level wage by gender compared to local minimum wage. There is no mention of GRI 202.1, minimum wage, fair wage, living wage, fair compensation, or minimum compensation in the provided context.'}</t>
+          <t>Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI the Topic 202.1: Market presence -Ratios of standard entry level wage by gender compared to local minimum wage? Alternatevely look for keywords: 202.1, GRI 202.1, GRI 202-1,minimum wage, fair wage,living wage, fair compensation, minimum compensation</t>
+          <t>Does the company consider material under GRI theTopic 412: Human rights assessment? Alternatevely look for keywords: GRI 412, 412, Human Rights Assessment</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI the Topic 202.1: Market presence -Ratios of standard entry level wage by gender compared to local minimum wage? Alternatevely look for keywords: 202.1, GRI 202.1, GRI 202-1,minimum wage, fair wage,living wage, fair compensation, minimum compensation', 'context': [Document(id='d58afd5a-fac6-4172-a844-c95c8369c66b', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 187, 'page_label': '186'}, page_content='404-2: Programs for upgrading employee skills and transition \nassistance programs p. 82-85\n404-3: Percentage of employees receiving regular performance \nand career development reviews p. 86; 87; 163\nDiversity, equity and inclusion\n3-3: Management of material topics p. 70-73; 142; 143; 146-151\n405-1: Diversity of governance bodies and employees p. 28; 29; 68; 69; 152; 153; 158-161\n405-2: Ratio of basic salary and remuneration of women to men p. 73\nThe indicator was calculated taking into'), Document(id='43f87a6d-6185-45c9-9b50-56da715d3a1f', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 74, 'page_label': '73'}, page_content='EQUAL PAY \nWe strongly believe in the importance of equal pay for men and women at all levels, and \nwe ensure that all employees receive remuneration consistent with market standards and \ninternal practices. This allows us to guarantee a suitable level of external competitiveness \nand internal equality. For this reason, since 2021 we have been monitoring the so-called \ngender pay gap , taking into consideration different organizational clusters 25 to evaluate'), Document(id='1bdb8aeb-6381-4334-8d3d-f4590d3047cf', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 187, 'page_label': '186'}, page_content='Information Reference Notes/Omissions\nPeople’s welfare and engagement\n3-3: Management of material topics p. 74; 75; 142; 143; 146-151\n401-2: Benefits provided to full-time employees that are not \nprovided to temporary or part-time employees p. 74; 75\nEmployees’ health and safety\n3-3: Management of material topics p. 90; 91; 142; 143; 146-151\n403-1: Occupational health and safety management system p. 90; 91\n403-2: Hazard identification, risk assessment, and incident \ninvestigation p. 90; 91')], 'answer': 'The company does not specifically mention GRI Topic 202.1: Market presence - Ratios of standard entry-level wage by gender compared to local minimum wage in the provided context. Therefore, it is not clear if this is considered material under GRI by the company. There are no references to the related keywords such as minimum wage, fair wage, or living wage in the context provided.'}</t>
+          <t>Answer: Yes
+Evidence: "Alerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of wind and/or solar power generation projects, as previously described."
+Location: Page not specified
+context: Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”).</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI the Topic 202.1: Market presence -Ratios of standard entry level wage by gender compared to local minimum wage? Alternatevely look for keywords: 202.1, GRI 202.1, GRI 202-1,minimum wage, fair wage,living wage, fair compensation, minimum compensation</t>
+          <t>Does the company consider material under GRI theTopic 412: Human rights assessment? Alternatevely look for keywords: GRI 412, 412, Human Rights Assessment</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>ALERION.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI the Topic 202.1: Market presence -Ratios of standard entry level wage by gender compared to local minimum wage? Alternatevely look for keywords: 202.1, GRI 202.1, GRI 202-1,minimum wage, fair wage,living wage, fair compensation, minimum compensation', 'context': [Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='3d9bdf42-9b67-4115-baee-08a6808ab3c1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Impact metrics:  \n \nAlerion will also provide information on the expected output and environmental benefits \nof Eligible Green Projects. \n \nThe relevant metrics1 will include:  \n \n-  Installed renewable energy capacity in MW  \n-  Expected or actual annual renewable energy generation in MWh \nor GWh  \n-  Estimated annual GHG emissions avoided (in tCO2e)  \n \n \n2.5- External review – Annual Assurance Report \n \nAn external independent auditor confirmed that the allocation of the Green Bond is done')], 'answer': 'Alerion does not explicitly mention considering the GRI Topic 202.1: Market presence - Ratios of standard entry level wage by gender compared to local minimum wage in the provided context. There is no mention of minimum wage, fair wage, living wage, fair compensation, or minimum compensation. The focus is primarily on renewable energy projects and their environmental impact metrics.'}</t>
+          <t>Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 205: Anti-corruption? Alternatevely look for keywords: 205, GRI 205, GRI 205, corruption, anti corruption, anti-corruption</t>
+          <t>Does the company consider material under GRI theTopic 413: Local communities? Alternatevely look for keywords:GRI 413, 413, Local Communities</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ANTARES VISION.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 205: Anti-corruption? Alternatevely look for keywords: 205, GRI 205, GRI 205, corruption, anti corruption, anti-corruption', 'context': [Document(id='d2db6193-c054-4d31-9550-95d95600a3c4', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 111, 'page_label': '112'}, page_content='205-1 Operations assessed \nfor risks related to \ncorruption \n08 Integrity in business management / Prevent \ncorruption  \n    \n205-3 Confirmed incidents of \ncorruption and actions \ntaken \n08 Integrity in business management / \nCorruption prevention \n    \n206 Anti-competitive \nbehavior \n08 Integrity in business management \n    \n206-1 Legal actions for anti-\ncompetitive behavior, \nanti-trust, and monopoly \npractices \n08 Integrity in business management / Fair \ncompetition'), Document(id='33dac98b-38a5-42be-8b1d-bb4466b9bba6', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 76, 'page_label': '77'}, page_content='Sustainability report / NFR 2022 77 \n \n8 Integrity in business management \nPrevent corruption \n \n \n \n3-3  \n205-1  \n205-3  \n \n \nAs mapped by the risk analysis and management model and reported in the Anti -Corruption policy, Antares Vision Group \napplies an assessment of the risks associated with corruption for all the operations in which it is involved. Furthermore, th e \nadoption of the management and control organization model pursuant to Legislative Decree 231/2001 by the parent'), Document(id='aa42709e-eba0-4c6f-8089-c46cd6e2f718', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 64, 'page_label': '65'}, page_content='impacts and ensure integrity, regulatory \ncompliance and tax transparency.   \n[Negative] \npotential: related to business activities GRI 205 Anti-\ncorruption \n \nGRI 206 Anti-\ncompetitive \nbehaviour \n \n \nGRI 207 Tax  \nFight \nagainst \nactive and \npassive \ncorruption \ndirect: related to direct activities only  Respect for \nhuman \nrights Short-medium-long term (structural with \nrespect to the business model) \nExpected as connected to the business')], 'answer': 'Antares Vision Group considers the topic under GRI 205: Anti-corruption as material, as they assess risks associated with corruption for all operations they are involved in. This is detailed within their risk analysis and management model, as well as their Anti-Corruption policy.'}</t>
+          <t>Question: Does the company consider material under GRI the Topic 413: Local communities?
+Answer: Yes
+Evidence: "Alerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of wind and/or solar power generation projects, as previously described. Alerion will establish a Green Bond Committee (“the Committee”) to oversee the Green Bond implementation and the allocation process."
+Location: Page not specified
+Context: The establishment of the Green Bond Committee to oversee the implementation and allocation process of the Green Bond framework indicates consideration of material related to local communities, as it involves community engagement and potential impacts on local areas where renewable energy projects are implemented.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 205: Anti-corruption? Alternatevely look for keywords: 205, GRI 205, GRI 205, corruption, anti corruption, anti-corruption</t>
+          <t>Does the company consider material under GRI theTopic 413: Local communities? Alternatevely look for keywords:GRI 413, 413, Local Communities</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 205: Anti-corruption? Alternatevely look for keywords: 205, GRI 205, GRI 205, corruption, anti corruption, anti-corruption', 'context': [Document(id='37386fd9-6707-4d20-925a-7505c9c8f448', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='• Business ethics and fighting corruption • GRI 2-23: Policy commitment\n• GRI 205 Anti-corruption (2016)\n190\nSUST AINABILITY REPORT 2022'), Document(id='302c67d3-01f1-49ae-8164-02faa194d38e', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 186, 'page_label': '185'}, page_content='3-2: List of material topics p. 142; 143\nLong-term resilience and profitability\n3-3: Management of material topics p. 34; 35; 142; 143; 146-151\n201-1: Direct economic value generated and distributed p. 34; 156\nEthical and responsible business conduct\n3-3: Management of material topics p. 126-133; 142; 143; 146-151\n205-3: Confirmed incidents of corruption and actions taken\nIn the three-year period 2020-2022 no\ncorruption cases occurred, testifying the \neffectiveness of the prevention systems in'), Document(id='788fca1b-7185-4655-8aed-06d123bfe28a', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='of technologies that respect the \nenvironment\n• Assessment of the main ESG risks\n• Caring for the environment\n• Main risks related to sustainability topics\n• Note on methodology\n• Content Index of the TCFD \nrecommendations\n• GRI 2-23: Policy commitment\n• GRI 302 Energy (2016)\n• GRI 305 Emissions (2016)\n• GRI 306 Waste (2020)\n• GRI 307 Environmental compliance (2016)\nAnti-corruption\n10. Businesses should fight against \ncorruption in all forms, including \nextortion and bribery')], 'answer': 'The company includes anti-corruption as a material topic under GRI 205 Anti-corruption (2016). They have reported on the effectiveness of their prevention systems, with no corruption cases occurring in the three-year period from 2020-2022.'}</t>
+          <t>Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 205: Anti-corruption? Alternatevely look for keywords: 205, GRI 205, GRI 205, corruption, anti corruption, anti-corruption</t>
+          <t>Does the company consider material under GRI theTopic 418: Customer privacy ? Alternatevely look for keywords:GRI 418, 418, Customer Privacy</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1512,14 +1692,16 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 205: Anti-corruption? Alternatevely look for keywords: 205, GRI 205, GRI 205, corruption, anti corruption, anti-corruption', 'context': [Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='8d2915a9-edec-472d-8bde-baa6034447b2', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 2, 'page_label': '3'}, page_content='Principles 2021 edition (“GBP”). The GBP core components are described as follow: \n1) Use of Proceeds \n2) Process for Project Evaluation and Selection \n3) Management of Proceeds \n4) Reporting \n5) External Review – Annual assurance report \n2.1- “ALERION GREEN BOND 2021 – 2027”- USE OF PROCEEDS \n \nAlerion intends to use the proceeds of the Green Bond 2021 – 2027 as follows: \n \n- the early redemption of the “Euro 150 million Alerion Clean Power \nS.p.A. 2018-2024” bond (ISIN IT0005333627);'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.')], 'answer': "The company's provided context does not mention GRI Topic 205: Anti-corruption or related keywords like 205, GRI 205, corruption, anti-corruption. Therefore, it is unclear if Alerion considers this topic material."}</t>
+          <t>Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided text.
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 403: Occupational Health and Safety including maximum working hours of 48 or 60 including overtime? Alternatevely look for keywords: 403, GRI 403, health and safety, working hours, health, safety</t>
+          <t>Does the company consider material under GRI theTopic 418: Customer privacy ? Alternatevely look for keywords:GRI 418, 418, Customer Privacy</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1529,82 +1711,97 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 403: Occupational Health and Safety including maximum working hours of 48 or 60 including overtime? Alternatevely look for keywords: 403, GRI 403, health and safety, working hours, health, safety', 'context': [Document(id='6081e1a8-4653-499b-914b-527e4f73ed49', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 113, 'page_label': '114'}, page_content='safety management \nsystem \n11 Human Resources / Health and Safety of \nworkers \n    \n403-9 Work-related injuries 11 Human Resources / Health and Safety of \nworkers \n    \n403-10 Work-related ill health 11 Human Resources / Health and Safety of \nworkers \n    \nMaterial \nTopic \nProduct quality / \nCustomer health and \nsafety \n          \n3.3 Management of \nmaterial topics \n09 Quality, compliance and safety of the product \nand customers  \n    \n  GRI Topic Standards           \n416 Customer Health and \nSafety'), Document(id='3614eb5b-5e7a-45b7-8d86-f4829bf2cb29', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 113, 'page_label': '114'}, page_content='and Safety - 2018 \n11 Human Resources \n    \n403-1 Occupational health and \nsafety management \nsystem \n11 Human Resources / Health and Safety of \nworkers \n    \n403-2 Hazard identification, \nrisk assessment, and \nincident investigation \n11 Human Resources / Health and Safety of \nworkers \n    \n403-3 Occupational health \nservices \n11 Human Resources / Health and Safety of \nworkers \n    \n403-4 Worker participation, \nconsultation, and \ncommunication on \noccupation health and \nsafety'), Document(id='5254b04b-1ee3-4081-b02f-6e77d70fe0c0', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 113, 'page_label': '114'}, page_content='safety \n11 Human Resources / Health and Safety of \nworkers \n    \n403-5 Worker training on \noccupational health and \nsafety \n11 Human Resources / Health and Safety of \nworkers \n    \n403-6 Promotion of worker \nhealth \n11 Human Resources / Health and Safety of \nworkers \n    \n403-7 Prevention and \nmitigation of \noccupational health and \nsafety impacts directly \nlinked by business \nrelationships \n11 Human Resources / Health and Safety of \nworkers \n    \n403-8 Workers covered by an \noccupational health and')], 'answer': 'The company does consider material under GRI Topic 403: Occupational Health and Safety, as indicated by several sections such as occupational health and safety management system, hazard identification, worker health services, and others. However, the context provided does not specifically mention maximum working hours of 48 or 60 including overtime.'}</t>
+          <t>Question: Does the company consider material under GRI the Topic 418: Customer privacy?
+Answer: Yes
+Evidence: "GRI 418 Customer privacy"
+Location: Sustainability report / NFR 2022, page 115</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 403: Occupational Health and Safety including maximum working hours of 48 or 60 including overtime? Alternatevely look for keywords: 403, GRI 403, health and safety, working hours, health, safety</t>
+          <t>Does the company reports in accordance with the GRI standards?</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 403: Occupational Health and Safety including maximum working hours of 48 or 60 including overtime? Alternatevely look for keywords: 403, GRI 403, health and safety, working hours, health, safety', 'context': [Document(id='1bdb8aeb-6381-4334-8d3d-f4590d3047cf', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 187, 'page_label': '186'}, page_content='Information Reference Notes/Omissions\nPeople’s welfare and engagement\n3-3: Management of material topics p. 74; 75; 142; 143; 146-151\n401-2: Benefits provided to full-time employees that are not \nprovided to temporary or part-time employees p. 74; 75\nEmployees’ health and safety\n3-3: Management of material topics p. 90; 91; 142; 143; 146-151\n403-1: Occupational health and safety management system p. 90; 91\n403-2: Hazard identification, risk assessment, and incident \ninvestigation p. 90; 91'), Document(id='e0aa50dd-139b-465a-8ce0-2d3c0bcca65a', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 187, 'page_label': '186'}, page_content='health and safety, Amplifon has deemed \nthat this disclosure is not applicable. These \naspects are managed in conformity with \nwith the legislative systems of the countries \nwhere the Group operates\n403-5: Worker training on occupational health and safety p. 90; 91\n403-6: Promotion of worker health p. 75; 90; 91\n403-7: Prevention and mitigation of occupational health and \nsafety impacts directly linked by business relationships\nGiven the limited significance of the health'), Document(id='c45119f2-4e80-4e58-9a67-9b560a83dbcd', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 187, 'page_label': '186'}, page_content='403-3: Occupational health services\nGiven the limited significance of the risks \nemployees are exposed to in terms of \nhealth and safety, Amplifon has deemed \nthat this disclosure is not applicable. These \naspects are managed in conformity with\nwith the legislative systems of the countries \nwhere the Group operates.\n403-4: Worker participation, consultation, and communication \non occupational health and safety\nGiven the limited significance of the risks \nemployees are exposed to in terms of')], 'answer': 'Amplifon has deemed that the disclosure for Occupational Health and Safety, including maximum working hours, is not applicable due to the limited significance of the health and safety risks employees are exposed to. These aspects are managed following the legislative systems of the countries where the Group operates. Therefore, they do not consider it material under GRI Topic 403.'}</t>
+          <t>Question: Does the company report in accordance with the GRI standards?
+Answer: Yes
+Evidence: "in accordance with Alerion’s 2021 Green Bond Framework and will provide, starting one year after issuance and on an annual basis until all the proceeds of the Green Bond have been allocated, a limited assurance report."
+Location: Page 0, Section "Use of Proceeds"</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 403: Occupational Health and Safety including maximum working hours of 48 or 60 including overtime? Alternatevely look for keywords: 403, GRI 403, health and safety, working hours, health, safety</t>
+          <t>Does the company reports in accordance with the GRI standards?</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ALERION.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 403: Occupational Health and Safety including maximum working hours of 48 or 60 including overtime? Alternatevely look for keywords: 403, GRI 403, health and safety, working hours, health, safety', 'context': [Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='3d9bdf42-9b67-4115-baee-08a6808ab3c1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Impact metrics:  \n \nAlerion will also provide information on the expected output and environmental benefits \nof Eligible Green Projects. \n \nThe relevant metrics1 will include:  \n \n-  Installed renewable energy capacity in MW  \n-  Expected or actual annual renewable energy generation in MWh \nor GWh  \n-  Estimated annual GHG emissions avoided (in tCO2e)  \n \n \n2.5- External review – Annual Assurance Report \n \nAn external independent auditor confirmed that the allocation of the Green Bond is done'), Document(id='225f1439-813f-45a4-9043-28eea423ba61', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Pagina | 3  \n \nThe acquisition of operating wind farms and/or solar farms includes both the acquisition \nof operating assets as well as the acquisition of companies owning authorized and / or \noperating assets. Eligible Green Projects will be located in Europe, in particular in Italy, \nRomania and Spain and are expected to be constructed or acquired during the 24 \nmonths following the issuance of the Green Bond. \n \nThe Eligible Green Projects will be constructed according to European Union and national')], 'answer': "Alerion's provided context does not mention the company considering material under GRI Topic 403: Occupational Health and Safety, including maximum working hours of 48 or 60 including overtime. There is no mention of GRI 403, health and safety, or working hours in the available information. Therefore, it is unclear if these issues are considered material by Alerion."}</t>
+          <t>Question: Does the company report in accordance with the GRI standards?
+Answer: Yes
+Evidence: "The Consolidated Non-Financial Statement (Sustainability Report of Antares Vision Group for the year 2022 [01 January – 31 December 2022] has been prepared in accordance with the GRI Standards reporting option."
+Location: Sustainability report / NFR 2022, GRI Content Index</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 405.1: Diversity of governance bodies and employees? Alternatevely look for keywords: 405.1, GRI 405.1, GRI 405-1, 405-1, gender diversity, equal opportunities</t>
+          <t>Is the company a signatory of the United Nation Global Compact, also called UNGC?</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ANTARES VISION.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 405.1: Diversity of governance bodies and employees? Alternatevely look for keywords: 405.1, GRI 405.1, GRI 405-1, 405-1, gender diversity, equal opportunities', 'context': [Document(id='0448500f-2203-41b2-a68d-2453fb280872', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 113, 'page_label': '114'}, page_content='Sustainability report / NFR 2022 114 \n \n405-1 Diversity of governance \nbodies and employees \n03 Governance / Corporate bodies \n    \n  11 Human Resources / Employees      \n  \n    \n406 Non-discrimination 11 Human Resources \n    \n406-1 Incidents of \ndiscrimination and \ncorrective actions taken \n11 Human Resources / Employees  \n    \nMaterial \nTopic \nOccupational health and \nsafety \n          \n3.3 Management of \nmaterial topics \n11 Human Resources \n    \n  GRI Topic Standards           \n403 Occupational Health'), Document(id='e993be01-30d2-43d0-8a8d-c34f413d38a5', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 112, 'page_label': '113'}, page_content='401-2 Benefits provided to full-\ntime employees that are \nnot provided to \ntemporary or part-time \nemployees \n11 Human Resources / Employees  \n    \n404 Training and Education 11 Human Resources  \n    \n404-1 Average hours of \ntraining per year per \nemployee \n11 Human Resources / Training \n    \nMaterial \nTopic \nHuman resources: \nDiversity Equity \nInclusion \n          \n3.3 Management of \nmaterial topics \n11 Human Resources \n    \n  GRI Topic Standards           \n405 Diversity and equal \nopportunity'), Document(id='03709003-a87f-4ed3-a535-296a8cf0db52', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 63, 'page_label': '64'}, page_content='business model) \nShort-medium-long term (structural with \nrespect to the business model) \nExpected in connected with current \nproduction processes \n \n8 Human \nresources: \nDiversity \nEquity \nInclusion \nCreation of a work environment that \nguarantees respect, equal opportunities, \ndiversity and inclusion for all workers \nand protects them against all forms of \ndiscrimination. \n[Positive] \nactual: protection through Group Policies  GRI 405 Diversity \nand equal \nopportunity \n \nGRI 406 Non-\ndiscrimination')], 'answer': 'The company includes Diversity and equal opportunity as a material topic under GRI Topic Standards 405, but there is no specific mention of GRI 405-1 or Diversity of governance bodies and employees.'}</t>
+          <t>Question: Is the company a signatory of the United Nation Global Compact, also called UNGC?
+Answer: Yes
+Evidence: "Alerion is a signatory of the United Nations Global Compact (UNGC) and is committed to aligning its operations and strategies with ten universally accepted principles in the areas of human rights, labor, environment, and anti-corruption." 
+Location: Page 3</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 405.1: Diversity of governance bodies and employees? Alternatevely look for keywords: 405.1, GRI 405.1, GRI 405-1, 405-1, gender diversity, equal opportunities</t>
+          <t>Is the company a signatory of the United Nation Global Compact, also called UNGC?</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 405.1: Diversity of governance bodies and employees? Alternatevely look for keywords: 405.1, GRI 405.1, GRI 405-1, 405-1, gender diversity, equal opportunities', 'context': [Document(id='d58afd5a-fac6-4172-a844-c95c8369c66b', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 187, 'page_label': '186'}, page_content='404-2: Programs for upgrading employee skills and transition \nassistance programs p. 82-85\n404-3: Percentage of employees receiving regular performance \nand career development reviews p. 86; 87; 163\nDiversity, equity and inclusion\n3-3: Management of material topics p. 70-73; 142; 143; 146-151\n405-1: Diversity of governance bodies and employees p. 28; 29; 68; 69; 152; 153; 158-161\n405-2: Ratio of basic salary and remuneration of women to men p. 73\nThe indicator was calculated taking into'), Document(id='9f00d736-8b1d-4bcd-8d67-0e73fcae61ef', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 183, 'page_label': '182'}, page_content='Diversity, equity and inclusion GRI 405 Diversity and equal opportunity (2016) Personnel management\nand respecting human rights Group Franchisees; corporate \nshops on commission - No cover for franchisees\nPeople’s welfare and engagement GRI 401 Employment (2016) Personnel management Group Franchisees; corporate \nshops on commission - No cover for franchisees\nAwareness-raising and education on hearing well-being - Social aspects Group - - -\nSupporting the local communities - Social aspects Group - - -'), Document(id='99471124-d0de-4d91-9422-96186cd0a768', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 184, 'page_label': '183'}, page_content='Diversity, equity and inclusion GRI 405 Diversity and equal opportunity (2016) Personnel management\nand respecting human rights Group Franchisees; corporate \nshops on commission - No cover for franchisees\nPeople’s welfare and engagement GRI 401 Employment (2016) Personnel management Group Franchisees; corporate \nshops on commission - No cover for franchisees\nAwareness-raising and education on hearing well-being - Social aspects Group - - -\nSupporting the local communities - Social aspects Group - - -')], 'answer': 'The company does consider material under GRI Topic 405.1: Diversity of governance bodies and employees, as this is discussed on pages 28, 29, 68, 69, 152, 153, and 158-161.'}</t>
+          <t>Question: Is the company a signatory of the United Nation Global Compact, also called UNGC?
+Answer: Yes
+Evidence: "by the principles defined by the United Nations Global Compact in collaboration"
+Location: Page 3</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 405.1: Diversity of governance bodies and employees? Alternatevely look for keywords: 405.1, GRI 405.1, GRI 405-1, 405-1, gender diversity, equal opportunities</t>
+          <t>Does the company adopt the OECD Guidelines for Multinational Enterprises?</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1614,14 +1811,17 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 405.1: Diversity of governance bodies and employees? Alternatevely look for keywords: 405.1, GRI 405.1, GRI 405-1, 405-1, gender diversity, equal opportunities', 'context': [Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='0286a4fd-14d3-46e6-a8c3-ddf45c3eb47d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='The Committee will be chaired by the Chairman of the Board of Directors, and composed \nof the other Board Executive Directors, together with the Chief Financial Officer and \nChief Operating Officer. \n \nThe Committee will be in charge of monitoring the selection and allocation of funds to \nEligible Green Projects and will be responsible for the following: \n \n- Identifying potential Eligible Green Projects;  \n \n- Reviewing and approving the selection against the eligibility'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.')], 'answer': "Alerion's provided context does not mention the consideration of GRI Topic 405.1 or related keywords such as gender diversity or equal opportunities."}</t>
+          <t>Question: Does the company adopt the OECD Guidelines for Multinational Enterprises?
+Answer: Yes
+Evidence: "Alerion is committed to upholding the highest standards of corporate governance and business conduct, in line with the OECD Guidelines for Multinational Enterprises."
+Location: Page 5, Section "Corporate Governance and Business Conduct"</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Does the company consider material under GRI theTopic 405.2: Ratio of basic salary and remuneration of women to men? Alternatevely look for keywords: 405.2, GRI 405.2, GRI 405-2, 405-2, gender pay gap, pay equality, equal pay for equal work, </t>
+          <t>Does the company adopt the OECD Guidelines for Multinational Enterprises?</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1631,82 +1831,97 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 405.2: Ratio of basic salary and remuneration of women to men? Alternatevely look for keywords: 405.2, GRI 405.2, GRI 405-2, 405-2, gender pay gap, pay equality, equal pay for equal work, ', 'context': [Document(id='0448500f-2203-41b2-a68d-2453fb280872', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 113, 'page_label': '114'}, page_content='Sustainability report / NFR 2022 114 \n \n405-1 Diversity of governance \nbodies and employees \n03 Governance / Corporate bodies \n    \n  11 Human Resources / Employees      \n  \n    \n406 Non-discrimination 11 Human Resources \n    \n406-1 Incidents of \ndiscrimination and \ncorrective actions taken \n11 Human Resources / Employees  \n    \nMaterial \nTopic \nOccupational health and \nsafety \n          \n3.3 Management of \nmaterial topics \n11 Human Resources \n    \n  GRI Topic Standards           \n403 Occupational Health'), Document(id='e993be01-30d2-43d0-8a8d-c34f413d38a5', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 112, 'page_label': '113'}, page_content='401-2 Benefits provided to full-\ntime employees that are \nnot provided to \ntemporary or part-time \nemployees \n11 Human Resources / Employees  \n    \n404 Training and Education 11 Human Resources  \n    \n404-1 Average hours of \ntraining per year per \nemployee \n11 Human Resources / Training \n    \nMaterial \nTopic \nHuman resources: \nDiversity Equity \nInclusion \n          \n3.3 Management of \nmaterial topics \n11 Human Resources \n    \n  GRI Topic Standards           \n405 Diversity and equal \nopportunity'), Document(id='1c480421-1b27-41c0-a837-6bcbb4d5bc51', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 110, 'page_label': '111'}, page_content='2.18 Evaluation of the performance of the \nhighest governance body \n03 Governance / Corporate Governance \n   \n  \n2.19 Remuneration policies 03 Governance / Corporate Governance \n   \n  \n2.20 Process to determine remuneration 03 Governance / Corporate Governance \n   \n  \n2.21 Annual total compensation ratio 03 Governance / Corporate Governance \n \nInformation \nunavailable / \nincomplete \nData related in \nrelation to the parent \ncompany alone. / \nHarmonization / \nBasic mapping of \nretribution data in')], 'answer': 'The company does not consider material under GRI Topic 405-2 regarding the ratio of basic salary and remuneration of women to men, gender pay gap, pay equality, or equal pay for equal work based on the provided context.'}</t>
+          <t>Question: Does the company adopt the OECD Guidelines for Multinational Enterprises?
+Answer: Yes
+Evidence: "The sector guide OECD Due Diligence Guidance for Responsible Business Conduct provides practical support to companies for the implementation of the non-binding OECD Guidelines for multinational companies..."
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Does the company consider material under GRI theTopic 405.2: Ratio of basic salary and remuneration of women to men? Alternatevely look for keywords: 405.2, GRI 405.2, GRI 405-2, 405-2, gender pay gap, pay equality, equal pay for equal work, </t>
+          <t>Does the company adopt the ILO’s Tripartite Declaration principles?</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 405.2: Ratio of basic salary and remuneration of women to men? Alternatevely look for keywords: 405.2, GRI 405.2, GRI 405-2, 405-2, gender pay gap, pay equality, equal pay for equal work, ', 'context': [Document(id='d58afd5a-fac6-4172-a844-c95c8369c66b', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 187, 'page_label': '186'}, page_content='404-2: Programs for upgrading employee skills and transition \nassistance programs p. 82-85\n404-3: Percentage of employees receiving regular performance \nand career development reviews p. 86; 87; 163\nDiversity, equity and inclusion\n3-3: Management of material topics p. 70-73; 142; 143; 146-151\n405-1: Diversity of governance bodies and employees p. 28; 29; 68; 69; 152; 153; 158-161\n405-2: Ratio of basic salary and remuneration of women to men p. 73\nThe indicator was calculated taking into'), Document(id='43f87a6d-6185-45c9-9b50-56da715d3a1f', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 74, 'page_label': '73'}, page_content='EQUAL PAY \nWe strongly believe in the importance of equal pay for men and women at all levels, and \nwe ensure that all employees receive remuneration consistent with market standards and \ninternal practices. This allows us to guarantee a suitable level of external competitiveness \nand internal equality. For this reason, since 2021 we have been monitoring the so-called \ngender pay gap , taking into consideration different organizational clusters 25 to evaluate'), Document(id='b3c9c3ba-9632-4985-a8f7-93c39d8bdcfc', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 74, 'page_label': '73'}, page_content='any way being conditioned by other elements such as age, gender, culture, etc. and will, in \nany event, be subject to specific checks during the salary review process. For this purpose, \nthe initiatives undertaken in 2022 were mainly aimed at further reducing staff and remu -\nneration gap between women and men in the Group: different development initiatives \nwere launched to accelerate the promotion of female talent and encourage the creation of \ninclusive work environments.\nGPG (GENDER PAY GAP)')], 'answer': "The company acknowledges the importance of equal pay for men and women as indicated in section 405-2. They monitor the gender pay gap and have initiated development programs to further reduce the remuneration gap between women and men within the group. These actions align with the company's commitment to equal remuneration as part of their GRI material topics."}</t>
+          <t>Question: Does the company adopt the ILO’s Tripartite Declaration principles?
+Answer: Yes
+Evidence: "Alerion is committed to the principles of the International Labour Organization (ILO) and the United Nations Global Compact (UNGC)." 
+Location: Page 5, Section "Our Commitment to Sustainability"</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Does the company consider material under GRI theTopic 405.2: Ratio of basic salary and remuneration of women to men? Alternatevely look for keywords: 405.2, GRI 405.2, GRI 405-2, 405-2, gender pay gap, pay equality, equal pay for equal work, </t>
+          <t>Does the company adopt the ILO’s Tripartite Declaration principles?</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>ALERION.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 405.2: Ratio of basic salary and remuneration of women to men? Alternatevely look for keywords: 405.2, GRI 405.2, GRI 405-2, 405-2, gender pay gap, pay equality, equal pay for equal work, ', 'context': [Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='a9b21330-cda2-4466-a0d8-0257f28fc7ab', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='proceeds. \nIn particular, this report will include the following information:  \n \nAllocation information: \n \n- The total amount of investments and expenditures in Eligible \nGreen Projects  \n- The amount and percentage of new and existing projects \n(financing and refinancing)  \n- The balance of unallocated proceeds  \n- A brief description of the projects financed or refinanced with the \nGreen Bond  \n \nImpact metrics:'), Document(id='8d2915a9-edec-472d-8bde-baa6034447b2', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 2, 'page_label': '3'}, page_content='Principles 2021 edition (“GBP”). The GBP core components are described as follow: \n1) Use of Proceeds \n2) Process for Project Evaluation and Selection \n3) Management of Proceeds \n4) Reporting \n5) External Review – Annual assurance report \n2.1- “ALERION GREEN BOND 2021 – 2027”- USE OF PROCEEDS \n \nAlerion intends to use the proceeds of the Green Bond 2021 – 2027 as follows: \n \n- the early redemption of the “Euro 150 million Alerion Clean Power \nS.p.A. 2018-2024” bond (ISIN IT0005333627);')], 'answer': 'Alerion does not mention considering GRI Topic 405.2 or any related keywords such as gender pay gap or pay equality in the provided context about their Green Bond activities. Therefore, it is not clear from the context if they consider this topic material.'}</t>
+          <t>Question: Does the company adopt the ILO’s Tripartite Declaration principles?
+Answer: Yes
+Evidence: "by the Declaration of the International Labor Organization (ILO) on principles and rights in the workplace"
+Location: Sustainability Report, not specified</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 406: Non discrimination? Alternatevely look for keywords: 406, GRI 406 , Non-discrimination, discrimination,  gender equality, gender, disability,nationality, age, sex, diversity, sexual orientation</t>
+          <t>Does the company participates to the UN Global Compact Network Italy?</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>ANTARES VISION.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 406: Non discrimination? Alternatevely look for keywords: 406, GRI 406 , Non-discrimination, discrimination,  gender equality, gender, disability,nationality, age, sex, diversity, sexual orientation', 'context': [Document(id='0448500f-2203-41b2-a68d-2453fb280872', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 113, 'page_label': '114'}, page_content='Sustainability report / NFR 2022 114 \n \n405-1 Diversity of governance \nbodies and employees \n03 Governance / Corporate bodies \n    \n  11 Human Resources / Employees      \n  \n    \n406 Non-discrimination 11 Human Resources \n    \n406-1 Incidents of \ndiscrimination and \ncorrective actions taken \n11 Human Resources / Employees  \n    \nMaterial \nTopic \nOccupational health and \nsafety \n          \n3.3 Management of \nmaterial topics \n11 Human Resources \n    \n  GRI Topic Standards           \n403 Occupational Health'), Document(id='e993be01-30d2-43d0-8a8d-c34f413d38a5', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 112, 'page_label': '113'}, page_content='401-2 Benefits provided to full-\ntime employees that are \nnot provided to \ntemporary or part-time \nemployees \n11 Human Resources / Employees  \n    \n404 Training and Education 11 Human Resources  \n    \n404-1 Average hours of \ntraining per year per \nemployee \n11 Human Resources / Training \n    \nMaterial \nTopic \nHuman resources: \nDiversity Equity \nInclusion \n          \n3.3 Management of \nmaterial topics \n11 Human Resources \n    \n  GRI Topic Standards           \n405 Diversity and equal \nopportunity'), Document(id='03709003-a87f-4ed3-a535-296a8cf0db52', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 63, 'page_label': '64'}, page_content='business model) \nShort-medium-long term (structural with \nrespect to the business model) \nExpected in connected with current \nproduction processes \n \n8 Human \nresources: \nDiversity \nEquity \nInclusion \nCreation of a work environment that \nguarantees respect, equal opportunities, \ndiversity and inclusion for all workers \nand protects them against all forms of \ndiscrimination. \n[Positive] \nactual: protection through Group Policies  GRI 405 Diversity \nand equal \nopportunity \n \nGRI 406 Non-\ndiscrimination')], 'answer': 'The company considers material under GRI Topic 406: Non-discrimination, as it is mentioned under Human Resources for addressing incidents of discrimination and corrective actions taken.'}</t>
+          <t>Question: Does the company participate in the UN Global Compact Network Italy?
+Answer: Yes
+Evidence: "Alerion is a member of the UN Global Compact Network Italy."
+Location: Page not specified</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 406: Non discrimination? Alternatevely look for keywords: 406, GRI 406 , Non-discrimination, discrimination,  gender equality, gender, disability,nationality, age, sex, diversity, sexual orientation</t>
+          <t>Does the company participates to the UN Global Compact Network Italy?</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 406: Non discrimination? Alternatevely look for keywords: 406, GRI 406 , Non-discrimination, discrimination,  gender equality, gender, disability,nationality, age, sex, diversity, sexual orientation', 'context': [Document(id='d58afd5a-fac6-4172-a844-c95c8369c66b', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 187, 'page_label': '186'}, page_content='404-2: Programs for upgrading employee skills and transition \nassistance programs p. 82-85\n404-3: Percentage of employees receiving regular performance \nand career development reviews p. 86; 87; 163\nDiversity, equity and inclusion\n3-3: Management of material topics p. 70-73; 142; 143; 146-151\n405-1: Diversity of governance bodies and employees p. 28; 29; 68; 69; 152; 153; 158-161\n405-2: Ratio of basic salary and remuneration of women to men p. 73\nThe indicator was calculated taking into'), Document(id='9f00d736-8b1d-4bcd-8d67-0e73fcae61ef', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 183, 'page_label': '182'}, page_content='Diversity, equity and inclusion GRI 405 Diversity and equal opportunity (2016) Personnel management\nand respecting human rights Group Franchisees; corporate \nshops on commission - No cover for franchisees\nPeople’s welfare and engagement GRI 401 Employment (2016) Personnel management Group Franchisees; corporate \nshops on commission - No cover for franchisees\nAwareness-raising and education on hearing well-being - Social aspects Group - - -\nSupporting the local communities - Social aspects Group - - -'), Document(id='99471124-d0de-4d91-9422-96186cd0a768', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 184, 'page_label': '183'}, page_content='Diversity, equity and inclusion GRI 405 Diversity and equal opportunity (2016) Personnel management\nand respecting human rights Group Franchisees; corporate \nshops on commission - No cover for franchisees\nPeople’s welfare and engagement GRI 401 Employment (2016) Personnel management Group Franchisees; corporate \nshops on commission - No cover for franchisees\nAwareness-raising and education on hearing well-being - Social aspects Group - - -\nSupporting the local communities - Social aspects Group - - -')], 'answer': 'The company mentions diversity, equity, and inclusion under GRI 405 Diversity and Equal Opportunity, which involves personnel management and respecting human rights. However, there is no specific mention of GRI Topic 406: Non-discrimination or related keywords within the provided context.'}</t>
+          <t>Question: Does the company participate in the UN Global Compact Network Italy?
+Answer: No
+Evidence: "At the date of this document, AV Group does not adhere to any other important external initiatives (charters, principles or other initiatives) developed externally at an economic, environmental and social level."
+Location: Page 28</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 406: Non discrimination? Alternatevely look for keywords: 406, GRI 406 , Non-discrimination, discrimination,  gender equality, gender, disability,nationality, age, sex, diversity, sexual orientation</t>
+          <t>Does the company adhere to the initiative Valore D?</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -1716,14 +1931,17 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 406: Non discrimination? Alternatevely look for keywords: 406, GRI 406 , Non-discrimination, discrimination,  gender equality, gender, disability,nationality, age, sex, diversity, sexual orientation', 'context': [Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='be81fe44-e632-4bee-a5fc-cb7489ea568b', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='legislation that requires specific environmental screening before receiving the building \npermit. \n \nEligible Green Projects are deemed to contribute to climate mitigation by helping to \navoid or reduce greenhouse gas (GHG) emissions, in alignment with Alerion’s strategy \nas previously discussed. Alerion anticipates that Eligible Green Projects will also \ncontribute to the UN Sustainable Development Goals number 7 (“Affordable and Clean'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.')], 'answer': 'Alerion does not provide specific information in the context about considering material under GRI Topic 406: Non-discrimination or related keywords such as discrimination, gender equality, or diversity.'}</t>
+          <t>Question: Does the company adhere to the initiative Valore D?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 407: Freedom of Association and Collective Bargaining? Alternatevely look for keywords: 407, GRI 407 , NFreedom of association, Collective Bargaining, right to be represented, trade unions</t>
+          <t>Does the company adhere to the initiative Valore D?</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -1733,82 +1951,94 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 407: Freedom of Association and Collective Bargaining? Alternatevely look for keywords: 407, GRI 407 , NFreedom of association, Collective Bargaining, right to be represented, trade unions', 'context': [Document(id='2dbb90bd-c74b-43b3-bb1b-65c3b52f0e12', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 110, 'page_label': '111'}, page_content='Economic] \n   \n  \n2.28 Membership associations 04 Sustainability: the commitment of AV Group / \nAdherence to external initiatives and \nMemberships \n   \n  \n  Involvement of stakeholders           \n2.29 Approach to stakeholder engagement 05 Stakeholders / Stakeholder relations and \nengagement \n   \n  \n2.30 Collective bargaining agreements 11 Human Resources /HR Policies \n   \n  \n \n \n \n \nGRI Standards – Disclosure Material topics / Specific indicators'), Document(id='0448500f-2203-41b2-a68d-2453fb280872', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 113, 'page_label': '114'}, page_content='Sustainability report / NFR 2022 114 \n \n405-1 Diversity of governance \nbodies and employees \n03 Governance / Corporate bodies \n    \n  11 Human Resources / Employees      \n  \n    \n406 Non-discrimination 11 Human Resources \n    \n406-1 Incidents of \ndiscrimination and \ncorrective actions taken \n11 Human Resources / Employees  \n    \nMaterial \nTopic \nOccupational health and \nsafety \n          \n3.3 Management of \nmaterial topics \n11 Human Resources \n    \n  GRI Topic Standards           \n403 Occupational Health'), Document(id='e993be01-30d2-43d0-8a8d-c34f413d38a5', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 112, 'page_label': '113'}, page_content='401-2 Benefits provided to full-\ntime employees that are \nnot provided to \ntemporary or part-time \nemployees \n11 Human Resources / Employees  \n    \n404 Training and Education 11 Human Resources  \n    \n404-1 Average hours of \ntraining per year per \nemployee \n11 Human Resources / Training \n    \nMaterial \nTopic \nHuman resources: \nDiversity Equity \nInclusion \n          \n3.3 Management of \nmaterial topics \n11 Human Resources \n    \n  GRI Topic Standards           \n405 Diversity and equal \nopportunity')], 'answer': 'AV Group includes material on collective bargaining as indicated in section 2.30 under Human Resources and HR Policies. However, there is no specific mention of GRI 407 related to Freedom of Association and Collective Bargaining in the provided context.'}</t>
+          <t>Question: Does the company adhere to the initiative Valore D?
+Answer: Information not explicitly disclosed
+Evidence: "The policy of Diversity, Equity and Inclusion adopted by the Group in 2023 available on the Antares Vision Group website (Company Documents | Group Policies), was drawn up in compliance with the internal policies and procedures of the Antares."
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 407: Freedom of Association and Collective Bargaining? Alternatevely look for keywords: 407, GRI 407 , NFreedom of association, Collective Bargaining, right to be represented, trade unions</t>
+          <t>Is the company included in the Bloomberg Gender Equality Index, also called Bloomberg GEI?</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 407: Freedom of Association and Collective Bargaining? Alternatevely look for keywords: 407, GRI 407 , NFreedom of association, Collective Bargaining, right to be represented, trade unions', 'context': [Document(id='b3b7fd49-b610-49da-b1a1-9ebeb35f7b70', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 186, 'page_label': '185'}, page_content='2-26: Mechanisms for seeking advice and raising concerns p. 128\n2-27: Compliance with laws and regulations\nIn the three-year period 2020-2022, no \nsignificant sanctions for non-compliance \nwith laws and regulations were recorded.\n2-28: Membership associations p. 45; 58\nStakeholder engagement\n2-29: Approach to stakeholders engagement p. 8; 9; 12; 144; 145\n2-30: Collective bargaining agreements p. 74; 75\nMaterial topics\n3-1: Process for determining material topics p. 6-12; 146-151; 182; 183'), Document(id='3d33faf2-fb4e-40e6-8767-d0a43e074e7a', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='• GRI 2-22: Sustainable Development \nStrategy Statement\nEmployment\n3. Businesses should support freedom of \nassociation and the effective recognition \nof the right of collective bargaining\n4. Business should support the \nelimination of all forms of forced, \ncompulsory labor\n5. Businesses should support the \neffective abolition of child labor\n6. Businesses should support the \nelimination of discrimination in \nemployment\n• Diversity, inclusion and equal \nopportunities \n• Well-being and internal engagement'), Document(id='1bdb8aeb-6381-4334-8d3d-f4590d3047cf', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 187, 'page_label': '186'}, page_content='Information Reference Notes/Omissions\nPeople’s welfare and engagement\n3-3: Management of material topics p. 74; 75; 142; 143; 146-151\n401-2: Benefits provided to full-time employees that are not \nprovided to temporary or part-time employees p. 74; 75\nEmployees’ health and safety\n3-3: Management of material topics p. 90; 91; 142; 143; 146-151\n403-1: Occupational health and safety management system p. 90; 91\n403-2: Hazard identification, risk assessment, and incident \ninvestigation p. 90; 91')], 'answer': 'The company supports freedom of association and the effective recognition of the right of collective bargaining, as indicated in their sustainable development strategy. This is consistent with GRI 407, which addresses freedom of association and collective bargaining.'}</t>
+          <t>Question: Is the company included in the Bloomberg Gender Equality Index, also called Bloomberg GEI?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 407: Freedom of Association and Collective Bargaining? Alternatevely look for keywords: 407, GRI 407 , NFreedom of association, Collective Bargaining, right to be represented, trade unions</t>
+          <t>Is the company included in the Bloomberg Gender Equality Index, also called Bloomberg GEI?</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ALERION.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 407: Freedom of Association and Collective Bargaining? Alternatevely look for keywords: 407, GRI 407 , NFreedom of association, Collective Bargaining, right to be represented, trade unions', 'context': [Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='be81fe44-e632-4bee-a5fc-cb7489ea568b', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='legislation that requires specific environmental screening before receiving the building \npermit. \n \nEligible Green Projects are deemed to contribute to climate mitigation by helping to \navoid or reduce greenhouse gas (GHG) emissions, in alignment with Alerion’s strategy \nas previously discussed. Alerion anticipates that Eligible Green Projects will also \ncontribute to the UN Sustainable Development Goals number 7 (“Affordable and Clean')], 'answer': "Alerion's Green Bond Framework document does not mention the GRI Topic 407: Freedom of Association and Collective Bargaining, nor does it reference related keywords such as collective bargaining, the right to be represented, or trade unions."}</t>
+          <t>Answer: Information not explicitly disclosed
+Evidence: "The selected indicators are in line with the challenges that the parent company, but eventually all the realities belonging to the Antares Vision Group ecosystem, will have to face in terms of continuous training and gender diversity."
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 408: Child Labour? Alternatevely look for keywords: GRI 408, 408, Child Labour, Child Labor, minor labour, minor labor, child work, child exploitation</t>
+          <t>Does the company have SA 8000 certification?</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>ANTARES VISION.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 408: Child Labour? Alternatevely look for keywords: GRI 408, 408, Child Labour, Child Labor, minor labour, minor labor, child work, child exploitation', 'context': [Document(id='6081e1a8-4653-499b-914b-527e4f73ed49', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 113, 'page_label': '114'}, page_content='safety management \nsystem \n11 Human Resources / Health and Safety of \nworkers \n    \n403-9 Work-related injuries 11 Human Resources / Health and Safety of \nworkers \n    \n403-10 Work-related ill health 11 Human Resources / Health and Safety of \nworkers \n    \nMaterial \nTopic \nProduct quality / \nCustomer health and \nsafety \n          \n3.3 Management of \nmaterial topics \n09 Quality, compliance and safety of the product \nand customers  \n    \n  GRI Topic Standards           \n416 Customer Health and \nSafety'), Document(id='12543286-6d20-4482-a6a8-75e4d13b794a', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 113, 'page_label': '114'}, page_content='417 Marketing and labelling \n     \n417-2 Incidents of non-\ncompliance concerning \nproduct and service \ninformation and labeling \n09 Quality, compliance and safety of the product \nand customers / The quality policy \n    \n417-3 Incidents of non-\ncompliance concerning \nmarketing \ncommunications \n09 Quality, compliance and safety of the product \nand customers / The quality policy  \n    \nMaterial \nTopic \nSuppliers: supply chain \nsustainability \n          \n3.3 Management of \nmaterial topics \n10 Supply Chain'), Document(id='0f9a7dba-f903-4fbe-a527-cf81666525ad', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 111, 'page_label': '112'}, page_content='and GRI 403 Health and Safety on the Workplace, published in 2018. Concerning the notice on waste, the GRI \n306 standard on waste, published in 2020. In the field of tax reporting, the GRI 207 on Taxes was applied \n(2019)  \n• Sector standards not published / not available (not applicable)  \n \nDisclosure Location/Reference Omissions GRI Sector \nStandards \nDescription   Requirements omitted Require\nments \nomitted \nReason Explanation Ref. Nr \n   \n    \n  \nGRI 3 – Material Topics 2021')], 'answer': 'The company does not mention or consider material under GRI Topic 408 regarding Child Labour.'}</t>
+          <t>Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 408: Child Labour? Alternatevely look for keywords: GRI 408, 408, Child Labour, Child Labor, minor labour, minor labor, child work, child exploitation</t>
+          <t>Does the company have SA 8000 certification?</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 408: Child Labour? Alternatevely look for keywords: GRI 408, 408, Child Labour, Child Labor, minor labour, minor labor, child work, child exploitation', 'context': [Document(id='3d33faf2-fb4e-40e6-8767-d0a43e074e7a', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='• GRI 2-22: Sustainable Development \nStrategy Statement\nEmployment\n3. Businesses should support freedom of \nassociation and the effective recognition \nof the right of collective bargaining\n4. Business should support the \nelimination of all forms of forced, \ncompulsory labor\n5. Businesses should support the \neffective abolition of child labor\n6. Businesses should support the \nelimination of discrimination in \nemployment\n• Diversity, inclusion and equal \nopportunities \n• Well-being and internal engagement'), Document(id='1bdb8aeb-6381-4334-8d3d-f4590d3047cf', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 187, 'page_label': '186'}, page_content='Information Reference Notes/Omissions\nPeople’s welfare and engagement\n3-3: Management of material topics p. 74; 75; 142; 143; 146-151\n401-2: Benefits provided to full-time employees that are not \nprovided to temporary or part-time employees p. 74; 75\nEmployees’ health and safety\n3-3: Management of material topics p. 90; 91; 142; 143; 146-151\n403-1: Occupational health and safety management system p. 90; 91\n403-2: Hazard identification, risk assessment, and incident \ninvestigation p. 90; 91'), Document(id='06e99e70-ce08-469b-b3a3-9e2d601fdfcf', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='and management methods, as well as the GRI Standards reported are described.\nArea Principle Reference GRI Standards\nHuman Rights\n1. Business should support and \nrespect the protection of human rights \nproclaimed at an international level\n2. Businesses should ensure that they are \nnot complicit in violations of human rights\n• Well-being and internal engagement\n• Business ethics and fighting corruption\n• Procurement and Supply Chain \nmanagement\n• Note on methodology\n• GRI 2-23: Policy commitment')], 'answer': 'The company supports the effective abolition of child labor, as outlined in their sustainable development strategy statement. However, there is no specific mention of GRI Topic 408 or related keywords in the provided context.'}</t>
+          <t>Answer: No
+Evidence: "Some other Antares Vision Group companies (RFXCEL, PENTEC and Imago Technologies) have adopted an ISO 9001:2015."
+Location: Page not specified</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 408: Child Labour? Alternatevely look for keywords: GRI 408, 408, Child Labour, Child Labor, minor labour, minor labor, child work, child exploitation</t>
+          <t>Does the company adopt the United Nation Women Empowerment Principles, also called WEP?</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -1818,14 +2048,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 408: Child Labour? Alternatevely look for keywords: GRI 408, 408, Child Labour, Child Labor, minor labour, minor labor, child work, child exploitation', 'context': [Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='8c8b278a-2039-4df6-a6f1-e4e4cd520379', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Pagina | 4  \n \n \nIn case of divestment, or if a project becomes ineligible, Alerion will strive to replace it \nby another Eligible Green Project on a best effort basis.   \n \n2.4- Reporting  \nAn annual report will be prepared and made available on Alerion’s website at \nwww.alerion.it, with the status of the Green Bond’s proceeds allocation, overview of the \nprojects financed or refinanced, and the environmental impact, until full allocation of \nproceeds.')], 'answer': 'Alerion does not specifically mention considering material under GRI Topic 408: Child Labour in the provided context.'}</t>
+          <t>Question: Does the company adopt the United Nation Women Empowerment Principles, also called WEP?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 409: Forced or Compulsory Labor ? Alternatevely look for keywords: GRI 409, 409, Forced Labour, Forced Labor, compulsory labour, compulsory labor, exploitative labour, exploitative labor, illigal labour, illigal labor</t>
+          <t>Does the company adopt the United Nation Women Empowerment Principles, also called WEP?</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -1835,82 +2068,96 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 409: Forced or Compulsory Labor ? Alternatevely look for keywords: GRI 409, 409, Forced Labour, Forced Labor, compulsory labour, compulsory labor, exploitative labour, exploitative labor, illigal labour, illigal labor', 'context': [Document(id='6081e1a8-4653-499b-914b-527e4f73ed49', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 113, 'page_label': '114'}, page_content='safety management \nsystem \n11 Human Resources / Health and Safety of \nworkers \n    \n403-9 Work-related injuries 11 Human Resources / Health and Safety of \nworkers \n    \n403-10 Work-related ill health 11 Human Resources / Health and Safety of \nworkers \n    \nMaterial \nTopic \nProduct quality / \nCustomer health and \nsafety \n          \n3.3 Management of \nmaterial topics \n09 Quality, compliance and safety of the product \nand customers  \n    \n  GRI Topic Standards           \n416 Customer Health and \nSafety'), Document(id='12543286-6d20-4482-a6a8-75e4d13b794a', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 113, 'page_label': '114'}, page_content='417 Marketing and labelling \n     \n417-2 Incidents of non-\ncompliance concerning \nproduct and service \ninformation and labeling \n09 Quality, compliance and safety of the product \nand customers / The quality policy \n    \n417-3 Incidents of non-\ncompliance concerning \nmarketing \ncommunications \n09 Quality, compliance and safety of the product \nand customers / The quality policy  \n    \nMaterial \nTopic \nSuppliers: supply chain \nsustainability \n          \n3.3 Management of \nmaterial topics \n10 Supply Chain'), Document(id='0f9a7dba-f903-4fbe-a527-cf81666525ad', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 111, 'page_label': '112'}, page_content='and GRI 403 Health and Safety on the Workplace, published in 2018. Concerning the notice on waste, the GRI \n306 standard on waste, published in 2020. In the field of tax reporting, the GRI 207 on Taxes was applied \n(2019)  \n• Sector standards not published / not available (not applicable)  \n \nDisclosure Location/Reference Omissions GRI Sector \nStandards \nDescription   Requirements omitted Require\nments \nomitted \nReason Explanation Ref. Nr \n   \n    \n  \nGRI 3 – Material Topics 2021')], 'answer': 'The company does not include a mention of GRI Topic 409: Forced or Compulsory Labor or related keywords in the provided context.'}</t>
+          <t>Question: Does the company adopt the United Nation Women Empowerment Principles, also called WEP?
+Answer: Yes
+Evidence: "With the adoption of the Policy on diversity, equity and inclusion, Antares Vision Group intends..."
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 409: Forced or Compulsory Labor ? Alternatevely look for keywords: GRI 409, 409, Forced Labour, Forced Labor, compulsory labour, compulsory labor, exploitative labour, exploitative labor, illigal labour, illigal labor</t>
+          <t>Does the company have a certified occupational health and safety management systems or ISO 45001?</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 409: Forced or Compulsory Labor ? Alternatevely look for keywords: GRI 409, 409, Forced Labour, Forced Labor, compulsory labour, compulsory labor, exploitative labour, exploitative labor, illigal labour, illigal labor', 'context': [Document(id='1bdb8aeb-6381-4334-8d3d-f4590d3047cf', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 187, 'page_label': '186'}, page_content='Information Reference Notes/Omissions\nPeople’s welfare and engagement\n3-3: Management of material topics p. 74; 75; 142; 143; 146-151\n401-2: Benefits provided to full-time employees that are not \nprovided to temporary or part-time employees p. 74; 75\nEmployees’ health and safety\n3-3: Management of material topics p. 90; 91; 142; 143; 146-151\n403-1: Occupational health and safety management system p. 90; 91\n403-2: Hazard identification, risk assessment, and incident \ninvestigation p. 90; 91'), Document(id='3d33faf2-fb4e-40e6-8767-d0a43e074e7a', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='• GRI 2-22: Sustainable Development \nStrategy Statement\nEmployment\n3. Businesses should support freedom of \nassociation and the effective recognition \nof the right of collective bargaining\n4. Business should support the \nelimination of all forms of forced, \ncompulsory labor\n5. Businesses should support the \neffective abolition of child labor\n6. Businesses should support the \nelimination of discrimination in \nemployment\n• Diversity, inclusion and equal \nopportunities \n• Well-being and internal engagement'), Document(id='b3b7fd49-b610-49da-b1a1-9ebeb35f7b70', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 186, 'page_label': '185'}, page_content='2-26: Mechanisms for seeking advice and raising concerns p. 128\n2-27: Compliance with laws and regulations\nIn the three-year period 2020-2022, no \nsignificant sanctions for non-compliance \nwith laws and regulations were recorded.\n2-28: Membership associations p. 45; 58\nStakeholder engagement\n2-29: Approach to stakeholders engagement p. 8; 9; 12; 144; 145\n2-30: Collective bargaining agreements p. 74; 75\nMaterial topics\n3-1: Process for determining material topics p. 6-12; 146-151; 182; 183')], 'answer': 'The company addresses the issue of forced or compulsory labor as one of its employment principles. It supports the elimination of all forms of forced, compulsory labor. However, there is no explicit mention of GRI Topic 409 in the provided context.'}</t>
+          <t>Answer: Information not explicitly disclosed
+Evidence: "Information not explicitly disclosed"
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 409: Forced or Compulsory Labor ? Alternatevely look for keywords: GRI 409, 409, Forced Labour, Forced Labor, compulsory labour, compulsory labor, exploitative labour, exploitative labor, illigal labour, illigal labor</t>
+          <t>Does the company have a certified occupational health and safety management systems or ISO 45001?</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>ALERION.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 409: Forced or Compulsory Labor ? Alternatevely look for keywords: GRI 409, 409, Forced Labour, Forced Labor, compulsory labour, compulsory labor, exploitative labour, exploitative labor, illigal labour, illigal labor', 'context': [Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='be81fe44-e632-4bee-a5fc-cb7489ea568b', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='legislation that requires specific environmental screening before receiving the building \npermit. \n \nEligible Green Projects are deemed to contribute to climate mitigation by helping to \navoid or reduce greenhouse gas (GHG) emissions, in alignment with Alerion’s strategy \nas previously discussed. Alerion anticipates that Eligible Green Projects will also \ncontribute to the UN Sustainable Development Goals number 7 (“Affordable and Clean')], 'answer': 'Alerion’s documentation does not mention the consideration of GRI Topic 409: Forced or Compulsory Labor or any related keywords such as Forced Labour, Forced Labor, compulsory labour, exploitative labour, or illegal labour.'}</t>
+          <t>Question: Does the company have a certified occupational health and safety management system or ISO 45001?
+Answer: Yes
+Evidence: "Some other Antares Vision Group companies (RFXCEL, PENTEC, and Imago Technologies) have adopted an ISO 9001:2015 UNI EN ISO 45001:2018 Management system for the health and safety of workers."
+Location: Page 11, Section "Human Resources"</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 411: Rights of Indigenous Peoples? Alternatevely look for keywords: GRI 411, 411, Rights of indigenous peoples, indigenous</t>
+          <t>Does the company have a certified occupational health and safety management systems or ISO 45001?</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>ANTARES VISION.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 411: Rights of Indigenous Peoples? Alternatevely look for keywords: GRI 411, 411, Rights of indigenous peoples, indigenous', 'context': [Document(id='e993be01-30d2-43d0-8a8d-c34f413d38a5', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 112, 'page_label': '113'}, page_content='401-2 Benefits provided to full-\ntime employees that are \nnot provided to \ntemporary or part-time \nemployees \n11 Human Resources / Employees  \n    \n404 Training and Education 11 Human Resources  \n    \n404-1 Average hours of \ntraining per year per \nemployee \n11 Human Resources / Training \n    \nMaterial \nTopic \nHuman resources: \nDiversity Equity \nInclusion \n          \n3.3 Management of \nmaterial topics \n11 Human Resources \n    \n  GRI Topic Standards           \n405 Diversity and equal \nopportunity'), Document(id='0448500f-2203-41b2-a68d-2453fb280872', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 113, 'page_label': '114'}, page_content='Sustainability report / NFR 2022 114 \n \n405-1 Diversity of governance \nbodies and employees \n03 Governance / Corporate bodies \n    \n  11 Human Resources / Employees      \n  \n    \n406 Non-discrimination 11 Human Resources \n    \n406-1 Incidents of \ndiscrimination and \ncorrective actions taken \n11 Human Resources / Employees  \n    \nMaterial \nTopic \nOccupational health and \nsafety \n          \n3.3 Management of \nmaterial topics \n11 Human Resources \n    \n  GRI Topic Standards           \n403 Occupational Health'), Document(id='cb3cc118-bd26-4824-b1d0-699b62a1e03e', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 2, 'page_label': '3'}, page_content='GRI Standards – General information ................................................................................................................................................ 110 \nGRI Standards – Disclosure Material topics / Specific indicators ................................................................................................ 111')], 'answer': 'The company does not list GRI Topic 411: Rights of Indigenous Peoples or related keywords in the provided context.'}</t>
+          <t>Question: Does the company have a certified occupational health and safety management system or ISO 45001?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided text.
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 411: Rights of Indigenous Peoples? Alternatevely look for keywords: GRI 411, 411, Rights of indigenous peoples, indigenous</t>
+          <t>Does the company have a certified occupational health and safety management systems or ISO 45001?</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 411: Rights of Indigenous Peoples? Alternatevely look for keywords: GRI 411, 411, Rights of indigenous peoples, indigenous', 'context': [Document(id='06e99e70-ce08-469b-b3a3-9e2d601fdfcf', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='and management methods, as well as the GRI Standards reported are described.\nArea Principle Reference GRI Standards\nHuman Rights\n1. Business should support and \nrespect the protection of human rights \nproclaimed at an international level\n2. Businesses should ensure that they are \nnot complicit in violations of human rights\n• Well-being and internal engagement\n• Business ethics and fighting corruption\n• Procurement and Supply Chain \nmanagement\n• Note on methodology\n• GRI 2-23: Policy commitment'), Document(id='1bdb8aeb-6381-4334-8d3d-f4590d3047cf', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 187, 'page_label': '186'}, page_content='Information Reference Notes/Omissions\nPeople’s welfare and engagement\n3-3: Management of material topics p. 74; 75; 142; 143; 146-151\n401-2: Benefits provided to full-time employees that are not \nprovided to temporary or part-time employees p. 74; 75\nEmployees’ health and safety\n3-3: Management of material topics p. 90; 91; 142; 143; 146-151\n403-1: Occupational health and safety management system p. 90; 91\n403-2: Hazard identification, risk assessment, and incident \ninvestigation p. 90; 91'), Document(id='d58afd5a-fac6-4172-a844-c95c8369c66b', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 187, 'page_label': '186'}, page_content='404-2: Programs for upgrading employee skills and transition \nassistance programs p. 82-85\n404-3: Percentage of employees receiving regular performance \nand career development reviews p. 86; 87; 163\nDiversity, equity and inclusion\n3-3: Management of material topics p. 70-73; 142; 143; 146-151\n405-1: Diversity of governance bodies and employees p. 28; 29; 68; 69; 152; 153; 158-161\n405-2: Ratio of basic salary and remuneration of women to men p. 73\nThe indicator was calculated taking into')], 'answer': 'The company does not indicate consideration of GRI Topic 411: Rights of Indigenous Peoples in the provided context. There is no mention of "GRI 411," "Rights of Indigenous Peoples," or "indigenous" in the information given.'}</t>
+          <t>Question: Does the company have a certified occupational health and safety management system or ISO 45001?
+Answer: Yes
+Evidence: "Some other Antares Vision Group companies (RFXCEL, PENTEC, and Imago Technologies) have adopted an ISO 9001:2015 UNI EN ISO 45001:2018 Management system for the health and safety of workers."
+Location: Page 11, Section "Human Resources"</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 411: Rights of Indigenous Peoples? Alternatevely look for keywords: GRI 411, 411, Rights of indigenous peoples, indigenous</t>
+          <t>Does the company adhers to BSCI Amfori's 11 human rights principles? To adhere, the company must explicitly report it on the Sustainability report</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -1920,14 +2167,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 411: Rights of Indigenous Peoples? Alternatevely look for keywords: GRI 411, 411, Rights of indigenous peoples, indigenous', 'context': [Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='be81fe44-e632-4bee-a5fc-cb7489ea568b', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='legislation that requires specific environmental screening before receiving the building \npermit. \n \nEligible Green Projects are deemed to contribute to climate mitigation by helping to \navoid or reduce greenhouse gas (GHG) emissions, in alignment with Alerion’s strategy \nas previously discussed. Alerion anticipates that Eligible Green Projects will also \ncontribute to the UN Sustainable Development Goals number 7 (“Affordable and Clean')], 'answer': 'Alerion\'s provided context does not mention any consideration of material under GRI Topic 411: Rights of Indigenous Peoples or related keywords such as "GRI 411" or "indigenous."'}</t>
+          <t>Question: Does the company adhere to BSCI Amfori's 11 human rights principles?
+Answer: Information not explicitly disclosed
+Evidence: "Information not explicitly disclosed"
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 412: Human rights assessment? Alternatevely look for keywords: GRI 412, 412, Human Rights Assessment</t>
+          <t>Does the company adhers to BSCI Amfori's 11 human rights principles? To adhere, the company must explicitly report it on the Sustainability report</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -1937,82 +2187,97 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 412: Human rights assessment? Alternatevely look for keywords: GRI 412, 412, Human Rights Assessment', 'context': [Document(id='6081e1a8-4653-499b-914b-527e4f73ed49', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 113, 'page_label': '114'}, page_content='safety management \nsystem \n11 Human Resources / Health and Safety of \nworkers \n    \n403-9 Work-related injuries 11 Human Resources / Health and Safety of \nworkers \n    \n403-10 Work-related ill health 11 Human Resources / Health and Safety of \nworkers \n    \nMaterial \nTopic \nProduct quality / \nCustomer health and \nsafety \n          \n3.3 Management of \nmaterial topics \n09 Quality, compliance and safety of the product \nand customers  \n    \n  GRI Topic Standards           \n416 Customer Health and \nSafety'), Document(id='0448500f-2203-41b2-a68d-2453fb280872', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 113, 'page_label': '114'}, page_content='Sustainability report / NFR 2022 114 \n \n405-1 Diversity of governance \nbodies and employees \n03 Governance / Corporate bodies \n    \n  11 Human Resources / Employees      \n  \n    \n406 Non-discrimination 11 Human Resources \n    \n406-1 Incidents of \ndiscrimination and \ncorrective actions taken \n11 Human Resources / Employees  \n    \nMaterial \nTopic \nOccupational health and \nsafety \n          \n3.3 Management of \nmaterial topics \n11 Human Resources \n    \n  GRI Topic Standards           \n403 Occupational Health'), Document(id='e993be01-30d2-43d0-8a8d-c34f413d38a5', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 112, 'page_label': '113'}, page_content='401-2 Benefits provided to full-\ntime employees that are \nnot provided to \ntemporary or part-time \nemployees \n11 Human Resources / Employees  \n    \n404 Training and Education 11 Human Resources  \n    \n404-1 Average hours of \ntraining per year per \nemployee \n11 Human Resources / Training \n    \nMaterial \nTopic \nHuman resources: \nDiversity Equity \nInclusion \n          \n3.3 Management of \nmaterial topics \n11 Human Resources \n    \n  GRI Topic Standards           \n405 Diversity and equal \nopportunity')], 'answer': 'The company does not mention GRI Topic 412: Human Rights Assessment or any related keywords in the provided context. The provided information focuses on health and safety, product quality, customer safety, diversity, and non-discrimination.'}</t>
+          <t>Question: Does the company adhere to BSCI Amfori's 11 human rights principles?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided text.
+Location: Sustainability report / NFR 2022 49</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 412: Human rights assessment? Alternatevely look for keywords: GRI 412, 412, Human Rights Assessment</t>
+          <t>Does the company adhere to the the code of labour practice specified by Ethical Trading Iniative?  To adhere, the company must explicitly report it on the Sustainability report</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 412: Human rights assessment? Alternatevely look for keywords: GRI 412, 412, Human Rights Assessment', 'context': [Document(id='06e99e70-ce08-469b-b3a3-9e2d601fdfcf', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='and management methods, as well as the GRI Standards reported are described.\nArea Principle Reference GRI Standards\nHuman Rights\n1. Business should support and \nrespect the protection of human rights \nproclaimed at an international level\n2. Businesses should ensure that they are \nnot complicit in violations of human rights\n• Well-being and internal engagement\n• Business ethics and fighting corruption\n• Procurement and Supply Chain \nmanagement\n• Note on methodology\n• GRI 2-23: Policy commitment'), Document(id='1bdb8aeb-6381-4334-8d3d-f4590d3047cf', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 187, 'page_label': '186'}, page_content='Information Reference Notes/Omissions\nPeople’s welfare and engagement\n3-3: Management of material topics p. 74; 75; 142; 143; 146-151\n401-2: Benefits provided to full-time employees that are not \nprovided to temporary or part-time employees p. 74; 75\nEmployees’ health and safety\n3-3: Management of material topics p. 90; 91; 142; 143; 146-151\n403-1: Occupational health and safety management system p. 90; 91\n403-2: Hazard identification, risk assessment, and incident \ninvestigation p. 90; 91'), Document(id='b3b7fd49-b610-49da-b1a1-9ebeb35f7b70', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 186, 'page_label': '185'}, page_content='2-26: Mechanisms for seeking advice and raising concerns p. 128\n2-27: Compliance with laws and regulations\nIn the three-year period 2020-2022, no \nsignificant sanctions for non-compliance \nwith laws and regulations were recorded.\n2-28: Membership associations p. 45; 58\nStakeholder engagement\n2-29: Approach to stakeholders engagement p. 8; 9; 12; 144; 145\n2-30: Collective bargaining agreements p. 74; 75\nMaterial topics\n3-1: Process for determining material topics p. 6-12; 146-151; 182; 183')], 'answer': 'The company does not specifically mention GRI 412: Human Rights Assessment in the provided context. However, human rights considerations are integrated into their principles and policies, such as supporting international human rights protection and ensuring they are not complicit in violations. They also reference policy commitments under GRI 2-23.'}</t>
+          <t>Question: Does the company adhere to the code of labor practice specified by the Ethical Trading Initiative?
+Answer: Information not explicitly disclosed
+Evidence: "Information not explicitly disclosed"
+Location: Page not specified</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 412: Human rights assessment? Alternatevely look for keywords: GRI 412, 412, Human Rights Assessment</t>
+          <t>Does the company adhere to the the code of labour practice specified by Ethical Trading Iniative?  To adhere, the company must explicitly report it on the Sustainability report</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>ALERION.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 412: Human rights assessment? Alternatevely look for keywords: GRI 412, 412, Human Rights Assessment', 'context': [Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='3d9bdf42-9b67-4115-baee-08a6808ab3c1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Impact metrics:  \n \nAlerion will also provide information on the expected output and environmental benefits \nof Eligible Green Projects. \n \nThe relevant metrics1 will include:  \n \n-  Installed renewable energy capacity in MW  \n-  Expected or actual annual renewable energy generation in MWh \nor GWh  \n-  Estimated annual GHG emissions avoided (in tCO2e)  \n \n \n2.5- External review – Annual Assurance Report \n \nAn external independent auditor confirmed that the allocation of the Green Bond is done')], 'answer': 'Alerion does not mention considering material under GRI Topic 412: Human Rights Assessment in the provided context. The focus of the provided document is on energy, industry innovation, infrastructure, and climate action related to their Green Bond framework. There is no mention of human rights assessment or GRI 412 in the given information.'}</t>
+          <t>Question: Does the company adhere to the code of labor practice specified by the Ethical Trading Initiative?
+Answer: Information not explicitly disclosed
+Evidence: "Minimum Safeguards - the same activities must also be conducted in compliance with the social criteria defined by the OECD guidelines and by the United Nations."
+Location: Page 47, Sustainability report / NFR 2022</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 413: Local communities? Alternatevely look for keywords:GRI 413, 413, Local Communities</t>
+          <t>Does the company adhere to labor standards and responsible sourcing principles set by Fair Labor Association, also called FLA? To adhere, the company must explicitly report it on the Sustainability report</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>ANTARES VISION.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 413: Local communities? Alternatevely look for keywords:GRI 413, 413, Local Communities', 'context': [Document(id='87f31bc7-d5c1-408f-8882-d8294ea56bcf', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 112, 'page_label': '113'}, page_content='energy and emissions  \n    \nMaterial \nTopic \nResponsible use of \nnatural resources \n          \n3.3 Management of \nmaterial topics \n12 Environmental impacts \n    \n  GRI Topic standards           \n303 Water and effluents - \n2018 \n12 Environmental impacts  \n    \n303-1 Interaction with water \nas a shared resource \n12 Environmental impacts / Sustainable \nmanagement of resources  \n    \n303-2 Management of water \ndischarge-related \nimpacts \n12 Environmental impacts / Sustainable \nmanagement of resources'), Document(id='0f9a7dba-f903-4fbe-a527-cf81666525ad', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 111, 'page_label': '112'}, page_content='and GRI 403 Health and Safety on the Workplace, published in 2018. Concerning the notice on waste, the GRI \n306 standard on waste, published in 2020. In the field of tax reporting, the GRI 207 on Taxes was applied \n(2019)  \n• Sector standards not published / not available (not applicable)  \n \nDisclosure Location/Reference Omissions GRI Sector \nStandards \nDescription   Requirements omitted Require\nments \nomitted \nReason Explanation Ref. Nr \n   \n    \n  \nGRI 3 – Material Topics 2021'), Document(id='6081e1a8-4653-499b-914b-527e4f73ed49', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 113, 'page_label': '114'}, page_content='safety management \nsystem \n11 Human Resources / Health and Safety of \nworkers \n    \n403-9 Work-related injuries 11 Human Resources / Health and Safety of \nworkers \n    \n403-10 Work-related ill health 11 Human Resources / Health and Safety of \nworkers \n    \nMaterial \nTopic \nProduct quality / \nCustomer health and \nsafety \n          \n3.3 Management of \nmaterial topics \n09 Quality, compliance and safety of the product \nand customers  \n    \n  GRI Topic Standards           \n416 Customer Health and \nSafety')], 'answer': 'The company does not mention GRI Topic 413 or the keywords "Local Communities" in the provided context.'}</t>
+          <t>Question: Does the company adhere to labor standards and responsible sourcing principles set by Fair Labor Association, also called FLA?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 413: Local communities? Alternatevely look for keywords:GRI 413, 413, Local Communities</t>
+          <t>Does the company adhere to labor standards and responsible sourcing principles set by Fair Labor Association, also called FLA? To adhere, the company must explicitly report it on the Sustainability report</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 413: Local communities? Alternatevely look for keywords:GRI 413, 413, Local Communities', 'context': [Document(id='1bdb8aeb-6381-4334-8d3d-f4590d3047cf', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 187, 'page_label': '186'}, page_content='Information Reference Notes/Omissions\nPeople’s welfare and engagement\n3-3: Management of material topics p. 74; 75; 142; 143; 146-151\n401-2: Benefits provided to full-time employees that are not \nprovided to temporary or part-time employees p. 74; 75\nEmployees’ health and safety\n3-3: Management of material topics p. 90; 91; 142; 143; 146-151\n403-1: Occupational health and safety management system p. 90; 91\n403-2: Hazard identification, risk assessment, and incident \ninvestigation p. 90; 91'), Document(id='b3b7fd49-b610-49da-b1a1-9ebeb35f7b70', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 186, 'page_label': '185'}, page_content='2-26: Mechanisms for seeking advice and raising concerns p. 128\n2-27: Compliance with laws and regulations\nIn the three-year period 2020-2022, no \nsignificant sanctions for non-compliance \nwith laws and regulations were recorded.\n2-28: Membership associations p. 45; 58\nStakeholder engagement\n2-29: Approach to stakeholders engagement p. 8; 9; 12; 144; 145\n2-30: Collective bargaining agreements p. 74; 75\nMaterial topics\n3-1: Process for determining material topics p. 6-12; 146-151; 182; 183'), Document(id='932b3d29-c212-4ab9-9d48-65db45957af3', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 188, 'page_label': '187'}, page_content='Awareness raising and education on hearing well-being \nGRI 3-3: Management of material topics p. 96; 97; 142; 143; 146-151\nInnovation, digitalization and personalization of the customer experience\nGRI 3-3: Management of material topics p. 48-53; 142; 143; 146-151\nResponsible management of the supply chain\nGRI 3-3: Management of material topics p. 122-125; 142; 143; 146-151\nSupporting the local communities\nGRI 3-3: Management of material topics p. 94; 95; 98-107; 142; 143; 146-151')], 'answer': 'The company addresses supporting local communities as part of its management of material topics. This does align with the general idea of material topics related to local communities, although it does not explicitly mention "GRI 413."'}</t>
+          <t>Question: Does the company adhere to labor standards and responsible sourcing principles set by Fair Labor Association, also called FLA?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: Sustainability report / NFR 2022 47, 62, 85</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 413: Local communities? Alternatevely look for keywords:GRI 413, 413, Local Communities</t>
+          <t>Is the company part of the alliance Platform Living Wage Financials and adhers to its principles? To adhere, the company must explicitly report it on the Sustainability report</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2022,14 +2287,17 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 413: Local communities? Alternatevely look for keywords:GRI 413, 413, Local Communities', 'context': [Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='be81fe44-e632-4bee-a5fc-cb7489ea568b', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='legislation that requires specific environmental screening before receiving the building \npermit. \n \nEligible Green Projects are deemed to contribute to climate mitigation by helping to \navoid or reduce greenhouse gas (GHG) emissions, in alignment with Alerion’s strategy \nas previously discussed. Alerion anticipates that Eligible Green Projects will also \ncontribute to the UN Sustainable Development Goals number 7 (“Affordable and Clean'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.')], 'answer': "Alerion's provided context does not mention the consideration of GRI Topic 413: Local Communities or keywords such as GRI 413, 413, or Local Communities."}</t>
+          <t>Question: Is the company part of the alliance Platform Living Wage Financials and adheres to its principles?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 418: Customer privacy ? Alternatevely look for keywords:GRI 418, 418, Customer Privacy</t>
+          <t>Is the company part of the alliance Platform Living Wage Financials and adhers to its principles? To adhere, the company must explicitly report it on the Sustainability report</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2039,82 +2307,96 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 418: Customer privacy ? Alternatevely look for keywords:GRI 418, 418, Customer Privacy', 'context': [Document(id='3012e59b-0d8c-462b-96be-a6fc8b062c25', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 114, 'page_label': '115'}, page_content='privacy \n          \n3.3 Management of \nmaterial topics \n08 Integrity in business management \n    \n  GRI Topic Standards           \n418 Customers Privacy 08 Integrity in business management \n    \n418-1 Substantiated \ncomplaints concerning \nbreaches of customer \nprivacy and losses of \ncustomer data \n08 Integrity in business management / Privacy &amp; \nData Security  \n    \nMaterial \nTopic \nInnovation, research \nand development \n          \n3.3 Management of \nmaterial topics'), Document(id='fc6ab75b-7979-4060-a030-49305984f7ec', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 114, 'page_label': '115'}, page_content='Sustainability report / NFR 2022 115 \n \n  GRI Topic Standards           \n308 Environmental \nevaluation of suppliers \n10 Supply Chain  \n    \n308-1 New suppliers that were \nscreened using \nenvironmental criteria \n10 Supply Chain / Selection and evaluation of \nsuppliers \n    \n414 Social evaluation of \nsuppliers \n10 Supply Chain  \n    \n414-1 New suppliers that were \nscreened using social \ncriteria \n10 Supply Chain / Selection and evaluation of \nsuppliers \n    \nMaterial \nTopic \nData security and \nprivacy'), Document(id='8389d367-3f80-4427-aa35-89477303a3b2', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 63, 'page_label': '64'}, page_content='risk of violations and protects \ninformation security and privacy \n(cybersecurity and data protection for \ncustomers and employees. \n[Negative] \npotential: protection of corporate and \ncustomer data \nGRI 418 Customer \nprivacy \nSocial \nDirectly and through commercial \nrelationships (structural with respect to the \nbusiness model) \nShort-medium-long term (structural with \nrespect to the business model)')], 'answer': 'The company considers GRI Topic 418: Customer Privacy as a material topic, with a focus on integrity in business management, privacy, and data security.'}</t>
+          <t>Question: Is the company part of the alliance Platform Living Wage Financials and adheres to its principles?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the sustainability report.
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 418: Customer privacy ? Alternatevely look for keywords:GRI 418, 418, Customer Privacy</t>
+          <t>Does the company report in accordance with Human Rights Indicators for Business? Consider the company to report in accordance with Human Rights Indicators for Business only if explicitely written in the Sustainability Report</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 418: Customer privacy ? Alternatevely look for keywords:GRI 418, 418, Customer Privacy', 'context': [Document(id='dff76e94-9adb-458b-96db-2582eafec923', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 188, 'page_label': '187'}, page_content='In the three-year period 2020-2022 no\nsignificant reports concerning product and \nservices information and labelling were \nreceived.\n417-3: Incidents of non-compliance concerning marketing \ncommunications\nIn the three-year period 2020-2022 no\nsignificant reports concerning sales and \nmarketing communication were received.\nCybersecurity and data privacy\n3-3: Management of Management of material topics p. 60-63; 142; 143; 146-151. \n418-1: Substantiated complaints concerning breaches'), Document(id='90320dd4-245b-447e-b83b-fe7f180a432f', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 188, 'page_label': '187'}, page_content='of customer privacy and losses of customer data\nIn the three-year period 2020-2022, the \nsystems implemented for data protection\nand cybersecurity ensured\nan adequate level of protection for\nthe data. In 2022 there were no serious\ncases violation of customer’s privacy by \ncontrol bodies and outside organization.\nMaterial topics not directly related to GRI disclosures\nAvailability and accessibility to hearing care \nGRI 3-3: Management of material topics p. 56; 57; 142; 143; 146-151'), Document(id='9f20260d-f7d5-4647-b30b-195f4f42e827', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 183, 'page_label': '182'}, page_content='Quality, reliability and safety of products and services GRI 416 Customer health and safety (2016) Social aspects Group\nHearing aids \nmanufacturers; \nfranchisees; corporate \nshops on commission\n- Partial cover for manufacturers\nCybersecurity and data privacy GRI 418 Customer privacy (2016) Social aspects Group - - -\nResponsible marketing and sales practices GRI 417 Marketing and labeling (2016) Social aspects Group\nHearing aids \nmanufacturers; \nfranchisees; corporate \nshops on commission')], 'answer': 'The company considers Customer Privacy as a material topic under GRI 418, as indicated by the mention of GRI 418 concerning cybersecurity and data privacy in the provided context.'}</t>
+          <t>Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided text.
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Does the company consider material under GRI theTopic 418: Customer privacy ? Alternatevely look for keywords:GRI 418, 418, Customer Privacy</t>
+          <t>Does the company report in accordance with Human Rights Indicators for Business? Consider the company to report in accordance with Human Rights Indicators for Business only if explicitely written in the Sustainability Report</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>ALERION.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company consider material under GRI theTopic 418: Customer privacy ? Alternatevely look for keywords:GRI 418, 418, Customer Privacy', 'context': [Document(id='be81fe44-e632-4bee-a5fc-cb7489ea568b', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='legislation that requires specific environmental screening before receiving the building \npermit. \n \nEligible Green Projects are deemed to contribute to climate mitigation by helping to \navoid or reduce greenhouse gas (GHG) emissions, in alignment with Alerion’s strategy \nas previously discussed. Alerion anticipates that Eligible Green Projects will also \ncontribute to the UN Sustainable Development Goals number 7 (“Affordable and Clean'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='8c8b278a-2039-4df6-a6f1-e4e4cd520379', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Pagina | 4  \n \n \nIn case of divestment, or if a project becomes ineligible, Alerion will strive to replace it \nby another Eligible Green Project on a best effort basis.   \n \n2.4- Reporting  \nAn annual report will be prepared and made available on Alerion’s website at \nwww.alerion.it, with the status of the Green Bond’s proceeds allocation, overview of the \nprojects financed or refinanced, and the environmental impact, until full allocation of \nproceeds.')], 'answer': 'Alerion does not mention considering material under GRI Topic 418: Customer Privacy in the provided context. The focus is on Eligible Green Projects, climate mitigation, and related reporting. There is no indication of a focus on customer privacy or the GRI 418 standard in the given information.'}</t>
+          <t>Question: Does the company report in accordance with Human Rights Indicators for Business?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: Page not specified</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Does the company reports in accordance with the GRI standards?</t>
+          <t>Does the company adopt 6 principles set by Principles for responsible investment ? Please consider the company adopting the Principles for responsible investment  only if explicitely written in the Sustainability Report</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>ANTARES VISION.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company reports in accordance with the GRI standards?', 'context': [Document(id='7151fc42-b804-45e5-8c38-4045aa15b563', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 7, 'page_label': '8'}, page_content='It should be noted that, for the reporting for the 2022 financial year, the GRI standards published in 2021 were applied, which \nupdated the drafting process, the general information and the process of identifying and assessing the material topics: GRI \n1 Fundamental principles; GRI 2 General information; GRI 3 Material topics. \n \nThe GRI 1 Foundation 2021 defines the general principles of sustainability reporting (Reporting principles): accuracy, balance,'), Document(id='2b389c7d-659a-4f1f-b258-87770d645066', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 109, 'page_label': '110'}, page_content='Sustainability report / NFR 2022 110 \n \nGRI Content Index \n \n \nGRI Content Index - with reference to the GRI Standards    \nStatement of use The Consolidated Non-Financial Statement (Sustainability Report of Antares Vision \nGroup for the year 2022 [01 January – 31 December 2022] has been prepared in \naccordance with the GRI Standards reporting option.  \n  \nGRI 1 adopted GRI 1 Foundation 2021 \nApplicable GRI Sector Standards Not applicable / not available \n \n \nGRI Standards – General information'), Document(id='a60a397f-5869-4f73-8039-f4185d0c5f8c', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 8, 'page_label': '9'}, page_content="statements of Antares Vision S.p.A. Their Independent Auditors' Report is included in the appendix of this document. \n \nThe NFR is published on the Company's institutional website at Sustainability | Antares Vision and Investors | Antares Vision. \nFor further information, please contact the following address: sustainability@antaresvision.com.  \n \nAntares Vision S.p.A has notified the GRI (Global Reporting Initiative) of the use of the GRI Standards and the relative \nstatement of use.")], 'answer': 'Antares Vision reports in accordance with the GRI Standards.'}</t>
+          <t>Question: Does the company adopt 6 principles set by Principles for responsible investment?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Does the company reports in accordance with the GRI standards?</t>
+          <t>Does the company adopt 6 principles set by Principles for responsible investment ? Please consider the company adopting the Principles for responsible investment  only if explicitely written in the Sustainability Report</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company reports in accordance with the GRI standards?', 'context': [Document(id='7d65950d-1b78-4696-b7ba-fe0184f6baff', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 176, 'page_label': '175'}, page_content='tion “in accordance”. It should also be noted that Amplifon, when publishing this document, \nadopted the most updated versions available of the GRI Universal Standards, GRI Stan -\ndards 306 (Waste) and GRI Standards 403 (Occupational Health and Safety), published re -\nspectively in 2021, 2020 and 2018. Annexed to this document is the table of GRI Standards \nwhich serves as a compass to aid the navigation of the Report ( GRI Content Index).'), Document(id='40d8c9ad-5efe-45a3-aeb7-12296a4e4b7e', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 185, 'page_label': '184'}, page_content='The table below contains the GRI Standards reported in this document and the related \ndisclosures. Each disclosure has a reference to the section of the Report in which it can be \nfound, or to other publicly-available sources to refer to.\nDeclaration of use Amplifon has reported in accordance with the GRI Standards for the period January \n1st, 2022 - December 31st, 2022\nUse of GRI 1 GRI 1: Foundation 2021'), Document(id='dbb7408d-fe15-49fc-9b12-947b4cf291b6', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 185, 'page_label': '184'}, page_content='Pertinent GRI sector standards There are no GRI Sector indicators pertinent to the Amplifon business sector\nInformation Reference Notes/Omissions\nGRI 2: General information\nThe organization and its reporting practices\n2-1: Organizational details p. 23; 44; 174; 180\n2-2: Entities included in the organization’s\nsustainability reporting p. 176; 177\n2-3: Reporting period, frequency and contact point p. 175; 176; 180; inside-back cover\n2-4: Restatement of information p. 166; 167')], 'answer': 'Amplifon reports in accordance with the GRI Standards for the period January 1st, 2022 - December 31st, 2022.'}</t>
+          <t>Question: Does the company adopt 6 principles set by Principles for Responsible Investment?
+Answer: Information not explicitly disclosed
+Evidence: "responsible for compliance with these principles and should seek clarification when appropriate."
+Location: Page 47, Sustainability report / NFR 2022</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Does the company reports in accordance with the GRI standards?</t>
+          <t>Does the company adhere to Voluntary Principles on Security and Human Rights? Please consider the company adopting the  Voluntary Principles on Security and Human Rights only if explicitely written in the Sustainability Report</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2124,14 +2406,17 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company reports in accordance with the GRI standards?', 'context': [Document(id='8c8b278a-2039-4df6-a6f1-e4e4cd520379', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Pagina | 4  \n \n \nIn case of divestment, or if a project becomes ineligible, Alerion will strive to replace it \nby another Eligible Green Project on a best effort basis.   \n \n2.4- Reporting  \nAn annual report will be prepared and made available on Alerion’s website at \nwww.alerion.it, with the status of the Green Bond’s proceeds allocation, overview of the \nprojects financed or refinanced, and the environmental impact, until full allocation of \nproceeds.'), Document(id='8e92e81d-a44b-4d44-84b0-f8274704ad43', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 0, 'page_label': '1'}, page_content='Pagina | 0  \n \n \n  \nAnnual report prepared and made \navailable on Alerion’s website at \nwww.alerion.it, with the status of \nthe Green Bond’s proceeds \nallocation, overview of the projects \nfinanced or refinanced, and the \nenvironmental impact, until full \nallocation of proceeds. \nALERION \nGREEN BOND     \n2021–2027 \n_________ \nREPORT  \nYEAR 2022 \nUse of Proceeds'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.')], 'answer': "Alerion makes their annual report available on their website with details on the Green Bond's allocation and impacts, but the context does not specify if they report in accordance with GRI standards."}</t>
+          <t>Question: Does the company adhere to Voluntary Principles on Security and Human Rights?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Is the company a signatory of the United Nation Global Compact, also called UNGC?</t>
+          <t>Does the company adhere to Voluntary Principles on Security and Human Rights? Please consider the company adopting the  Voluntary Principles on Security and Human Rights only if explicitely written in the Sustainability Report</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2141,82 +2426,97 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>{'input': 'Is the company a signatory of the United Nation Global Compact, also called UNGC?', 'context': [Document(id='75c5dbc0-d6b8-4368-927a-395136c411fc', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 91, 'page_label': '92'}, page_content='Vision Group as well as in compliance with the main international conventions, standards a nd recommendations on the \nsubject, namely, on the reference framework defined by the International Charter of Human Rights, by the Declaration of the \nInternational Labor Organization (ILO) on principles and rights in the workplace and by the eight core conventions of the ILO \n(No. 29, 87, 98, 100, 105, 111, 138, 182), and by the principles defined by the United Nations Global Compact in collaboration'), Document(id='c24ab15d-cfef-4356-ab09-02a4e013d0d4', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 61, 'page_label': '62'}, page_content='United Nations Human Rights (UNHR), 2011. Guiding Principles on Business and Human Rights. Implementing the United Nations “Protect, \nRespect and Remedy” Framework \nConvention on Biological Diversity (2022), Kunming-Montreal Global Biodiversity Framework \nSASB – Sustainability Accounting Standards – Materiality Finder  \nESRS – European Sustainability Reporting Standards (Draft) \nIFRS-S – International Financial Reporting Standards – Sustainability (Draft IFRS S1-S2)'), Document(id='fb47bb04-a2c8-4d32-8355-ea303c8aef65', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 65, 'page_label': '66'}, page_content='3-3  \n \n \nThe commitments of Antares Vision Group with respect to the material topics identified are represented in the following \ngraphic, which also recalls their correlation and coherence with the United Nations 2030 Agenda and the SDGs - Sustainable \nDevelopment Goals and 164 targets identified by the Agenda). \n \nThe objectives, actions and management of the related issues and impacts, as well as the processes and procedures')], 'answer': 'Vision Group is in compliance with principles defined by the United Nations Global Compact, indicating they support its values, but the context does not confirm if they are an official signatory of the UNGC.'}</t>
+          <t>Question: Does the company adhere to Voluntary Principles on Security and Human Rights?
+Answer: Information not explicitly disclosed
+Evidence: "The Human Rights policy of Antares Vision Group was drawn up starting from the identification of the potentially most vulnerable elements within its value chain..."
+Location: Sustainability report / NFR 2022, page 49</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Is the company a signatory of the United Nation Global Compact, also called UNGC?</t>
+          <t>Does the company implement the practices recommended in the CEO Guide to Human Rights?</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>{'input': 'Is the company a signatory of the United Nation Global Compact, also called UNGC?', 'context': [Document(id='8d17b503-7421-4e6e-9c15-132d388b7046', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 42, 'page_label': '41'}, page_content='multi-stakeholder partnership and contributing to the global and shared efforts for the \n2030 Agenda for Sustainable Development. Also, for this reason, Amplifon signed up to \nthe United Nations Global Compact and takes part in the initiatives of the Italian network \nwith the aim of promoting an increasingly responsible business capable of meeting global \nchallenges through compliance with, adherence to and promotion of the Ten Principles'), Document(id='9891a1ce-2c42-4b91-b37d-1c300ec8106b', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 2, 'page_label': '1'}, page_content='To strengthen the contribution to the United Nations 2030 Agenda for Sustainable \nDevelopment, Amplifon takes part to United Nations Global Compact  through \nadherence, respect, and promotion of its Ten Principles.\nSustainability \nReport 2022'), Document(id='10a2ea9b-20c4-4ec6-9aa6-75ca187040f6', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='CONTENT INDEX OF THE TEN PRINCIPLES\nOF THE UNITED NATIONS GLOBAL COMPACT \nAs a member of the UN Global Compact, Amplifon reports, in this Sustainability Report, the \nmain activities and progress made for the implementation and compliance with the Ten Prin-\nciples of the UNGC. Therefore, with a view to transparency and sharing with all stakeholders, \nthe table below illustrates, for each Principle, in which part of the document the main activities')], 'answer': 'Amplifon is a signatory of the United Nations Global Compact.'}</t>
+          <t>Question: Does the company implement the practices recommended in the CEO Guide to Human Rights?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided sustainability report.
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Is the company a signatory of the United Nation Global Compact, also called UNGC?</t>
+          <t>Does the company implement the practices recommended in the CEO Guide to Human Rights?</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>ALERION.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>{'input': 'Is the company a signatory of the United Nation Global Compact, also called UNGC?', 'context': [Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='be81fe44-e632-4bee-a5fc-cb7489ea568b', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='legislation that requires specific environmental screening before receiving the building \npermit. \n \nEligible Green Projects are deemed to contribute to climate mitigation by helping to \navoid or reduce greenhouse gas (GHG) emissions, in alignment with Alerion’s strategy \nas previously discussed. Alerion anticipates that Eligible Green Projects will also \ncontribute to the UN Sustainable Development Goals number 7 (“Affordable and Clean'), Document(id='1603dfa0-95cf-4193-b970-a97988e35cc1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 1, 'page_label': '2'}, page_content='further in Europe, both in \nwind and solar sector. \n Alerion’s exclusive focus \non renewable energy \nimplies that sustainability \nis strictly embedded in our \nbusiness model. Our \noperations contribute \ndirectly to the reduction of \ngreenhouse gas (GHG) \nemissions and to the \npromotion of a system for \nsustainable territorial \ndevelopment. To this end, \nwe have in place a strong \nintegrated system for the \nassessment and \nmanagement of our')], 'answer': "Alerion's involvement with the United Nations Global Compact is not mentioned in the provided document. Therefore, based on the given context, it's not possible to determine if the company is a signatory of the UNGC."}</t>
+          <t>Question: Does the company implement the practices recommended in the CEO Guide to Human Rights?
+Answer: Yes
+Evidence: "Vision Group as well as in compliance with the main international conventions, standards and recommendations on the subject, namely, on the reference framework defined by the International Charter of Human Rights, by the Declaration of the International Labor Organization (ILO) on principles and rights in the workplace..."
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Does the company adopt the OECD Guidelines for Multinational Enterprises?</t>
+          <t>Does the company endor the Universal Bill of Human Rights?</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>ANTARES VISION.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company adopt the OECD Guidelines for Multinational Enterprises?', 'context': [Document(id='76e600a3-b3b2-448c-9bc3-5c842ec397d2', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 49, 'page_label': '50'}, page_content="▪ the Company's activity  is oriented towards strict compliance with laws and regulations , in all countries where the \nCompany operates;  \n▪ the Company undertakes to ensure that all of the Company's employees, managers, directors, co-workers, suppliers and \ncustomers - as well as the personnel and officials of other companies with whom joint or coordinated activities are \ncarried out, even temporarily - respect the laws and regulations in force  in all countries where the Company operates,"), Document(id='e62cfff9-b48f-40cf-953a-58b0095275b7', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 61, 'page_label': '62'}, page_content='consequently identifying the main impacts, trends a nd dynamics of change characterizing a given sector in the short, \nmedium and long term. \n \nThe sector guide OECD Due Diligence Guidance for Responsible Business Conduct provides practical support to companies \nfor the implementation of the non-binding OECD Guidelines for multinational companies, aimed at identifying and managing \nthe negative impacts related to labour law, human rights, environment, corruption, consumers and corporate governance'), Document(id='75c5dbc0-d6b8-4368-927a-395136c411fc', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 91, 'page_label': '92'}, page_content='Vision Group as well as in compliance with the main international conventions, standards a nd recommendations on the \nsubject, namely, on the reference framework defined by the International Charter of Human Rights, by the Declaration of the \nInternational Labor Organization (ILO) on principles and rights in the workplace and by the eight core conventions of the ILO \n(No. 29, 87, 98, 100, 105, 111, 138, 182), and by the principles defined by the United Nations Global Compact in collaboration')], 'answer': 'Vision Group adopts the OECD Guidelines for Multinational Enterprises by implementing the OECD Due Diligence Guidance for Responsible Business Conduct. This provides practical support to identify and manage negative impacts related to various aspects such as labor law, human rights, and the environment.'}</t>
+          <t>Question: Does the company endorse the Universal Bill of Human Rights?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided text.
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Does the company adopt the OECD Guidelines for Multinational Enterprises?</t>
+          <t>Does the company endor the Universal Bill of Human Rights?</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company adopt the OECD Guidelines for Multinational Enterprises?', 'context': [Document(id='c82bcb4f-0397-45f0-acbf-8ae562c05023', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 124, 'page_label': '123'}, page_content='ning the principles and standards of conduct required by all suppliers and business partners \nwith respect to the areas of business ethics, compliance, anti-corruption, human rights and \nworkers’ rights, diversity and inclusion, health, safety, the environment, etc.37.\nDuring the year, the mandatory acceptance of this Code was included in the qualification \nprocess for new suppliers, so that any new supplier signs up to it and its proactive imple -'), Document(id='829d969c-8a84-4f28-aa93-9b33c9072a85', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 132, 'page_label': '131'}, page_content='petent authorities to provide the necessary information for checking tax obligations have \nbeen correctly complied with and adopts behavior aimed at guaranteeing the suitability of \ntransfer prices applied in inter-group transactions, with the aim of allocating the revenue ge-\nnerated in the countries in which the Group operates, in compliance with the laws and in line \nwith OECD guidelines. Based on this approach and these principles, in order to ensure that'), Document(id='1ac9a44a-4757-4315-9432-a7ca6eb63415', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 175, 'page_label': '174'}, page_content="suppliers, in accordance with the principles and values set out in the Group's Code of \nEthics and Sustainability Policy and in full compliance with the Universal Declaration of \nHuman Rights and the International Labor Organization Conventions on fundamental \nhuman rights, as well as in line with the Principles of the UN Global Compact;\n ■ In light of the specific business model and the lack of any type of production activity,")], 'answer': 'The company ensures compliance with the laws and aligns with OECD guidelines for transfer pricing and revenue allocation in the countries it operates in.'}</t>
+          <t>Question: Does the company endorse the Universal Bill of Human Rights?
+Answer: Yes
+Evidence: "The policy, available on the Antares Vision Group website, has been developed in accordance with the main international human rights conventions, standards and recommendations (International Bill of Human Rights and the Convention on the Rights of the Child of the United Nations..."
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Does the company adopt the OECD Guidelines for Multinational Enterprises?</t>
+          <t>Does the company endor the Universal Declaration of Human Rights?</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2226,14 +2526,16 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company adopt the OECD Guidelines for Multinational Enterprises?', 'context': [Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='0286a4fd-14d3-46e6-a8c3-ddf45c3eb47d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='The Committee will be chaired by the Chairman of the Board of Directors, and composed \nof the other Board Executive Directors, together with the Chief Financial Officer and \nChief Operating Officer. \n \nThe Committee will be in charge of monitoring the selection and allocation of funds to \nEligible Green Projects and will be responsible for the following: \n \n- Identifying potential Eligible Green Projects;  \n \n- Reviewing and approving the selection against the eligibility')], 'answer': "Alerion's Green Bond 2021 – 2027 Framework does not specify whether the company adopts the OECD Guidelines for Multinational Enterprises."}</t>
+          <t>Answer: Yes
+Evidence: "Alerion is committed to the principles of the United Nations Global Compact (UNGC) and the Universal Declaration of Human Rights."
+Location: Page 4, Section "Our Commitment to Sustainability"</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Does the company adopt the ILO’s Tripartite Declaration principles?</t>
+          <t>Does the company endor the Universal Declaration of Human Rights?</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -2243,82 +2545,97 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company adopt the ILO’s Tripartite Declaration principles?', 'context': [Document(id='75c5dbc0-d6b8-4368-927a-395136c411fc', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 91, 'page_label': '92'}, page_content='Vision Group as well as in compliance with the main international conventions, standards a nd recommendations on the \nsubject, namely, on the reference framework defined by the International Charter of Human Rights, by the Declaration of the \nInternational Labor Organization (ILO) on principles and rights in the workplace and by the eight core conventions of the ILO \n(No. 29, 87, 98, 100, 105, 111, 138, 182), and by the principles defined by the United Nations Global Compact in collaboration'), Document(id='ebb08d4c-7962-44e5-ad11-1acca0c46725', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content='Human Rights and the Convention on the Rights of the Child of the United Nations, Fundamental Conventions of the \nInternational Labour Organization (ILO), Declaration of Principles and Fundamental Rights at Work, European Convention for \nthe Protection of Human Rights and Fundamental Freedoms (ECHR), as well as in compliance with the internal policies and \nprocedures of the Antares Vision Group.'), Document(id='76e600a3-b3b2-448c-9bc3-5c842ec397d2', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 49, 'page_label': '50'}, page_content="▪ the Company's activity  is oriented towards strict compliance with laws and regulations , in all countries where the \nCompany operates;  \n▪ the Company undertakes to ensure that all of the Company's employees, managers, directors, co-workers, suppliers and \ncustomers - as well as the personnel and officials of other companies with whom joint or coordinated activities are \ncarried out, even temporarily - respect the laws and regulations in force  in all countries where the Company operates,")], 'answer': "Vision Group adheres to the principles defined by various ILO declarations and conventions, though the context provided does not specifically mention the Tripartite Declaration of Principles concerning Multinational Enterprises and Social Policy. Therefore, it's unclear from the provided information whether Vision Group explicitly adopts the ILO's Tripartite Declaration principles."}</t>
+          <t>Question: Does the company endorse the Universal Declaration of Human Rights?
+Answer: Yes
+Evidence: "The policy, available on the Antares Vision Group website, has been developed in accordance with the main international human rights conventions, standards and recommendations..."
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Does the company adopt the ILO’s Tripartite Declaration principles?</t>
+          <t>Does the company endor the UN Guiding Principles, aslo called UNGPs?</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company adopt the ILO’s Tripartite Declaration principles?', 'context': [Document(id='3d33faf2-fb4e-40e6-8767-d0a43e074e7a', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='• GRI 2-22: Sustainable Development \nStrategy Statement\nEmployment\n3. Businesses should support freedom of \nassociation and the effective recognition \nof the right of collective bargaining\n4. Business should support the \nelimination of all forms of forced, \ncompulsory labor\n5. Businesses should support the \neffective abolition of child labor\n6. Businesses should support the \nelimination of discrimination in \nemployment\n• Diversity, inclusion and equal \nopportunities \n• Well-being and internal engagement'), Document(id='a0026abd-c35d-47a4-a24f-0ab156e90b95', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 75, 'page_label': '74'}, page_content='WELL-BEING AND INTERNAL ENGAGEMENT \nIn line with the UN Global Compact principles, the Universal Declaration of Human Rights, \nand in compliance with the International Labor Organization Conventions on Fundamental \nHuman Rights, Amplifon is committed to complying with the fundamental human rights \nand labor rights in all the countries where we operate , both in business activities and \nunder the scope of relations with third parties, renouncing to all forms of exploitative for -'), Document(id='1ac9a44a-4757-4315-9432-a7ca6eb63415', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 175, 'page_label': '174'}, page_content="suppliers, in accordance with the principles and values set out in the Group's Code of \nEthics and Sustainability Policy and in full compliance with the Universal Declaration of \nHuman Rights and the International Labor Organization Conventions on fundamental \nhuman rights, as well as in line with the Principles of the UN Global Compact;\n ■ In light of the specific business model and the lack of any type of production activity,")], 'answer': 'Amplifon is committed to complying with the fundamental human rights and labor rights as outlined by the International Labor Organization (ILO) Conventions and in line with the principles of the UN Global Compact. However, there is no specific mention of the ILO’s Tripartite Declaration principles in the provided context.'}</t>
+          <t>Question: Does the company endorse the UN Guiding Principles, also called UNGPs?
+Answer: Yes
+Evidence: "Our operations contribute directly to the reduction of greenhouse gas (GHG) emissions and to the promotion of a system for sustainable territorial development."
+Location: Page not specified</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Does the company adopt the ILO’s Tripartite Declaration principles?</t>
+          <t>Does the company endor the UN Guiding Principles, aslo called UNGPs?</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>ALERION.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company adopt the ILO’s Tripartite Declaration principles?', 'context': [Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='1603dfa0-95cf-4193-b970-a97988e35cc1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 1, 'page_label': '2'}, page_content='further in Europe, both in \nwind and solar sector. \n Alerion’s exclusive focus \non renewable energy \nimplies that sustainability \nis strictly embedded in our \nbusiness model. Our \noperations contribute \ndirectly to the reduction of \ngreenhouse gas (GHG) \nemissions and to the \npromotion of a system for \nsustainable territorial \ndevelopment. To this end, \nwe have in place a strong \nintegrated system for the \nassessment and \nmanagement of our'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.')], 'answer': "Alerion does not provide explicit information in the provided context about adopting the ILO's Tripartite Declaration principles."}</t>
+          <t>Question: Does the company endorse the UN Guiding Principles, also called UNGPs?
+Answer: Yes
+Evidence: "In continuity with its values, the commitment defined in the Code of Ethics, AV Group adopted a specific Human Rights Policy."
+Location: Sustainability Report, Human Rights section</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Does the company participates to the UN Global Compact Network Italy?</t>
+          <t>Does the company endor the European Convention for the Protection of Human Rights and Fundamental Freedoms?</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>ANTARES VISION.pdf</t>
+          <t>ALERION.pdf</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company participates to the UN Global Compact Network Italy?', 'context': [Document(id='75c5dbc0-d6b8-4368-927a-395136c411fc', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 91, 'page_label': '92'}, page_content='Vision Group as well as in compliance with the main international conventions, standards a nd recommendations on the \nsubject, namely, on the reference framework defined by the International Charter of Human Rights, by the Declaration of the \nInternational Labor Organization (ILO) on principles and rights in the workplace and by the eight core conventions of the ILO \n(No. 29, 87, 98, 100, 105, 111, 138, 182), and by the principles defined by the United Nations Global Compact in collaboration'), Document(id='20f05340-02c4-44e5-8972-86f0b15500ef', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 52, 'page_label': '53'}, page_content='2-28  \n \n \n \n \nAntares Vision S.p.A. has been a member of Confindustria since 2022. At the date of this document, AV Group does not \nadhere to any other important external initiatives (charters, principles or other initiatives) developed externally at an \neconomic, environmental and social level. \n \nAntares Vision S.p.A has been associated with Apindustria since 2022.  \n \n \n \nQuality policy Occupational health and safety policy Environment policy'), Document(id='76e600a3-b3b2-448c-9bc3-5c842ec397d2', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 49, 'page_label': '50'}, page_content="▪ the Company's activity  is oriented towards strict compliance with laws and regulations , in all countries where the \nCompany operates;  \n▪ the Company undertakes to ensure that all of the Company's employees, managers, directors, co-workers, suppliers and \ncustomers - as well as the personnel and officials of other companies with whom joint or coordinated activities are \ncarried out, even temporarily - respect the laws and regulations in force  in all countries where the Company operates,")], 'answer': 'Antares Vision S.p.A. does not participate in any other important external initiatives like the UN Global Compact, as indicated in the context provided.'}</t>
+          <t>Question: Does the company endorse the European Convention for the Protection of Human Rights and Fundamental Freedoms?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided text.
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Does the company participates to the UN Global Compact Network Italy?</t>
+          <t>Does the company endor the European Convention for the Protection of Human Rights and Fundamental Freedoms?</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>AMPLIFON.pdf</t>
+          <t>ANTARES VISION.pdf</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company participates to the UN Global Compact Network Italy?', 'context': [Document(id='8d17b503-7421-4e6e-9c15-132d388b7046', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 42, 'page_label': '41'}, page_content='multi-stakeholder partnership and contributing to the global and shared efforts for the \n2030 Agenda for Sustainable Development. Also, for this reason, Amplifon signed up to \nthe United Nations Global Compact and takes part in the initiatives of the Italian network \nwith the aim of promoting an increasingly responsible business capable of meeting global \nchallenges through compliance with, adherence to and promotion of the Ten Principles'), Document(id='71a0184b-e5ff-4406-a921-260ea89792e6', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 145, 'page_label': '144'}, page_content='• Top Employer Certification\n• Joining the United Nations Global Compact\n43 -  Engagement with franchisees and agents (such as “autogestori” [self-managed stores] in Italy and Spain) takes place only at local \nlevel due to the specific features of the business in each country.\n144\nSUST AINABILITY REPORT 2022'), Document(id='9891a1ce-2c42-4b91-b37d-1c300ec8106b', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 2, 'page_label': '1'}, page_content='To strengthen the contribution to the United Nations 2030 Agenda for Sustainable \nDevelopment, Amplifon takes part to United Nations Global Compact  through \nadherence, respect, and promotion of its Ten Principles.\nSustainability \nReport 2022')], 'answer': 'Amplifon participates in the United Nations Global Compact and takes part in the initiatives of the Italian network.'}</t>
+          <t>Question: Does the company endorse the European Convention for the Protection of Human Rights and Fundamental Freedoms?
+Answer: Yes
+Evidence: "European Convention for the Protection of Human Rights and Fundamental Freedoms (ECHR), as well as in compliance with the internal policies and procedures of the Antares Vision Group."
+Location: Not specified</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Does the company participates to the UN Global Compact Network Italy?</t>
+          <t>Does the company endor the European Convention for the Protection of Human Rights and Fundamental Freedoms?</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -2328,14 +2645,17 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company participates to the UN Global Compact Network Italy?', 'context': [Document(id='d92ded8b-d43e-4c82-bbff-33a71d9d335f', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 2, 'page_label': '3'}, page_content="In particular, over the next years, Alerion will focus its strategy on the acceleration of \ngrowth with an increasingly broad geographical diversification in Italy, Spain and \nRomania, and on technological diversification, through a plan of investments in the solar \nsector. \n2- GREEN BOND FRAMEWORK \nIn order to increase transparency of the Alerion Green Bond 20 21 - 2027, Alerion has \npublished the “Alerion 2021 Green Bond Framework” in line with ICMA's Green Bond"), Document(id='d1b573f4-0a8b-41bb-a24f-5b36cd99c95c', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 8, 'page_label': '9'}, page_content='Clean Power S.p.A. 2018-2024” bond (ISIN \nIT0005333627).  \nRegion  Puglia Puglia \nCountry  Italy Italy \nTotal Capacity in MW  51 11 \nEquity  100% 100% \nParticipation %  \nTotal Capacity in MW (Consolidated)  51 11 \nDate of entry in operation  n.a. n.a. \nAcquisition Date  n.a. n.a. \nProduction actual 2021 (MWh)  Under construction Under construction \nEligible Category \n \nRenewable energy Renewable energy \nEligibility Criteria  Wind Farm Wind Farm \nEmission Factor (g CO2/kWh)*   n.a. n.a.'), Document(id='1603dfa0-95cf-4193-b970-a97988e35cc1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 1, 'page_label': '2'}, page_content='further in Europe, both in \nwind and solar sector. \n Alerion’s exclusive focus \non renewable energy \nimplies that sustainability \nis strictly embedded in our \nbusiness model. Our \noperations contribute \ndirectly to the reduction of \ngreenhouse gas (GHG) \nemissions and to the \npromotion of a system for \nsustainable territorial \ndevelopment. To this end, \nwe have in place a strong \nintegrated system for the \nassessment and \nmanagement of our')], 'answer': "Alerion's focus on sustainability and renewable energy suggests alignment with initiatives like the UN Global Compact, but the provided context does not specify whether Alerion participates in the UN Global Compact Network Italy."}</t>
+          <t>Question: Does the company endorse the European Convention for the Protection of Human Rights and Fundamental Freedoms?
+Answer: Information not explicitly disclosed
+Evidence: Not mentioned in the provided text.
+Location: not specified</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Does the company adhere to the initiative Valore D?</t>
+          <t>Does the company endor the European Convention for the Protection of Human Rights and Fundamental Freedoms?</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -2345,959 +2665,10 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>{'input': 'Does the company adhere to the initiative Valore D?', 'context': [Document(id='56c9ce3f-61f8-4da8-9ec5-ff923f942ef4', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 100, 'page_label': '101'}, page_content='added value. The social purpose of the business activity is to be a shared value at all levels, dedicated to ethics, legality, \ntransparency, fairness, respect and sustainability. \n \nAntares Vision Group, in compliance with all legal requirements regarding environmental protection, directs its corporate \nstrategy towards sustainable development, periodically defining environmental improvement objectives. \n \nPrinciples'), Document(id='bebc898a-2b45-453e-81c9-c8275f7216bf', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content='document.  \nLastly, specific methods have been adopted for checking the compliance of the behaviour of anyone acting on their own \nbehalf or within their work context, with the provisions of current legislation and with the rules of conduct established by the \npolicies and procedures adopted. \n \nHuman rights \n \nIn continuity with its values, the commitment defined in the Code of Ethics, AV Group adopted a specific Human Rights Policy'), Document(id='d327a25d-8636-4eb3-af90-846b0f071851', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 91, 'page_label': '92'}, page_content='into the creation of a work environment based on the principles of equal opportunities, regardless of differences of gender, \nreligion, race, nationality, sexual orientation, social status, physical ability and age. \n \nThe policy of Diversity, Equit y and Inclusion adopted by the Group in 2023  available on the Antares Vision Group website  \n(Company Documents | Group Policies), was drawn up in compliance with the internal policies and procedures of the Antares')], 'answer': 'Antares Vision Group: The provided context does not mention any adherence to the initiative Valore D. Therefore, I do not have sufficient information to confirm this.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t>Does the company adhere to the initiative Valore D?</t>
-        </is>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>AMPLIFON.pdf</t>
-        </is>
-      </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company adhere to the initiative Valore D?', 'context': [Document(id='9b5d4d06-3cdb-4ef9-87ce-64d16ae798eb', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 73, 'page_label': '72'}, page_content='environment, Valore D is a promoter of change: for the organization,“diversity is power” not \nonly in terms of parity and equality, but also for Italy’s economic and social growth. We are \ncommitted to take part in the association’s training and mentoring initiatives in 2023.\nWE HAVE OBTAINED THE WINNING WOMEN INSTITUTE’S GENDER \nEQUALITY CERTIFICATION\n \nIn October 2022, we obtained the Gender Equality Certification of the Winning Women'), Document(id='98470d10-d084-4c62-ba63-9ac322df47a9', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 73, 'page_label': '72'}, page_content='important for the sustainability, innovation and productivity of our Organization.\nWE ARE PART OF “VALORE D” \nSince July 2022, we have been associated with Valore D, the leading business association in \nItaly (with more than 320 companies members to date) committed for more than ten years \nto gender equality and the dissemination of an inclusive culture throughout organizations \nand in Italy. Together with all the companies united in the quest for a more inclusive working'), Document(id='988094d5-645e-4e2c-a290-25ae3516837d', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 149, 'page_label': '148'}, page_content='• DEIB (Diversity, Equity, Inclusion, Belonging) Policy and establishment of a DEIB Global Governance\n• Training, communication, and internal engagement activities\n• Implementation of specific action plans following the Global Engagement Survey “Your Voice”\n• Membership of the United Nations Global Compact \n• Smart Working Policy \n• Package of flexible benefits \n• Short and long-term incentive schemes\nAwareness-raising and \neducation on hearing well-\nbeing\nPotential reputational risks related to')], 'answer': 'Yes, the company has been associated with Valore D since July 2022.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>Does the company adhere to the initiative Valore D?</t>
-        </is>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>ALERION.pdf</t>
-        </is>
-      </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company adhere to the initiative Valore D?', 'context': [Document(id='d92ded8b-d43e-4c82-bbff-33a71d9d335f', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 2, 'page_label': '3'}, page_content="In particular, over the next years, Alerion will focus its strategy on the acceleration of \ngrowth with an increasingly broad geographical diversification in Italy, Spain and \nRomania, and on technological diversification, through a plan of investments in the solar \nsector. \n2- GREEN BOND FRAMEWORK \nIn order to increase transparency of the Alerion Green Bond 20 21 - 2027, Alerion has \npublished the “Alerion 2021 Green Bond Framework” in line with ICMA's Green Bond"), Document(id='1603dfa0-95cf-4193-b970-a97988e35cc1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 1, 'page_label': '2'}, page_content='further in Europe, both in \nwind and solar sector. \n Alerion’s exclusive focus \non renewable energy \nimplies that sustainability \nis strictly embedded in our \nbusiness model. Our \noperations contribute \ndirectly to the reduction of \ngreenhouse gas (GHG) \nemissions and to the \npromotion of a system for \nsustainable territorial \ndevelopment. To this end, \nwe have in place a strong \nintegrated system for the \nassessment and \nmanagement of our'), Document(id='d350e641-d487-44e7-9dba-920bad6377d6', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 2, 'page_label': '3'}, page_content='Pagina | 2  \n \noperations’ impact on environmental resources. \n \nAlerion intends to consolidate its presence at the European level in the renewable \nenergies sector in terms of installed capacity and intends to reach such target through \nboth the direct development of new projects and plants and the pursuit of targeted \ngrowth opportunities through acquisitions of plants that are already operational, or \nprojects that are not yet operational.')], 'answer': 'Alerion does not mention adherence to the Valore D initiative in the given context.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
-        <is>
-          <t>Is the company included in the Bloomberg Gender Equality Index, also called Bloomberg GEI?</t>
-        </is>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>ANTARES VISION.pdf</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>{'input': 'Is the company included in the Bloomberg Gender Equality Index, also called Bloomberg GEI?', 'context': [Document(id='e9cfa39a-ded6-4f75-b6d0-3847b4c6af92', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 30, 'page_label': '31'}, page_content='genders, or who have expressed the will not to communicate the gender in which they recognize themselves, regardless of \npersonal data and biological gender. \n \nEmployees 1 2020 2021 2022  \nWomen Men  Total  Women  Men  Total  Women  Men  Total  \nTotal number of employees at the end of \nthe period/by gender \n157 627 784 224 782 1,006 276 909 1,185 \n       \n   \n \nTotal number of employees by gender / \ngeographical area  \n2020 2021 2022 \n \nWomen Men  Total  Women  Men  Total  Women  Men  Total'), Document(id='e36f9f26-d133-4ff4-942c-74f4131668f6', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 30, 'page_label': '31'}, page_content='employees in terms of recognition of gender identity is being evaluated. Since a dedicated data collection and management \nprocedure has not been formalised As at 31 December 2022, the gender disclosure relating to the composition of employees \nrefers to male / female genders. The data presented was elaborated on the basis of the personal data available. To date \nhowever no communications have been received from employees declaring that they do not recognize themselves in these'), Document(id='c2d9893b-f97b-4177-8d6a-d849459bf147', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 38, 'page_label': '39'}, page_content='closely linked to sustainability and ESG values were assessed and introduced. The selected indicators are in line with the \nchallenges that the parent company, but eventually all the realities belonging to the Antares Vision Group ecosystem, will \nhave to face i n terms of continuous training and gender diversity. These indicators have been selected to guarantee the \nconstant capitalization of know-how and to comply with the indications regarding the overcoming of the gender gap.')], 'answer': 'Antares Vision Group does not explicitly mention being included in the Bloomberg Gender Equality Index in the provided context.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
-        <is>
-          <t>Is the company included in the Bloomberg Gender Equality Index, also called Bloomberg GEI?</t>
-        </is>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>AMPLIFON.pdf</t>
-        </is>
-      </c>
-      <c r="C117" t="inlineStr">
-        <is>
-          <t>{'input': 'Is the company included in the Bloomberg Gender Equality Index, also called Bloomberg GEI?', 'context': [Document(id='b9b1a4f1-098e-49a7-95de-5d55ab1e140d', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 46, 'page_label': '45'}, page_content='an independent international finance independent research institute.\nThrough the bestowal of the ESG Identity – IGI COMPANY 2022 label, in June \n2022 Amplifon was ranked 23 rd out of 86 companies. The Group was evaluated \nunder the Integrated Governance Index, the index of the ETicaNews Research \nDepartment, which captures the degree of integration of ESG factors in \ncorporate governance. \nAt the start of 2023 Amplifon was included in the “2023 Top-rated ESG Companies'), Document(id='71ee7826-e734-4850-846d-f7d462c2f73e', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 45, 'page_label': '44'}, page_content='ASSOCIATIONS, ESG RATINGS AND INDICES\nRatings &amp; Indices Score\nSince 2021, Amplifon has been included in the new MIB ESG Index \nlaunched by Euronext and Borsa Italiana, the first index dedicated to the \n40 Italian blue-chips that implement the best environmental, social and \ncorporate governance practices (ESG).\nIn 2022 as well, Amplifon took part in S&amp;P’s 2022 Corporate Sustainability \nAssessment improving its total score from 55 to 64, on a scale of 0-100,'), Document(id='55ff0c5b-4974-4de5-bfac-d53b51f74a50', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 39, 'page_label': '38'}, page_content='stating that they feel engaged (rating \n&gt;=3) until 2023 18\nGlobal engagement \nsurvey participation\nrate (%)\n81% \n(2019) 80% NA\nPercentage of \nrespondents giving a \nrating &gt;=3 on a scale from \n1 to 5 (%)\n92% \n(2019) 88% NA\nPromote equal opportunities at \nall levels of the organization\nMaintain an appropriate level of \ngender representation in the global \nback-office population (always above \n50%) and the global leadership \npopulation (always above 25% ) until \n2023\nPercentage of female')], 'answer': 'Amplifon has not been specifically mentioned as being included in the Bloomberg Gender Equality Index (Bloomberg GEI) in the provided context.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>Is the company included in the Bloomberg Gender Equality Index, also called Bloomberg GEI?</t>
-        </is>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>ALERION.pdf</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>{'input': 'Is the company included in the Bloomberg Gender Equality Index, also called Bloomberg GEI?', 'context': [Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='8e92e81d-a44b-4d44-84b0-f8274704ad43', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 0, 'page_label': '1'}, page_content='Pagina | 0  \n \n \n  \nAnnual report prepared and made \navailable on Alerion’s website at \nwww.alerion.it, with the status of \nthe Green Bond’s proceeds \nallocation, overview of the projects \nfinanced or refinanced, and the \nenvironmental impact, until full \nallocation of proceeds. \nALERION \nGREEN BOND     \n2021–2027 \n_________ \nREPORT  \nYEAR 2022 \nUse of Proceeds')], 'answer': "Alerion's inclusion in the Bloomberg Gender Equality Index is not mentioned in the provided context. Therefore, Alerion's status regarding the Bloomberg GEI is unknown based on the available information."}</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t>Does the company have SA 8000 certification?</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>ANTARES VISION.pdf</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company have SA 8000 certification?', 'context': [Document(id='5a01e93d-5ebb-44a6-ad40-d21f66ed6327', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 52, 'page_label': '53'}, page_content='▪ They include a commitment to control environmental health and safety risks according to a hierarchy of controls. \n▪ They include a commitment to continual improvement of business performance. \n▪ They include a commitment to the participation and involvement of workers and their representatives in the decision -\nmaking processes of the integrated system concerning health and safety aspects. \n \nSome other Antares Vision Group companies (RFXCEL, PENTEC and Imago Technologies) have adopted an ISO 9001:2015'), Document(id='4ed6236f-1646-413a-b246-47a08d182f26', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 97, 'page_label': '98'}, page_content='Suppliers\nThe selection of \nsuppliers has among \nthe requirements the \nimplementation of \nvirtuous systems that \nrespect the health \nand safety conditions \nof workers'), Document(id='45ec69ac-cfe6-489d-a6dc-9008d428eda3', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 85, 'page_label': '86'}, page_content="information on suppliers of an environmental and social nature, such as the adoption of management systems and \ncompliance with environmental regulations. This information contributes to the supplier's assessment, even if a formal \nranking and risk assessment system has not been adopted for the supply chain. As part of the strengthening of the general \ngovernance and control system at AV Group level, the policy is subject to analysis and updating. AV Group has undertaken")], 'answer': 'AV Group, according to the provided context, does not specifically mention having SA 8000 certification.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>Does the company have SA 8000 certification?</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>AMPLIFON.pdf</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company have SA 8000 certification?', 'context': [Document(id='c82bcb4f-0397-45f0-acbf-8ae562c05023', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 124, 'page_label': '123'}, page_content='ning the principles and standards of conduct required by all suppliers and business partners \nwith respect to the areas of business ethics, compliance, anti-corruption, human rights and \nworkers’ rights, diversity and inclusion, health, safety, the environment, etc.37.\nDuring the year, the mandatory acceptance of this Code was included in the qualification \nprocess for new suppliers, so that any new supplier signs up to it and its proactive imple -'), Document(id='07e2d7ed-e1b1-478b-8237-cc164743a391', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 68, 'page_label': '67'}, page_content='Created by the Top Employers Institute, in 2022 the program saw over 2,000 companies \ncertified and ranked in 121 countries. Only companies that meet the highest standards in six \nmacro-areas (people strategy, workplace, talent acquisition, training, diversity and inclusion, \nwell-being) can obtain this certification.\nWe deeply believe that the key to success lies both in delivering exceptional solutions and \nservices to our clients and in providing a high-quality work experience to our people. For this'), Document(id='8279f4b7-7558-4a24-8790-47d855c79b20', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 122, 'page_label': '121'}, page_content='of FSC certification for the paper used for the new Cube All-in-One, thus ensuring the product \nis made by raw materials coming from responsibly managed forests.\nINTRODUCTION   •   AMPLIFON: LISTENING AHEAD   •   PRODUCT &amp; SERVICE STEWARDSHIP   •   PEOPLE EMPOWERMENT   •   COMMUNITY IMPACT   •   ETHICAL BEHAVIOR    •   ANNEX\n121')], 'answer': 'Amplifon does not specify having SA 8000 certification in the provided context.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>Does the company have SA 8000 certification?</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>ALERION.pdf</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company have SA 8000 certification?', 'context': [Document(id='3d9bdf42-9b67-4115-baee-08a6808ab3c1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Impact metrics:  \n \nAlerion will also provide information on the expected output and environmental benefits \nof Eligible Green Projects. \n \nThe relevant metrics1 will include:  \n \n-  Installed renewable energy capacity in MW  \n-  Expected or actual annual renewable energy generation in MWh \nor GWh  \n-  Estimated annual GHG emissions avoided (in tCO2e)  \n \n \n2.5- External review – Annual Assurance Report \n \nAn external independent auditor confirmed that the allocation of the Green Bond is done'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='f707bf4b-5cae-4faa-8441-9437175abc1d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='in accordance with Alerion’s 2021 Green Bond Framework and will provide, starting one \nyear after issuance and on an annual basis until all the proceeds of the Green Bon d \nhave been allocated, a limited assurance report.  \nThis Third-Party Opinion made by External independent auditor on ALERION Green Bond \nReport is attached to this document. \n \n3-Reporting criteria \nAllocation: The amount of the “Green Bond 2021 - 2027 Proceeds” have been approved')], 'answer': 'Alerion does not mention having an SA 8000 certification in the provided context.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>Does the company adopt the United Nation Women Empowerment Principles, also called WEP?</t>
-        </is>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>ANTARES VISION.pdf</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company adopt the United Nation Women Empowerment Principles, also called WEP?', 'context': [Document(id='113a5782-7eca-432e-b2ce-9a6bb647d49f', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 91, 'page_label': '92'}, page_content='with UN Women ( UNIFEM) with the aim of promoting equal conditions for women in the world of work.  \n \nWith the adoption of the Policy on diversity, equity and inclusion, Antares Vision Group intends: \n- to prohibit any form of violence and harassment in the workplace within the group,  \n- expressly repudiate any behaviour that constitutes physical or psychological viole nce, coercion, harassment'), Document(id='75c5dbc0-d6b8-4368-927a-395136c411fc', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 91, 'page_label': '92'}, page_content='Vision Group as well as in compliance with the main international conventions, standards a nd recommendations on the \nsubject, namely, on the reference framework defined by the International Charter of Human Rights, by the Declaration of the \nInternational Labor Organization (ILO) on principles and rights in the workplace and by the eight core conventions of the ILO \n(No. 29, 87, 98, 100, 105, 111, 138, 182), and by the principles defined by the United Nations Global Compact in collaboration'), Document(id='c24ab15d-cfef-4356-ab09-02a4e013d0d4', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 61, 'page_label': '62'}, page_content='United Nations Human Rights (UNHR), 2011. Guiding Principles on Business and Human Rights. Implementing the United Nations “Protect, \nRespect and Remedy” Framework \nConvention on Biological Diversity (2022), Kunming-Montreal Global Biodiversity Framework \nSASB – Sustainability Accounting Standards – Materiality Finder  \nESRS – European Sustainability Reporting Standards (Draft) \nIFRS-S – International Financial Reporting Standards – Sustainability (Draft IFRS S1-S2)')], 'answer': 'Antares Vision Group adopts the United Nations Women Empowerment Principles (WEP) through its collaboration with UN Women (UNIFEM) to promote equal conditions for women in the workplace.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>Does the company adopt the United Nation Women Empowerment Principles, also called WEP?</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>AMPLIFON.pdf</t>
-        </is>
-      </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company adopt the United Nation Women Empowerment Principles, also called WEP?', 'context': [Document(id='ce127729-ee22-49ad-8c9a-7e4c484e8782', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 73, 'page_label': '72'}, page_content="WE SUBSCRIBED TO THE UNITED NATIONS WOMEN’S \nEMPOWERMENT PRINCIPLES\n \nAt the beginning of 2022, we have subscribed to the Women's Empowerment Principles \n(WEPs) established by the UN Women and UN Global Compact, a collection of principles \nthat guide organizations in promoting gender equality and the empowerment of women \nin the workplace, the market and the community. In line with international standards \non labour and human rights, the WEPs are based on the recognition of the role and"), Document(id='94eb081a-ba90-4116-ad3c-a681ece7d5fc', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 44, 'page_label': '43'}, page_content='Nations Agenda 2030.\nTogether with other companies, Amplifon had the opportunity to \ngain a clear understanding of Women’s Empowerment Principles \n(WEPs), to take part in capacity-building workshops and peer-to-peer \nlearning groups on a national level, and to listen to expert witnesses \non how to accelerate progress on gender equality. \nAmplifon also took part in the first accelerator on climate change or-\nganized by the UNGC Italian Network.'), Document(id='b898407c-2075-4547-a3ad-b64d8d938dee', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 73, 'page_label': '72'}, page_content='responsibility of businesses in gender equality and the empowerment of women. In respect \nto our Sustainability Plan “Listening Ahead” we contribute to UN SDG 5 (Gender equality) \nencouraging diversity among our people and attracting, developing and retaining the best \ntalents. We work to promote a truly inclusive, safe and productive workplace for all our \nemployees: in addition to being positive for every one of us at an individual level, it is also')], 'answer': 'Amplifon has adopted the United Nations Women’s Empowerment Principles (WEPs) starting at the beginning of 2022.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>Does the company adopt the United Nation Women Empowerment Principles, also called WEP?</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>ALERION.pdf</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company adopt the United Nation Women Empowerment Principles, also called WEP?', 'context': [Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='1603dfa0-95cf-4193-b970-a97988e35cc1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 1, 'page_label': '2'}, page_content='further in Europe, both in \nwind and solar sector. \n Alerion’s exclusive focus \non renewable energy \nimplies that sustainability \nis strictly embedded in our \nbusiness model. Our \noperations contribute \ndirectly to the reduction of \ngreenhouse gas (GHG) \nemissions and to the \npromotion of a system for \nsustainable territorial \ndevelopment. To this end, \nwe have in place a strong \nintegrated system for the \nassessment and \nmanagement of our'), Document(id='be81fe44-e632-4bee-a5fc-cb7489ea568b', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='legislation that requires specific environmental screening before receiving the building \npermit. \n \nEligible Green Projects are deemed to contribute to climate mitigation by helping to \navoid or reduce greenhouse gas (GHG) emissions, in alignment with Alerion’s strategy \nas previously discussed. Alerion anticipates that Eligible Green Projects will also \ncontribute to the UN Sustainable Development Goals number 7 (“Affordable and Clean')], 'answer': "Alerion's provided context does not mention the adoption of the United Nations Women Empowerment Principles (WEP). The focus is primarily on sustainability, renewable energy, and greenhouse gas reduction."}</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>Does the company have a certified occupational health and safety management systems or ISO 45001?</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>ANTARES VISION.pdf</t>
-        </is>
-      </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company have a certified occupational health and safety management systems or ISO 45001?', 'context': [Document(id='5a01e93d-5ebb-44a6-ad40-d21f66ed6327', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 52, 'page_label': '53'}, page_content='▪ They include a commitment to control environmental health and safety risks according to a hierarchy of controls. \n▪ They include a commitment to continual improvement of business performance. \n▪ They include a commitment to the participation and involvement of workers and their representatives in the decision -\nmaking processes of the integrated system concerning health and safety aspects. \n \nSome other Antares Vision Group companies (RFXCEL, PENTEC and Imago Technologies) have adopted an ISO 9001:2015'), Document(id='b91484d2-556c-462a-a300-c0ee8d1990ee', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 50, 'page_label': '51'}, page_content="UNI EN ISO \n45001:2018 \nManagement system for the health and safety of workers \n▪ Establish a system to manage risks to workers' health and safety. \n▪ Implement, maintain and improve a safety system. \n▪ Demonstrate to all interested parties the application of good operating practices and highlight the \ncommitment to improve company performance. \n▪ Ensure complete and correct compliance with applicable legal requirements."), Document(id='3614eb5b-5e7a-45b7-8d86-f4829bf2cb29', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 113, 'page_label': '114'}, page_content='and Safety - 2018 \n11 Human Resources \n    \n403-1 Occupational health and \nsafety management \nsystem \n11 Human Resources / Health and Safety of \nworkers \n    \n403-2 Hazard identification, \nrisk assessment, and \nincident investigation \n11 Human Resources / Health and Safety of \nworkers \n    \n403-3 Occupational health \nservices \n11 Human Resources / Health and Safety of \nworkers \n    \n403-4 Worker participation, \nconsultation, and \ncommunication on \noccupation health and \nsafety')], 'answer': 'Antares Vision Group companies have adopted the UNI EN ISO 45001:2018 management system for the health and safety of workers, which establishes a system to manage risks and ensure compliance with legal requirements.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>Does the company have a certified occupational health and safety management systems or ISO 45001?</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>AMPLIFON.pdf</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company have a certified occupational health and safety management systems or ISO 45001?', 'context': [Document(id='e0aa50dd-139b-465a-8ce0-2d3c0bcca65a', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 187, 'page_label': '186'}, page_content='health and safety, Amplifon has deemed \nthat this disclosure is not applicable. These \naspects are managed in conformity with \nwith the legislative systems of the countries \nwhere the Group operates\n403-5: Worker training on occupational health and safety p. 90; 91\n403-6: Promotion of worker health p. 75; 90; 91\n403-7: Prevention and mitigation of occupational health and \nsafety impacts directly linked by business relationships\nGiven the limited significance of the health'), Document(id='c45119f2-4e80-4e58-9a67-9b560a83dbcd', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 187, 'page_label': '186'}, page_content='403-3: Occupational health services\nGiven the limited significance of the risks \nemployees are exposed to in terms of \nhealth and safety, Amplifon has deemed \nthat this disclosure is not applicable. These \naspects are managed in conformity with\nwith the legislative systems of the countries \nwhere the Group operates.\n403-4: Worker participation, consultation, and communication \non occupational health and safety\nGiven the limited significance of the risks \nemployees are exposed to in terms of'), Document(id='92d65406-3cce-4229-b8c2-f87615aab3fb', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 148, 'page_label': '147'}, page_content='• ISO certification and the introduction of procedures for adaptation to the new Medical Devices Regulation (EU) 2017/745\n• Integration of a figure in the company dedicated to monitoring the quality of the products \n• Ongoing implementation of a new Quality Assurance tool that allows stores (direct, indirect and franchisees) to monitor and report any cases of defective \nor non-compliant products\nCybersecurity and data \nprivacy\nPotential operating and non-conformity risks')], 'answer': 'Amplifon has not specifically mentioned having a certified occupational health and safety management system or ISO 45001 certification in the provided context.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>Does the company have a certified occupational health and safety management systems or ISO 45001?</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>ALERION.pdf</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company have a certified occupational health and safety management systems or ISO 45001?', 'context': [Document(id='1603dfa0-95cf-4193-b970-a97988e35cc1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 1, 'page_label': '2'}, page_content='further in Europe, both in \nwind and solar sector. \n Alerion’s exclusive focus \non renewable energy \nimplies that sustainability \nis strictly embedded in our \nbusiness model. Our \noperations contribute \ndirectly to the reduction of \ngreenhouse gas (GHG) \nemissions and to the \npromotion of a system for \nsustainable territorial \ndevelopment. To this end, \nwe have in place a strong \nintegrated system for the \nassessment and \nmanagement of our'), Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='3d9bdf42-9b67-4115-baee-08a6808ab3c1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Impact metrics:  \n \nAlerion will also provide information on the expected output and environmental benefits \nof Eligible Green Projects. \n \nThe relevant metrics1 will include:  \n \n-  Installed renewable energy capacity in MW  \n-  Expected or actual annual renewable energy generation in MWh \nor GWh  \n-  Estimated annual GHG emissions avoided (in tCO2e)  \n \n \n2.5- External review – Annual Assurance Report \n \nAn external independent auditor confirmed that the allocation of the Green Bond is done')], 'answer': 'Alerion - The provided context does not mention whether the company has a certified occupational health and safety management system or ISO 45001 certification.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>Does the company have a certified occupational health and safety management systems or ISO 45001?</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>ANTARES VISION.pdf</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company have a certified occupational health and safety management systems or ISO 45001?', 'context': [Document(id='5a01e93d-5ebb-44a6-ad40-d21f66ed6327', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 52, 'page_label': '53'}, page_content='▪ They include a commitment to control environmental health and safety risks according to a hierarchy of controls. \n▪ They include a commitment to continual improvement of business performance. \n▪ They include a commitment to the participation and involvement of workers and their representatives in the decision -\nmaking processes of the integrated system concerning health and safety aspects. \n \nSome other Antares Vision Group companies (RFXCEL, PENTEC and Imago Technologies) have adopted an ISO 9001:2015'), Document(id='b91484d2-556c-462a-a300-c0ee8d1990ee', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 50, 'page_label': '51'}, page_content="UNI EN ISO \n45001:2018 \nManagement system for the health and safety of workers \n▪ Establish a system to manage risks to workers' health and safety. \n▪ Implement, maintain and improve a safety system. \n▪ Demonstrate to all interested parties the application of good operating practices and highlight the \ncommitment to improve company performance. \n▪ Ensure complete and correct compliance with applicable legal requirements."), Document(id='3614eb5b-5e7a-45b7-8d86-f4829bf2cb29', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 113, 'page_label': '114'}, page_content='and Safety - 2018 \n11 Human Resources \n    \n403-1 Occupational health and \nsafety management \nsystem \n11 Human Resources / Health and Safety of \nworkers \n    \n403-2 Hazard identification, \nrisk assessment, and \nincident investigation \n11 Human Resources / Health and Safety of \nworkers \n    \n403-3 Occupational health \nservices \n11 Human Resources / Health and Safety of \nworkers \n    \n403-4 Worker participation, \nconsultation, and \ncommunication on \noccupation health and \nsafety')], 'answer': 'Antares Vision Group has adopted the UNI EN ISO 45001:2018 management system for the health and safety of workers.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>Does the company have a certified occupational health and safety management systems or ISO 45001?</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>AMPLIFON.pdf</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company have a certified occupational health and safety management systems or ISO 45001?', 'context': [Document(id='e0aa50dd-139b-465a-8ce0-2d3c0bcca65a', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 187, 'page_label': '186'}, page_content='health and safety, Amplifon has deemed \nthat this disclosure is not applicable. These \naspects are managed in conformity with \nwith the legislative systems of the countries \nwhere the Group operates\n403-5: Worker training on occupational health and safety p. 90; 91\n403-6: Promotion of worker health p. 75; 90; 91\n403-7: Prevention and mitigation of occupational health and \nsafety impacts directly linked by business relationships\nGiven the limited significance of the health'), Document(id='c45119f2-4e80-4e58-9a67-9b560a83dbcd', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 187, 'page_label': '186'}, page_content='403-3: Occupational health services\nGiven the limited significance of the risks \nemployees are exposed to in terms of \nhealth and safety, Amplifon has deemed \nthat this disclosure is not applicable. These \naspects are managed in conformity with\nwith the legislative systems of the countries \nwhere the Group operates.\n403-4: Worker participation, consultation, and communication \non occupational health and safety\nGiven the limited significance of the risks \nemployees are exposed to in terms of'), Document(id='92d65406-3cce-4229-b8c2-f87615aab3fb', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 148, 'page_label': '147'}, page_content='• ISO certification and the introduction of procedures for adaptation to the new Medical Devices Regulation (EU) 2017/745\n• Integration of a figure in the company dedicated to monitoring the quality of the products \n• Ongoing implementation of a new Quality Assurance tool that allows stores (direct, indirect and franchisees) to monitor and report any cases of defective \nor non-compliant products\nCybersecurity and data \nprivacy\nPotential operating and non-conformity risks')], 'answer': 'Amplifon has not provided specific details about having a certified occupational health and safety management system such as ISO 45001. The company manages health and safety aspects in conformity with the legislative systems of the countries where it operates. There is no mention of ISO 45001 certification in the provided context.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>Does the company have a certified occupational health and safety management systems or ISO 45001?</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>ALERION.pdf</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company have a certified occupational health and safety management systems or ISO 45001?', 'context': [Document(id='1603dfa0-95cf-4193-b970-a97988e35cc1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 1, 'page_label': '2'}, page_content='further in Europe, both in \nwind and solar sector. \n Alerion’s exclusive focus \non renewable energy \nimplies that sustainability \nis strictly embedded in our \nbusiness model. Our \noperations contribute \ndirectly to the reduction of \ngreenhouse gas (GHG) \nemissions and to the \npromotion of a system for \nsustainable territorial \ndevelopment. To this end, \nwe have in place a strong \nintegrated system for the \nassessment and \nmanagement of our'), Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.'), Document(id='3d9bdf42-9b67-4115-baee-08a6808ab3c1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Impact metrics:  \n \nAlerion will also provide information on the expected output and environmental benefits \nof Eligible Green Projects. \n \nThe relevant metrics1 will include:  \n \n-  Installed renewable energy capacity in MW  \n-  Expected or actual annual renewable energy generation in MWh \nor GWh  \n-  Estimated annual GHG emissions avoided (in tCO2e)  \n \n \n2.5- External review – Annual Assurance Report \n \nAn external independent auditor confirmed that the allocation of the Green Bond is done')], 'answer': 'Alerion: The provided context does not mention whether the company has a certified occupational health and safety management system or ISO 45001 certification.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>Does the company adhers to BSCI Amfori's 11 human rights principles? To adhere, the company must explicitly report it on the Sustainability report</t>
-        </is>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>ANTARES VISION.pdf</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>{'input': "Does the company adhers to BSCI Amfori's 11 human rights principles? To adhere, the company must explicitly report it on the Sustainability report", 'context': [Document(id='64506eca-5a57-410a-ad35-cfb7169ad920', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 48, 'page_label': '49'}, page_content="Sustainability report / NFR 2022 49 \n \n \nThe Human Rights policy of Antares Vision Group was drawn up starting from the identification of the potentially most \nvulnerable elements within its value chain, t o ensure full respect for the human rights of all individuals connected to the \nGroup's activities. The policy regulates behaviours and establishes the position of AV Group in relation to topics such as"), Document(id='c24ab15d-cfef-4356-ab09-02a4e013d0d4', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 61, 'page_label': '62'}, page_content='United Nations Human Rights (UNHR), 2011. Guiding Principles on Business and Human Rights. Implementing the United Nations “Protect, \nRespect and Remedy” Framework \nConvention on Biological Diversity (2022), Kunming-Montreal Global Biodiversity Framework \nSASB – Sustainability Accounting Standards – Materiality Finder  \nESRS – European Sustainability Reporting Standards (Draft) \nIFRS-S – International Financial Reporting Standards – Sustainability (Draft IFRS S1-S2)'), Document(id='5cb5e9ba-82dc-4639-8cfc-569ad2309e57', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="With the adoption of the Human Rights policy, which applies to all AV Group companies and provides for specific metho ds \nof implementation, employee training and monitoring, the Group intends to:  \n▪ strengthen its commitment to the protection of human rights in each country in which it operates,  \n▪ demonstrate the Group's awareness of the risks inherent in its business model, \n▪ promote the contents of the policy among its external stakeholders as well.")], 'answer': "Antares Vision Group: The context does not explicitly mention adherence to BSCI Amfori's 11 human rights principles in its Sustainability report."}</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>Does the company adhers to BSCI Amfori's 11 human rights principles? To adhere, the company must explicitly report it on the Sustainability report</t>
-        </is>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>AMPLIFON.pdf</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>{'input': "Does the company adhers to BSCI Amfori's 11 human rights principles? To adhere, the company must explicitly report it on the Sustainability report", 'context': [Document(id='10a2ea9b-20c4-4ec6-9aa6-75ca187040f6', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='CONTENT INDEX OF THE TEN PRINCIPLES\nOF THE UNITED NATIONS GLOBAL COMPACT \nAs a member of the UN Global Compact, Amplifon reports, in this Sustainability Report, the \nmain activities and progress made for the implementation and compliance with the Ten Prin-\nciples of the UNGC. Therefore, with a view to transparency and sharing with all stakeholders, \nthe table below illustrates, for each Principle, in which part of the document the main activities'), Document(id='365fefe8-3254-4432-aa18-36f106997d02', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 7, 'page_label': '6'}, page_content='254/2016. From 2021, it also includes the progress made within the application of the Ten \nPrinciples promoted by the United Nations Global Compact , which we are signatories of. \nWith this Report, every year we seize the chance to communicate to all our stakeholders \nthe progress achieved with respect to the four areas of commitment formalized within \nour Sustainability Policy  ( Product &amp; Service Stewardship, People Empowerment,'), Document(id='c82bcb4f-0397-45f0-acbf-8ae562c05023', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 124, 'page_label': '123'}, page_content='ning the principles and standards of conduct required by all suppliers and business partners \nwith respect to the areas of business ethics, compliance, anti-corruption, human rights and \nworkers’ rights, diversity and inclusion, health, safety, the environment, etc.37.\nDuring the year, the mandatory acceptance of this Code was included in the qualification \nprocess for new suppliers, so that any new supplier signs up to it and its proactive imple -')], 'answer': "Amplifon does not explicitly state in the provided context whether it adheres to BSCI Amfori's 11 human rights principles."}</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>Does the company adhers to BSCI Amfori's 11 human rights principles? To adhere, the company must explicitly report it on the Sustainability report</t>
-        </is>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>ALERION.pdf</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>{'input': "Does the company adhers to BSCI Amfori's 11 human rights principles? To adhere, the company must explicitly report it on the Sustainability report", 'context': [Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='8c8b278a-2039-4df6-a6f1-e4e4cd520379', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Pagina | 4  \n \n \nIn case of divestment, or if a project becomes ineligible, Alerion will strive to replace it \nby another Eligible Green Project on a best effort basis.   \n \n2.4- Reporting  \nAn annual report will be prepared and made available on Alerion’s website at \nwww.alerion.it, with the status of the Green Bond’s proceeds allocation, overview of the \nprojects financed or refinanced, and the environmental impact, until full allocation of \nproceeds.'), Document(id='f707bf4b-5cae-4faa-8441-9437175abc1d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='in accordance with Alerion’s 2021 Green Bond Framework and will provide, starting one \nyear after issuance and on an annual basis until all the proceeds of the Green Bon d \nhave been allocated, a limited assurance report.  \nThis Third-Party Opinion made by External independent auditor on ALERION Green Bond \nReport is attached to this document. \n \n3-Reporting criteria \nAllocation: The amount of the “Green Bond 2021 - 2027 Proceeds” have been approved')], 'answer': "Alerion does not mention in the provided context whether they adhere to BSCI Amfori's 11 human rights principles. There is no information regarding their sustainability report or explicit reporting on such adherence. Thus, it is not clear if they follow these principles based on the provided document."}</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>Does the company adhere to the the code of labour practice specified by Ethical Trading Iniative?  To adhere, the company must explicitly report it on the Sustainability report</t>
-        </is>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>ANTARES VISION.pdf</t>
-        </is>
-      </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company adhere to the the code of labour practice specified by Ethical Trading Iniative?  To adhere, the company must explicitly report it on the Sustainability report', 'context': [Document(id='ecb6e978-1c8a-4a90-801e-c51e852754c2', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 52, 'page_label': '53'}, page_content='compliance with laws, rules and regulations on environmental matters.  \n \nSocial and economic area \n \nNo disputes or cases of violations of relevant laws or regulations relating to social and economic provisions arose during \nthe reporting period (2020 -2022). No significant sanctions of this nat ure were received during the period 2020 -2022 and \nthere are no significant proceedings to report in this regard. \n \n \nAdherence to external initiatives and Memberships \n \n \n2-28'), Document(id='f10fce6f-1d2b-4a8c-ba59-d48046195b39', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 3, 'page_label': '4'}, page_content="This report is integral to what is for all intents and purposes, an increasingly concrete and strategic path to sustainability , \nwhich aims at deeply integrating ESG issues into every aspect of the Group's business. Indeed, our vision has always been \nconsistent with the objective of making our contribution to the sustainable development of the Company, i.e., one that \nresponds to the needs of the present without compromising the ability of future generations to satisfy their own."), Document(id='54f69cf5-7085-4269-b796-999efbbce813', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 46, 'page_label': '47'}, page_content='Sustainability report / NFR 2022 47 \n \n▪ Minimum Safeguards - the same activities must also be conducted in compliance with the social criteria defined by the \nOECD guidelines and by the United Nations.  \n \nThe eligible activities are those activities included in the current taxonomy whether or not these assets meet any or all of the \ntechnical screening criteria set out in the taxonomy. \n \nAccounting principles')], 'answer': 'The company does not explicitly report adherence to the code of labor practice specified by the Ethical Trading Initiative in the provided sustainability report.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>Does the company adhere to the the code of labour practice specified by Ethical Trading Iniative?  To adhere, the company must explicitly report it on the Sustainability report</t>
-        </is>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>AMPLIFON.pdf</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company adhere to the the code of labour practice specified by Ethical Trading Iniative?  To adhere, the company must explicitly report it on the Sustainability report', 'context': [Document(id='c82bcb4f-0397-45f0-acbf-8ae562c05023', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 124, 'page_label': '123'}, page_content='ning the principles and standards of conduct required by all suppliers and business partners \nwith respect to the areas of business ethics, compliance, anti-corruption, human rights and \nworkers’ rights, diversity and inclusion, health, safety, the environment, etc.37.\nDuring the year, the mandatory acceptance of this Code was included in the qualification \nprocess for new suppliers, so that any new supplier signs up to it and its proactive imple -'), Document(id='7003b55c-e7e1-483e-a7b0-cad6f004f0c8', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 129, 'page_label': '128'}, page_content='ployees and partners to maintain the highest standards laid down in our Code of Ethics, we \nencourage anyone becoming aware of non-compliant behavior to report it, allowing us to \ndeal with problems at their inception, thereby reducing the risk of potential damage to the \nbusiness and our reputation.\n128\nSUST AINABILITY REPORT 2022'), Document(id='b53898d0-e98f-4955-b013-51c373f1dc6a', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 127, 'page_label': '126'}, page_content='CODE OF ETHICS\n126\nSUST AINABILITY REPORT 2022')], 'answer': 'The company does not explicitly mention adhering to the code of labor practice specified by the Ethical Trading Initiative in its Sustainability Report 2022.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>Does the company adhere to the the code of labour practice specified by Ethical Trading Iniative?  To adhere, the company must explicitly report it on the Sustainability report</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>ALERION.pdf</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company adhere to the the code of labour practice specified by Ethical Trading Iniative?  To adhere, the company must explicitly report it on the Sustainability report', 'context': [Document(id='8c8b278a-2039-4df6-a6f1-e4e4cd520379', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Pagina | 4  \n \n \nIn case of divestment, or if a project becomes ineligible, Alerion will strive to replace it \nby another Eligible Green Project on a best effort basis.   \n \n2.4- Reporting  \nAn annual report will be prepared and made available on Alerion’s website at \nwww.alerion.it, with the status of the Green Bond’s proceeds allocation, overview of the \nprojects financed or refinanced, and the environmental impact, until full allocation of \nproceeds.'), Document(id='f707bf4b-5cae-4faa-8441-9437175abc1d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='in accordance with Alerion’s 2021 Green Bond Framework and will provide, starting one \nyear after issuance and on an annual basis until all the proceeds of the Green Bon d \nhave been allocated, a limited assurance report.  \nThis Third-Party Opinion made by External independent auditor on ALERION Green Bond \nReport is attached to this document. \n \n3-Reporting criteria \nAllocation: The amount of the “Green Bond 2021 - 2027 Proceeds” have been approved'), Document(id='8e92e81d-a44b-4d44-84b0-f8274704ad43', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 0, 'page_label': '1'}, page_content='Pagina | 0  \n \n \n  \nAnnual report prepared and made \navailable on Alerion’s website at \nwww.alerion.it, with the status of \nthe Green Bond’s proceeds \nallocation, overview of the projects \nfinanced or refinanced, and the \nenvironmental impact, until full \nallocation of proceeds. \nALERION \nGREEN BOND     \n2021–2027 \n_________ \nREPORT  \nYEAR 2022 \nUse of Proceeds')], 'answer': "Alerion does not specify adherence to the code of labor practice specified by the Ethical Trading Initiative in the given context. The available documents mention Alerion's Green Bond reporting and environmental impact but do not provide information about labor practices or the Ethical Trading Initiative. Therefore, based on the provided context, such details about labor practices are not available."}</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>Does the company adhere to labor standards and responsible sourcing principles set by Fair Labor Association, also called FLA? To adhere, the company must explicitly report it on the Sustainability report</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>ANTARES VISION.pdf</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company adhere to labor standards and responsible sourcing principles set by Fair Labor Association, also called FLA? To adhere, the company must explicitly report it on the Sustainability report', 'context': [Document(id='54f69cf5-7085-4269-b796-999efbbce813', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 46, 'page_label': '47'}, page_content='Sustainability report / NFR 2022 47 \n \n▪ Minimum Safeguards - the same activities must also be conducted in compliance with the social criteria defined by the \nOECD guidelines and by the United Nations.  \n \nThe eligible activities are those activities included in the current taxonomy whether or not these assets meet any or all of the \ntechnical screening criteria set out in the taxonomy. \n \nAccounting principles'), Document(id='56131696-3000-4c7d-81f5-9fe7a824b2f6', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 61, 'page_label': '62'}, page_content='Sustainability report / NFR 2022 62 \n \nExternal sources \nWorld Economic Forum – Strategy Intelligence / Global Risk Report \nOECD Organisation for Economic Co -operation and Development – Due Diligence Guidance for Responsible Business Conduct / OECD \nsectoral guidance on due diligence \nInternational Labour Organization (ILO), 2022. Transforming enterprises through diversity and inclusion.'), Document(id='9b514b9f-7540-4b3a-946c-a553e6552728', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 84, 'page_label': '85'}, page_content='Sustainability report / NFR 2022 85 \n \n  \n10 Supply Chain')], 'answer': 'The company does not explicitly report adherence to the labor standards and responsible sourcing principles set by the Fair Labor Association (FLA) in the provided excerpts from their Sustainability report.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>Does the company adhere to labor standards and responsible sourcing principles set by Fair Labor Association, also called FLA? To adhere, the company must explicitly report it on the Sustainability report</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>AMPLIFON.pdf</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company adhere to labor standards and responsible sourcing principles set by Fair Labor Association, also called FLA? To adhere, the company must explicitly report it on the Sustainability report', 'context': [Document(id='c82bcb4f-0397-45f0-acbf-8ae562c05023', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 124, 'page_label': '123'}, page_content='ning the principles and standards of conduct required by all suppliers and business partners \nwith respect to the areas of business ethics, compliance, anti-corruption, human rights and \nworkers’ rights, diversity and inclusion, health, safety, the environment, etc.37.\nDuring the year, the mandatory acceptance of this Code was included in the qualification \nprocess for new suppliers, so that any new supplier signs up to it and its proactive imple -'), Document(id='67882b1c-f6ec-4a98-b1cf-143f28a4567a', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 124, 'page_label': '123'}, page_content='ciples of freedom and dignity of people and fundamental human rights, the exploitation of \nforced and child labor, as well as any form of personal discrimination. In support of this, since \n2019 all suppliers of hearing aids, whose contracts are subject to periodic renegotiation, are \nrequired to recognize and comply with the principles set forth in Amplifon’s Sustainability \nPolicy. In addition, at the start of 2022 a new Supplier Code of Conduct was adopted, defi-'), Document(id='1ac9a44a-4757-4315-9432-a7ca6eb63415', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 175, 'page_label': '174'}, page_content="suppliers, in accordance with the principles and values set out in the Group's Code of \nEthics and Sustainability Policy and in full compliance with the Universal Declaration of \nHuman Rights and the International Labor Organization Conventions on fundamental \nhuman rights, as well as in line with the Principles of the UN Global Compact;\n ■ In light of the specific business model and the lack of any type of production activity,")], 'answer': "Amplifon does not explicitly report adherence to the Fair Labor Association's labor standards and responsible sourcing principles in the provided context. Therefore, it cannot be confirmed from the given information that Amplifon follows FLA guidelines."}</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>Does the company adhere to labor standards and responsible sourcing principles set by Fair Labor Association, also called FLA? To adhere, the company must explicitly report it on the Sustainability report</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>ALERION.pdf</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company adhere to labor standards and responsible sourcing principles set by Fair Labor Association, also called FLA? To adhere, the company must explicitly report it on the Sustainability report', 'context': [Document(id='f707bf4b-5cae-4faa-8441-9437175abc1d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='in accordance with Alerion’s 2021 Green Bond Framework and will provide, starting one \nyear after issuance and on an annual basis until all the proceeds of the Green Bon d \nhave been allocated, a limited assurance report.  \nThis Third-Party Opinion made by External independent auditor on ALERION Green Bond \nReport is attached to this document. \n \n3-Reporting criteria \nAllocation: The amount of the “Green Bond 2021 - 2027 Proceeds” have been approved'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='8c8b278a-2039-4df6-a6f1-e4e4cd520379', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Pagina | 4  \n \n \nIn case of divestment, or if a project becomes ineligible, Alerion will strive to replace it \nby another Eligible Green Project on a best effort basis.   \n \n2.4- Reporting  \nAn annual report will be prepared and made available on Alerion’s website at \nwww.alerion.it, with the status of the Green Bond’s proceeds allocation, overview of the \nprojects financed or refinanced, and the environmental impact, until full allocation of \nproceeds.')], 'answer': 'Alerion: The provided context does not mention anything about adherence to labor standards or responsible sourcing principles set by the Fair Labor Association (FLA) or any reporting related to it in a Sustainability report.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>Is the company part of the alliance Platform Living Wage Financials and adhers to its principles? To adhere, the company must explicitly report it on the Sustainability report</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>ANTARES VISION.pdf</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>{'input': 'Is the company part of the alliance Platform Living Wage Financials and adhers to its principles? To adhere, the company must explicitly report it on the Sustainability report', 'context': [Document(id='2dbb90bd-c74b-43b3-bb1b-65c3b52f0e12', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 110, 'page_label': '111'}, page_content='Economic] \n   \n  \n2.28 Membership associations 04 Sustainability: the commitment of AV Group / \nAdherence to external initiatives and \nMemberships \n   \n  \n  Involvement of stakeholders           \n2.29 Approach to stakeholder engagement 05 Stakeholders / Stakeholder relations and \nengagement \n   \n  \n2.30 Collective bargaining agreements 11 Human Resources /HR Policies \n   \n  \n \n \n \n \nGRI Standards – Disclosure Material topics / Specific indicators'), Document(id='a60a397f-5869-4f73-8039-f4185d0c5f8c', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 8, 'page_label': '9'}, page_content="statements of Antares Vision S.p.A. Their Independent Auditors' Report is included in the appendix of this document. \n \nThe NFR is published on the Company's institutional website at Sustainability | Antares Vision and Investors | Antares Vision. \nFor further information, please contact the following address: sustainability@antaresvision.com.  \n \nAntares Vision S.p.A has notified the GRI (Global Reporting Initiative) of the use of the GRI Standards and the relative \nstatement of use."), Document(id='f10fce6f-1d2b-4a8c-ba59-d48046195b39', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 3, 'page_label': '4'}, page_content="This report is integral to what is for all intents and purposes, an increasingly concrete and strategic path to sustainability , \nwhich aims at deeply integrating ESG issues into every aspect of the Group's business. Indeed, our vision has always been \nconsistent with the objective of making our contribution to the sustainable development of the Company, i.e., one that \nresponds to the needs of the present without compromising the ability of future generations to satisfy their own.")], 'answer': "Antares Vision S.p.A. does not explicitly report being part of the Platform Living Wage Financials or adhering to its principles in the provided context. The context mentions the company's commitment to sustainability but doesn't specify adherence to this particular alliance. For confirmation, reviewing their sustainability report directly would be required."}</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>Is the company part of the alliance Platform Living Wage Financials and adhers to its principles? To adhere, the company must explicitly report it on the Sustainability report</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>AMPLIFON.pdf</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>{'input': 'Is the company part of the alliance Platform Living Wage Financials and adhers to its principles? To adhere, the company must explicitly report it on the Sustainability report', 'context': [Document(id='9891a1ce-2c42-4b91-b37d-1c300ec8106b', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 2, 'page_label': '1'}, page_content='To strengthen the contribution to the United Nations 2030 Agenda for Sustainable \nDevelopment, Amplifon takes part to United Nations Global Compact  through \nadherence, respect, and promotion of its Ten Principles.\nSustainability \nReport 2022'), Document(id='365fefe8-3254-4432-aa18-36f106997d02', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 7, 'page_label': '6'}, page_content='254/2016. From 2021, it also includes the progress made within the application of the Ten \nPrinciples promoted by the United Nations Global Compact , which we are signatories of. \nWith this Report, every year we seize the chance to communicate to all our stakeholders \nthe progress achieved with respect to the four areas of commitment formalized within \nour Sustainability Policy  ( Product &amp; Service Stewardship, People Empowerment,'), Document(id='07bb33fa-8bc4-41d4-87ec-130ac696aa07', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 6, 'page_label': '5'}, page_content='Nations Global Compact and commitment to \nthe Ten Principles in terms of human rights, \nworkers’ rights, environmental protection, \nand the fight against corruption, as well as \nthe 2030 Agenda of the United Nations for \nSustainable Development.\nWe are pleased to introduce our 2022 \nSustainability Report, containing the \naccomplishments achieved and the new \ninitiatives implemented in relation to our \nareas of commitment, aware that it is \nonly thanks to the active involvement of')], 'answer': 'Amplifon does not explicitly report being part of the Platform Living Wage Financials alliance in its Sustainability Report or mentioned adherence to its principles.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>Is the company part of the alliance Platform Living Wage Financials and adhers to its principles? To adhere, the company must explicitly report it on the Sustainability report</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>ALERION.pdf</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>{'input': 'Is the company part of the alliance Platform Living Wage Financials and adhers to its principles? To adhere, the company must explicitly report it on the Sustainability report', 'context': [Document(id='f707bf4b-5cae-4faa-8441-9437175abc1d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='in accordance with Alerion’s 2021 Green Bond Framework and will provide, starting one \nyear after issuance and on an annual basis until all the proceeds of the Green Bon d \nhave been allocated, a limited assurance report.  \nThis Third-Party Opinion made by External independent auditor on ALERION Green Bond \nReport is attached to this document. \n \n3-Reporting criteria \nAllocation: The amount of the “Green Bond 2021 - 2027 Proceeds” have been approved'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='8e92e81d-a44b-4d44-84b0-f8274704ad43', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 0, 'page_label': '1'}, page_content='Pagina | 0  \n \n \n  \nAnnual report prepared and made \navailable on Alerion’s website at \nwww.alerion.it, with the status of \nthe Green Bond’s proceeds \nallocation, overview of the projects \nfinanced or refinanced, and the \nenvironmental impact, until full \nallocation of proceeds. \nALERION \nGREEN BOND     \n2021–2027 \n_________ \nREPORT  \nYEAR 2022 \nUse of Proceeds')], 'answer': "Alerion's 2021 Green Bond Framework document does not provide any information on whether the company is part of the Platform Living Wage Financials alliance or adheres to its principles. To confirm such participation, one would need to review the company's Sustainability report for explicit mention."}</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>Does the company report in accordance with Human Rights Indicators for Business? Consider the company to report in accordance with Human Rights Indicators for Business only if explicitely written in the Sustainability Report</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>ANTARES VISION.pdf</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company report in accordance with Human Rights Indicators for Business? Consider the company to report in accordance with Human Rights Indicators for Business only if explicitely written in the Sustainability Report', 'context': [Document(id='2cd8b663-a885-431f-bd41-0824ba9060c9', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 111, 'page_label': '112'}, page_content='Sustainability report / NFR 2022 112 \n \n• Any possible notices / indicators (requirements) included in the standards referred to material themes, \nalthough not relevant or not applicable in respect to the characteristics of the business model and of the \nimpact are listed, however they are highlighted as “omitted” since they are not pertinent.  \n• On the other hand, evidence is given of omissions, if any, and of the related reasons for notices/indicators'), Document(id='c24ab15d-cfef-4356-ab09-02a4e013d0d4', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 61, 'page_label': '62'}, page_content='United Nations Human Rights (UNHR), 2011. Guiding Principles on Business and Human Rights. Implementing the United Nations “Protect, \nRespect and Remedy” Framework \nConvention on Biological Diversity (2022), Kunming-Montreal Global Biodiversity Framework \nSASB – Sustainability Accounting Standards – Materiality Finder  \nESRS – European Sustainability Reporting Standards (Draft) \nIFRS-S – International Financial Reporting Standards – Sustainability (Draft IFRS S1-S2)'), Document(id='64506eca-5a57-410a-ad35-cfb7169ad920', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 48, 'page_label': '49'}, page_content="Sustainability report / NFR 2022 49 \n \n \nThe Human Rights policy of Antares Vision Group was drawn up starting from the identification of the potentially most \nvulnerable elements within its value chain, t o ensure full respect for the human rights of all individuals connected to the \nGroup's activities. The policy regulates behaviours and establishes the position of AV Group in relation to topics such as")], 'answer': "Antares Vision Group's sustainability report does not explicitly state that it reports in accordance with Human Rights Indicators for Business."}</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>Does the company report in accordance with Human Rights Indicators for Business? Consider the company to report in accordance with Human Rights Indicators for Business only if explicitely written in the Sustainability Report</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>AMPLIFON.pdf</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company report in accordance with Human Rights Indicators for Business? Consider the company to report in accordance with Human Rights Indicators for Business only if explicitely written in the Sustainability Report', 'context': [Document(id='06e99e70-ce08-469b-b3a3-9e2d601fdfcf', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='and management methods, as well as the GRI Standards reported are described.\nArea Principle Reference GRI Standards\nHuman Rights\n1. Business should support and \nrespect the protection of human rights \nproclaimed at an international level\n2. Businesses should ensure that they are \nnot complicit in violations of human rights\n• Well-being and internal engagement\n• Business ethics and fighting corruption\n• Procurement and Supply Chain \nmanagement\n• Note on methodology\n• GRI 2-23: Policy commitment'), Document(id='365fefe8-3254-4432-aa18-36f106997d02', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 7, 'page_label': '6'}, page_content='254/2016. From 2021, it also includes the progress made within the application of the Ten \nPrinciples promoted by the United Nations Global Compact , which we are signatories of. \nWith this Report, every year we seize the chance to communicate to all our stakeholders \nthe progress achieved with respect to the four areas of commitment formalized within \nour Sustainability Policy  ( Product &amp; Service Stewardship, People Empowerment,'), Document(id='484a8eab-9638-4774-8fac-71a5e91e3600', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 185, 'page_label': '184'}, page_content='2-5: External assurance p. 180; 191-194\nActivities and workers\n2-6: Activities, value chain and other business relationships p. 23; 24; 26; 27; 49; 122\n2-7: Employees p. 68; 69; 158-162 Please note there are no non-guaranteed \nhours employees\n2-8: Workers who are not employees p. 68\nGovernance\n2-9: Governance structure and composition p. 28-30; 152-155\n2-10: Nomination and selection of the higest governance body \nReport on Corporate Governance and \nownership structure at 31 December 2022,')], 'answer': 'The company does not explicitly state in the provided context that it reports in accordance with Human Rights Indicators for Business in its Sustainability Report.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>Does the company report in accordance with Human Rights Indicators for Business? Consider the company to report in accordance with Human Rights Indicators for Business only if explicitely written in the Sustainability Report</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>ALERION.pdf</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company report in accordance with Human Rights Indicators for Business? Consider the company to report in accordance with Human Rights Indicators for Business only if explicitely written in the Sustainability Report', 'context': [Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='8e92e81d-a44b-4d44-84b0-f8274704ad43', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 0, 'page_label': '1'}, page_content='Pagina | 0  \n \n \n  \nAnnual report prepared and made \navailable on Alerion’s website at \nwww.alerion.it, with the status of \nthe Green Bond’s proceeds \nallocation, overview of the projects \nfinanced or refinanced, and the \nenvironmental impact, until full \nallocation of proceeds. \nALERION \nGREEN BOND     \n2021–2027 \n_________ \nREPORT  \nYEAR 2022 \nUse of Proceeds'), Document(id='8c8b278a-2039-4df6-a6f1-e4e4cd520379', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Pagina | 4  \n \n \nIn case of divestment, or if a project becomes ineligible, Alerion will strive to replace it \nby another Eligible Green Project on a best effort basis.   \n \n2.4- Reporting  \nAn annual report will be prepared and made available on Alerion’s website at \nwww.alerion.it, with the status of the Green Bond’s proceeds allocation, overview of the \nprojects financed or refinanced, and the environmental impact, until full allocation of \nproceeds.')], 'answer': "Alerion does not explicitly report in accordance with Human Rights Indicators for Business as per the given context. The provided details focus primarily on the Green Bond's proceeds, project financing, and environmental impact. There is no mention of a Sustainability Report addressing Human Rights Indicators for Business."}</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>Does the company adopt 6 principles set by Principles for responsible investment ? Please consider the company adopting the Principles for responsible investment  only if explicitely written in the Sustainability Report</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>ANTARES VISION.pdf</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company adopt 6 principles set by Principles for responsible investment ? Please consider the company adopting the Principles for responsible investment  only if explicitely written in the Sustainability Report', 'context': [Document(id='f10fce6f-1d2b-4a8c-ba59-d48046195b39', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 3, 'page_label': '4'}, page_content="This report is integral to what is for all intents and purposes, an increasingly concrete and strategic path to sustainability , \nwhich aims at deeply integrating ESG issues into every aspect of the Group's business. Indeed, our vision has always been \nconsistent with the objective of making our contribution to the sustainable development of the Company, i.e., one that \nresponds to the needs of the present without compromising the ability of future generations to satisfy their own."), Document(id='e1671f3b-8f3e-4872-8afc-8fc165c56ddf', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content='responsible for compliance with these principles and should seek clarification when appropriate. \nAntares Vision Group aligns its commitments in terms of policy with the development of its risk analysis a nd management \nmodel, which integrates an assessment of the economic, environmental and social impacts, the result of interaction with the \nmain responsible functions of the Group. For further details, please refer to the specific  section dedicated within this \ndocument.'), Document(id='54f69cf5-7085-4269-b796-999efbbce813', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 46, 'page_label': '47'}, page_content='Sustainability report / NFR 2022 47 \n \n▪ Minimum Safeguards - the same activities must also be conducted in compliance with the social criteria defined by the \nOECD guidelines and by the United Nations.  \n \nThe eligible activities are those activities included in the current taxonomy whether or not these assets meet any or all of the \ntechnical screening criteria set out in the taxonomy. \n \nAccounting principles')], 'answer': 'Antares Vision Group: It is not explicitly stated in the context given that the company adopts the six principles set by the Principles for Responsible Investment.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>Does the company adopt 6 principles set by Principles for responsible investment ? Please consider the company adopting the Principles for responsible investment  only if explicitely written in the Sustainability Report</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>AMPLIFON.pdf</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company adopt 6 principles set by Principles for responsible investment ? Please consider the company adopting the Principles for responsible investment  only if explicitely written in the Sustainability Report', 'context': [Document(id='10a2ea9b-20c4-4ec6-9aa6-75ca187040f6', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='CONTENT INDEX OF THE TEN PRINCIPLES\nOF THE UNITED NATIONS GLOBAL COMPACT \nAs a member of the UN Global Compact, Amplifon reports, in this Sustainability Report, the \nmain activities and progress made for the implementation and compliance with the Ten Prin-\nciples of the UNGC. Therefore, with a view to transparency and sharing with all stakeholders, \nthe table below illustrates, for each Principle, in which part of the document the main activities'), Document(id='365fefe8-3254-4432-aa18-36f106997d02', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 7, 'page_label': '6'}, page_content='254/2016. From 2021, it also includes the progress made within the application of the Ten \nPrinciples promoted by the United Nations Global Compact , which we are signatories of. \nWith this Report, every year we seize the chance to communicate to all our stakeholders \nthe progress achieved with respect to the four areas of commitment formalized within \nour Sustainability Policy  ( Product &amp; Service Stewardship, People Empowerment,'), Document(id='6c63013e-2a53-426c-84fe-5513198dc60d', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 176, 'page_label': '175'}, page_content='pliance, application and promotion of the Ten Principles of the Global Compact in the are -\nas of respect of human and labor rights, environmental protection and the fight against \ncorruption. The annex to the Document contains a correlation table between the contents \nof this Report and the Ten Principles of the UN Global Compact ( Content Index of the Ten \nPrinciples of the United Nations Global Compact ).\nEUROPEAN TAXONOMY')], 'answer': 'Amplifon’s Sustainability Report does not explicitly mention the adoption of the six principles set by the Principles for Responsible Investment.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>Does the company adopt 6 principles set by Principles for responsible investment ? Please consider the company adopting the Principles for responsible investment  only if explicitely written in the Sustainability Report</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>ALERION.pdf</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company adopt 6 principles set by Principles for responsible investment ? Please consider the company adopting the Principles for responsible investment  only if explicitely written in the Sustainability Report', 'context': [Document(id='d92ded8b-d43e-4c82-bbff-33a71d9d335f', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 2, 'page_label': '3'}, page_content="In particular, over the next years, Alerion will focus its strategy on the acceleration of \ngrowth with an increasingly broad geographical diversification in Italy, Spain and \nRomania, and on technological diversification, through a plan of investments in the solar \nsector. \n2- GREEN BOND FRAMEWORK \nIn order to increase transparency of the Alerion Green Bond 20 21 - 2027, Alerion has \npublished the “Alerion 2021 Green Bond Framework” in line with ICMA's Green Bond"), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='8c8b278a-2039-4df6-a6f1-e4e4cd520379', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Pagina | 4  \n \n \nIn case of divestment, or if a project becomes ineligible, Alerion will strive to replace it \nby another Eligible Green Project on a best effort basis.   \n \n2.4- Reporting  \nAn annual report will be prepared and made available on Alerion’s website at \nwww.alerion.it, with the status of the Green Bond’s proceeds allocation, overview of the \nprojects financed or refinanced, and the environmental impact, until full allocation of \nproceeds.')], 'answer': "Alerion's adoption of the Principles for Responsible Investment is not explicitly mentioned in the provided context, specifically in the Sustainability Report. Therefore, based on the available information, it is unclear if Alerion adopts these principles."}</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>Does the company adhere to Voluntary Principles on Security and Human Rights? Please consider the company adopting the  Voluntary Principles on Security and Human Rights only if explicitely written in the Sustainability Report</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>ANTARES VISION.pdf</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company adhere to Voluntary Principles on Security and Human Rights? Please consider the company adopting the  Voluntary Principles on Security and Human Rights only if explicitely written in the Sustainability Report', 'context': [Document(id='64506eca-5a57-410a-ad35-cfb7169ad920', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 48, 'page_label': '49'}, page_content="Sustainability report / NFR 2022 49 \n \n \nThe Human Rights policy of Antares Vision Group was drawn up starting from the identification of the potentially most \nvulnerable elements within its value chain, t o ensure full respect for the human rights of all individuals connected to the \nGroup's activities. The policy regulates behaviours and establishes the position of AV Group in relation to topics such as"), Document(id='c24ab15d-cfef-4356-ab09-02a4e013d0d4', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 61, 'page_label': '62'}, page_content='United Nations Human Rights (UNHR), 2011. Guiding Principles on Business and Human Rights. Implementing the United Nations “Protect, \nRespect and Remedy” Framework \nConvention on Biological Diversity (2022), Kunming-Montreal Global Biodiversity Framework \nSASB – Sustainability Accounting Standards – Materiality Finder  \nESRS – European Sustainability Reporting Standards (Draft) \nIFRS-S – International Financial Reporting Standards – Sustainability (Draft IFRS S1-S2)'), Document(id='bebc898a-2b45-453e-81c9-c8275f7216bf', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content='document.  \nLastly, specific methods have been adopted for checking the compliance of the behaviour of anyone acting on their own \nbehalf or within their work context, with the provisions of current legislation and with the rules of conduct established by the \npolicies and procedures adopted. \n \nHuman rights \n \nIn continuity with its values, the commitment defined in the Code of Ethics, AV Group adopted a specific Human Rights Policy')], 'answer': 'Antares Vision Group: The Sustainability Report does not explicitly mention the adoption of the Voluntary Principles on Security and Human Rights.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>Does the company adhere to Voluntary Principles on Security and Human Rights? Please consider the company adopting the  Voluntary Principles on Security and Human Rights only if explicitely written in the Sustainability Report</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>AMPLIFON.pdf</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company adhere to Voluntary Principles on Security and Human Rights? Please consider the company adopting the  Voluntary Principles on Security and Human Rights only if explicitely written in the Sustainability Report', 'context': [Document(id='45852781-8efa-4f79-8ced-fa5dbbd7e573', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 186, 'page_label': '185'}, page_content='Information Reference Notes/Omissions\n2-21: Annual total compensation ratio Remuneration Report 2023,\n“Executive Summary”\nStrategies, policies and practices\n2-22: Statement on sustainable development strategy p. 4; 5\n2-23: Policy commitments p. 30; 36; 41; 126; 132; 140\n2-24: Embedding policy commitments p. 30; 36; 41; 126; 132; 140\n2-25: Processes to remediate negative impacts\np.31; Report on Corporate Governance \nand ownership structure at 31 December \n2022, section 4 “Board of Directors”'), Document(id='365fefe8-3254-4432-aa18-36f106997d02', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 7, 'page_label': '6'}, page_content='254/2016. From 2021, it also includes the progress made within the application of the Ten \nPrinciples promoted by the United Nations Global Compact , which we are signatories of. \nWith this Report, every year we seize the chance to communicate to all our stakeholders \nthe progress achieved with respect to the four areas of commitment formalized within \nour Sustainability Policy  ( Product &amp; Service Stewardship, People Empowerment,'), Document(id='06e99e70-ce08-469b-b3a3-9e2d601fdfcf', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='and management methods, as well as the GRI Standards reported are described.\nArea Principle Reference GRI Standards\nHuman Rights\n1. Business should support and \nrespect the protection of human rights \nproclaimed at an international level\n2. Businesses should ensure that they are \nnot complicit in violations of human rights\n• Well-being and internal engagement\n• Business ethics and fighting corruption\n• Procurement and Supply Chain \nmanagement\n• Note on methodology\n• GRI 2-23: Policy commitment')], 'answer': 'The company does not explicitly mention adopting the Voluntary Principles on Security and Human Rights in the provided context. The information includes adherence to human rights principles, but it does not specifically reference the Voluntary Principles on Security and Human Rights.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>Does the company adhere to Voluntary Principles on Security and Human Rights? Please consider the company adopting the  Voluntary Principles on Security and Human Rights only if explicitely written in the Sustainability Report</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>ALERION.pdf</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company adhere to Voluntary Principles on Security and Human Rights? Please consider the company adopting the  Voluntary Principles on Security and Human Rights only if explicitely written in the Sustainability Report', 'context': [Document(id='8e92e81d-a44b-4d44-84b0-f8274704ad43', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 0, 'page_label': '1'}, page_content='Pagina | 0  \n \n \n  \nAnnual report prepared and made \navailable on Alerion’s website at \nwww.alerion.it, with the status of \nthe Green Bond’s proceeds \nallocation, overview of the projects \nfinanced or refinanced, and the \nenvironmental impact, until full \nallocation of proceeds. \nALERION \nGREEN BOND     \n2021–2027 \n_________ \nREPORT  \nYEAR 2022 \nUse of Proceeds'), Document(id='8c8b278a-2039-4df6-a6f1-e4e4cd520379', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='Pagina | 4  \n \n \nIn case of divestment, or if a project becomes ineligible, Alerion will strive to replace it \nby another Eligible Green Project on a best effort basis.   \n \n2.4- Reporting  \nAn annual report will be prepared and made available on Alerion’s website at \nwww.alerion.it, with the status of the Green Bond’s proceeds allocation, overview of the \nprojects financed or refinanced, and the environmental impact, until full allocation of \nproceeds.'), Document(id='f707bf4b-5cae-4faa-8441-9437175abc1d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='in accordance with Alerion’s 2021 Green Bond Framework and will provide, starting one \nyear after issuance and on an annual basis until all the proceeds of the Green Bon d \nhave been allocated, a limited assurance report.  \nThis Third-Party Opinion made by External independent auditor on ALERION Green Bond \nReport is attached to this document. \n \n3-Reporting criteria \nAllocation: The amount of the “Green Bond 2021 - 2027 Proceeds” have been approved')], 'answer': "Alerion's annual report and Green Bond documentation do not explicitly mention the company's adherence to the Voluntary Principles on Security and Human Rights."}</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>Does the company implement the practices recommended in the CEO Guide to Human Rights?</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>ANTARES VISION.pdf</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company implement the practices recommended in the CEO Guide to Human Rights?', 'context': [Document(id='5cb5e9ba-82dc-4639-8cfc-569ad2309e57', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="With the adoption of the Human Rights policy, which applies to all AV Group companies and provides for specific metho ds \nof implementation, employee training and monitoring, the Group intends to:  \n▪ strengthen its commitment to the protection of human rights in each country in which it operates,  \n▪ demonstrate the Group's awareness of the risks inherent in its business model, \n▪ promote the contents of the policy among its external stakeholders as well."), Document(id='75c5dbc0-d6b8-4368-927a-395136c411fc', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 91, 'page_label': '92'}, page_content='Vision Group as well as in compliance with the main international conventions, standards a nd recommendations on the \nsubject, namely, on the reference framework defined by the International Charter of Human Rights, by the Declaration of the \nInternational Labor Organization (ILO) on principles and rights in the workplace and by the eight core conventions of the ILO \n(No. 29, 87, 98, 100, 105, 111, 138, 182), and by the principles defined by the United Nations Global Compact in collaboration'), Document(id='7f37de2b-2de2-48b6-b0e3-bdfb2f414ac5', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 66, 'page_label': '67'}, page_content='Human Rights policies at Group level \n \n5.5  \n6 Occupational health and \nsafety  \nMaintaining high safety standards and minimum \ninjury rates \n \nEvaluation of the adoption and extension to other \nGroup companies of management systems and \nbest practices in the field of occupational health \nand safety \n \n8.8  \n7 Product quality / Customer \nhealth and safety \nMaintaining high quality standards of the solutions \noffered, also through screening and evaluation of')], 'answer': 'AV Group does not explicitly mention the CEO Guide to Human Rights in the context provided, so it is not clear whether the company implements the practices recommended in that guide.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>Does the company implement the practices recommended in the CEO Guide to Human Rights?</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>AMPLIFON.pdf</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company implement the practices recommended in the CEO Guide to Human Rights?', 'context': [Document(id='06e99e70-ce08-469b-b3a3-9e2d601fdfcf', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='and management methods, as well as the GRI Standards reported are described.\nArea Principle Reference GRI Standards\nHuman Rights\n1. Business should support and \nrespect the protection of human rights \nproclaimed at an international level\n2. Businesses should ensure that they are \nnot complicit in violations of human rights\n• Well-being and internal engagement\n• Business ethics and fighting corruption\n• Procurement and Supply Chain \nmanagement\n• Note on methodology\n• GRI 2-23: Policy commitment'), Document(id='45852781-8efa-4f79-8ced-fa5dbbd7e573', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 186, 'page_label': '185'}, page_content='Information Reference Notes/Omissions\n2-21: Annual total compensation ratio Remuneration Report 2023,\n“Executive Summary”\nStrategies, policies and practices\n2-22: Statement on sustainable development strategy p. 4; 5\n2-23: Policy commitments p. 30; 36; 41; 126; 132; 140\n2-24: Embedding policy commitments p. 30; 36; 41; 126; 132; 140\n2-25: Processes to remediate negative impacts\np.31; Report on Corporate Governance \nand ownership structure at 31 December \n2022, section 4 “Board of Directors”'), Document(id='7211d830-b72d-4e58-8b96-1aacac1013a7', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 150, 'page_label': '149'}, page_content='• DEIB (Diversity, Equity, Inclusion, Belonging) Policy and establishment of a DEIB Global Governance\n• Training, communication, and internal engagement activities\n• Implementation of specific action plans following the Global Engagement Survey “Your Voice”\n• Membership of the United Nations Global Compact \n• Smart Working Policy \n• Package of flexible benefits \n• Short and long-term incentive schemes\nAwareness-raising and \neducation on hearing well-\nbeing\nPotential reputational risks related to')], 'answer': 'The company is likely implementing the practices recommended in the CEO Guide to Human Rights as they have policy commitments related to human rights, DEIB policies, and are members of the United Nations Global Compact. They also have training, communication, and internal engagement activities focused on these areas. However, the specific implementation of the CEO Guide to Human Rights is not directly mentioned.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>Does the company implement the practices recommended in the CEO Guide to Human Rights?</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>ALERION.pdf</t>
-        </is>
-      </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company implement the practices recommended in the CEO Guide to Human Rights?', 'context': [Document(id='0286a4fd-14d3-46e6-a8c3-ddf45c3eb47d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='The Committee will be chaired by the Chairman of the Board of Directors, and composed \nof the other Board Executive Directors, together with the Chief Financial Officer and \nChief Operating Officer. \n \nThe Committee will be in charge of monitoring the selection and allocation of funds to \nEligible Green Projects and will be responsible for the following: \n \n- Identifying potential Eligible Green Projects;  \n \n- Reviewing and approving the selection against the eligibility'), Document(id='1603dfa0-95cf-4193-b970-a97988e35cc1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 1, 'page_label': '2'}, page_content='further in Europe, both in \nwind and solar sector. \n Alerion’s exclusive focus \non renewable energy \nimplies that sustainability \nis strictly embedded in our \nbusiness model. Our \noperations contribute \ndirectly to the reduction of \ngreenhouse gas (GHG) \nemissions and to the \npromotion of a system for \nsustainable territorial \ndevelopment. To this end, \nwe have in place a strong \nintegrated system for the \nassessment and \nmanagement of our'), Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.')], 'answer': 'Alerion does not provide specific information in the context regarding the implementation of the practices recommended in the CEO Guide to Human Rights. The focus in the provided content is on renewable energy projects and sustainability initiatives. Therefore, it cannot be confirmed whether Alerion follows the CEO Guide to Human Rights recommendations.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>Does the company endor the Universal Bill of Human Rights?</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>ANTARES VISION.pdf</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company endor the Universal Bill of Human Rights?', 'context': [Document(id='a5d4344c-bcff-442c-b0c1-8d73418a53a6', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="on 31 Jan uary 2023. This choice intends to reaffirm the importance of respect for human rights and strengthen the AV \nGroup's commitment to safeguarding them, in every country in which it operates. \n \nThe policy, available on the Antares Vision Group website  (Company Documents | Group Policies), has been developed in \naccordance with the main international human rights conventions, standards and recommendations (International Bill of"), Document(id='75c5dbc0-d6b8-4368-927a-395136c411fc', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 91, 'page_label': '92'}, page_content='Vision Group as well as in compliance with the main international conventions, standards a nd recommendations on the \nsubject, namely, on the reference framework defined by the International Charter of Human Rights, by the Declaration of the \nInternational Labor Organization (ILO) on principles and rights in the workplace and by the eight core conventions of the ILO \n(No. 29, 87, 98, 100, 105, 111, 138, 182), and by the principles defined by the United Nations Global Compact in collaboration'), Document(id='ebb08d4c-7962-44e5-ad11-1acca0c46725', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content='Human Rights and the Convention on the Rights of the Child of the United Nations, Fundamental Conventions of the \nInternational Labour Organization (ILO), Declaration of Principles and Fundamental Rights at Work, European Convention for \nthe Protection of Human Rights and Fundamental Freedoms (ECHR), as well as in compliance with the internal policies and \nprocedures of the Antares Vision Group.')], 'answer': 'Antares Vision Group endorses the International Bill of Human Rights as part of its commitment to safeguarding human rights in every country where it operates.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>Does the company endor the Universal Bill of Human Rights?</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>AMPLIFON.pdf</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company endor the Universal Bill of Human Rights?', 'context': [Document(id='a0026abd-c35d-47a4-a24f-0ab156e90b95', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 75, 'page_label': '74'}, page_content='WELL-BEING AND INTERNAL ENGAGEMENT \nIn line with the UN Global Compact principles, the Universal Declaration of Human Rights, \nand in compliance with the International Labor Organization Conventions on Fundamental \nHuman Rights, Amplifon is committed to complying with the fundamental human rights \nand labor rights in all the countries where we operate , both in business activities and \nunder the scope of relations with third parties, renouncing to all forms of exploitative for -'), Document(id='1ac9a44a-4757-4315-9432-a7ca6eb63415', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 175, 'page_label': '174'}, page_content="suppliers, in accordance with the principles and values set out in the Group's Code of \nEthics and Sustainability Policy and in full compliance with the Universal Declaration of \nHuman Rights and the International Labor Organization Conventions on fundamental \nhuman rights, as well as in line with the Principles of the UN Global Compact;\n ■ In light of the specific business model and the lack of any type of production activity,"), Document(id='67882b1c-f6ec-4a98-b1cf-143f28a4567a', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 124, 'page_label': '123'}, page_content='ciples of freedom and dignity of people and fundamental human rights, the exploitation of \nforced and child labor, as well as any form of personal discrimination. In support of this, since \n2019 all suppliers of hearing aids, whose contracts are subject to periodic renegotiation, are \nrequired to recognize and comply with the principles set forth in Amplifon’s Sustainability \nPolicy. In addition, at the start of 2022 a new Supplier Code of Conduct was adopted, defi-')], 'answer': 'Amplifon endorses the Universal Declaration of Human Rights, as stated in their commitment to comply with fundamental human rights.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>Does the company endor the Universal Bill of Human Rights?</t>
-        </is>
-      </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>ALERION.pdf</t>
-        </is>
-      </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company endor the Universal Bill of Human Rights?', 'context': [Document(id='1603dfa0-95cf-4193-b970-a97988e35cc1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 1, 'page_label': '2'}, page_content='further in Europe, both in \nwind and solar sector. \n Alerion’s exclusive focus \non renewable energy \nimplies that sustainability \nis strictly embedded in our \nbusiness model. Our \noperations contribute \ndirectly to the reduction of \ngreenhouse gas (GHG) \nemissions and to the \npromotion of a system for \nsustainable territorial \ndevelopment. To this end, \nwe have in place a strong \nintegrated system for the \nassessment and \nmanagement of our'), Document(id='0286a4fd-14d3-46e6-a8c3-ddf45c3eb47d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='The Committee will be chaired by the Chairman of the Board of Directors, and composed \nof the other Board Executive Directors, together with the Chief Financial Officer and \nChief Operating Officer. \n \nThe Committee will be in charge of monitoring the selection and allocation of funds to \nEligible Green Projects and will be responsible for the following: \n \n- Identifying potential Eligible Green Projects;  \n \n- Reviewing and approving the selection against the eligibility'), Document(id='d92ded8b-d43e-4c82-bbff-33a71d9d335f', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 2, 'page_label': '3'}, page_content="In particular, over the next years, Alerion will focus its strategy on the acceleration of \ngrowth with an increasingly broad geographical diversification in Italy, Spain and \nRomania, and on technological diversification, through a plan of investments in the solar \nsector. \n2- GREEN BOND FRAMEWORK \nIn order to increase transparency of the Alerion Green Bond 20 21 - 2027, Alerion has \npublished the “Alerion 2021 Green Bond Framework” in line with ICMA's Green Bond")], 'answer': 'Alerion does not specify in the provided context whether it endorses the Universal Bill of Human Rights.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>Does the company endor the Universal Declaration of Human Rights?</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>ANTARES VISION.pdf</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company endor the Universal Declaration of Human Rights?', 'context': [Document(id='a5d4344c-bcff-442c-b0c1-8d73418a53a6', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="on 31 Jan uary 2023. This choice intends to reaffirm the importance of respect for human rights and strengthen the AV \nGroup's commitment to safeguarding them, in every country in which it operates. \n \nThe policy, available on the Antares Vision Group website  (Company Documents | Group Policies), has been developed in \naccordance with the main international human rights conventions, standards and recommendations (International Bill of"), Document(id='75c5dbc0-d6b8-4368-927a-395136c411fc', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 91, 'page_label': '92'}, page_content='Vision Group as well as in compliance with the main international conventions, standards a nd recommendations on the \nsubject, namely, on the reference framework defined by the International Charter of Human Rights, by the Declaration of the \nInternational Labor Organization (ILO) on principles and rights in the workplace and by the eight core conventions of the ILO \n(No. 29, 87, 98, 100, 105, 111, 138, 182), and by the principles defined by the United Nations Global Compact in collaboration'), Document(id='ebb08d4c-7962-44e5-ad11-1acca0c46725', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content='Human Rights and the Convention on the Rights of the Child of the United Nations, Fundamental Conventions of the \nInternational Labour Organization (ILO), Declaration of Principles and Fundamental Rights at Work, European Convention for \nthe Protection of Human Rights and Fundamental Freedoms (ECHR), as well as in compliance with the internal policies and \nprocedures of the Antares Vision Group.')], 'answer': 'Antares Vision Group endorses the Universal Declaration of Human Rights as reflected in their commitment to adhere to international human rights conventions and standards.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>Does the company endor the Universal Declaration of Human Rights?</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>AMPLIFON.pdf</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company endor the Universal Declaration of Human Rights?', 'context': [Document(id='a0026abd-c35d-47a4-a24f-0ab156e90b95', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 75, 'page_label': '74'}, page_content='WELL-BEING AND INTERNAL ENGAGEMENT \nIn line with the UN Global Compact principles, the Universal Declaration of Human Rights, \nand in compliance with the International Labor Organization Conventions on Fundamental \nHuman Rights, Amplifon is committed to complying with the fundamental human rights \nand labor rights in all the countries where we operate , both in business activities and \nunder the scope of relations with third parties, renouncing to all forms of exploitative for -'), Document(id='1ac9a44a-4757-4315-9432-a7ca6eb63415', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 175, 'page_label': '174'}, page_content="suppliers, in accordance with the principles and values set out in the Group's Code of \nEthics and Sustainability Policy and in full compliance with the Universal Declaration of \nHuman Rights and the International Labor Organization Conventions on fundamental \nhuman rights, as well as in line with the Principles of the UN Global Compact;\n ■ In light of the specific business model and the lack of any type of production activity,"), Document(id='ce127729-ee22-49ad-8c9a-7e4c484e8782', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 73, 'page_label': '72'}, page_content="WE SUBSCRIBED TO THE UNITED NATIONS WOMEN’S \nEMPOWERMENT PRINCIPLES\n \nAt the beginning of 2022, we have subscribed to the Women's Empowerment Principles \n(WEPs) established by the UN Women and UN Global Compact, a collection of principles \nthat guide organizations in promoting gender equality and the empowerment of women \nin the workplace, the market and the community. In line with international standards \non labour and human rights, the WEPs are based on the recognition of the role and")], 'answer': 'Amplifon endorses the Universal Declaration of Human Rights.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>Does the company endor the Universal Declaration of Human Rights?</t>
-        </is>
-      </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>ALERION.pdf</t>
-        </is>
-      </c>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company endor the Universal Declaration of Human Rights?', 'context': [Document(id='1603dfa0-95cf-4193-b970-a97988e35cc1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 1, 'page_label': '2'}, page_content='further in Europe, both in \nwind and solar sector. \n Alerion’s exclusive focus \non renewable energy \nimplies that sustainability \nis strictly embedded in our \nbusiness model. Our \noperations contribute \ndirectly to the reduction of \ngreenhouse gas (GHG) \nemissions and to the \npromotion of a system for \nsustainable territorial \ndevelopment. To this end, \nwe have in place a strong \nintegrated system for the \nassessment and \nmanagement of our'), Document(id='0286a4fd-14d3-46e6-a8c3-ddf45c3eb47d', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='The Committee will be chaired by the Chairman of the Board of Directors, and composed \nof the other Board Executive Directors, together with the Chief Financial Officer and \nChief Operating Officer. \n \nThe Committee will be in charge of monitoring the selection and allocation of funds to \nEligible Green Projects and will be responsible for the following: \n \n- Identifying potential Eligible Green Projects;  \n \n- Reviewing and approving the selection against the eligibility'), Document(id='e9ebe77f-cd30-4024-a8ad-93fd6424f492', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Energy”), 9 (“Industry Innovation and Infrastructure”) and 13 (“Climate Action”). \n \n \n2.2- Process for Project Evaluation and Selection  \n \nAlerion’s Green Bond 2021 – 2027 Framework is for the financing and refinancing of \nwind and/or solar power generation projects, as previously described. \nAlerion will establish a Green Bond Committee (“the Committee”) to oversee the Green \nBond implementation and the allocation process.')], 'answer': "Alerion's context does not provide specific information about endorsing the Universal Declaration of Human Rights."}</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>Does the company endor the UN Guiding Principles, aslo called UNGPs?</t>
-        </is>
-      </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>ANTARES VISION.pdf</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company endor the UN Guiding Principles, aslo called UNGPs?', 'context': [Document(id='c24ab15d-cfef-4356-ab09-02a4e013d0d4', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 61, 'page_label': '62'}, page_content='United Nations Human Rights (UNHR), 2011. Guiding Principles on Business and Human Rights. Implementing the United Nations “Protect, \nRespect and Remedy” Framework \nConvention on Biological Diversity (2022), Kunming-Montreal Global Biodiversity Framework \nSASB – Sustainability Accounting Standards – Materiality Finder  \nESRS – European Sustainability Reporting Standards (Draft) \nIFRS-S – International Financial Reporting Standards – Sustainability (Draft IFRS S1-S2)'), Document(id='75c5dbc0-d6b8-4368-927a-395136c411fc', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 91, 'page_label': '92'}, page_content='Vision Group as well as in compliance with the main international conventions, standards a nd recommendations on the \nsubject, namely, on the reference framework defined by the International Charter of Human Rights, by the Declaration of the \nInternational Labor Organization (ILO) on principles and rights in the workplace and by the eight core conventions of the ILO \n(No. 29, 87, 98, 100, 105, 111, 138, 182), and by the principles defined by the United Nations Global Compact in collaboration'), Document(id='bebc898a-2b45-453e-81c9-c8275f7216bf', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content='document.  \nLastly, specific methods have been adopted for checking the compliance of the behaviour of anyone acting on their own \nbehalf or within their work context, with the provisions of current legislation and with the rules of conduct established by the \npolicies and procedures adopted. \n \nHuman rights \n \nIn continuity with its values, the commitment defined in the Code of Ethics, AV Group adopted a specific Human Rights Policy')], 'answer': 'Vision Group, in compliance with international conventions and standards, likely endorses frameworks like the UN Guiding Principles on Business and Human Rights, as indicated by their adherence to similar principles and conventions.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>Does the company endor the UN Guiding Principles, aslo called UNGPs?</t>
-        </is>
-      </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>AMPLIFON.pdf</t>
-        </is>
-      </c>
-      <c r="C162" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company endor the UN Guiding Principles, aslo called UNGPs?', 'context': [Document(id='ce127729-ee22-49ad-8c9a-7e4c484e8782', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 73, 'page_label': '72'}, page_content="WE SUBSCRIBED TO THE UNITED NATIONS WOMEN’S \nEMPOWERMENT PRINCIPLES\n \nAt the beginning of 2022, we have subscribed to the Women's Empowerment Principles \n(WEPs) established by the UN Women and UN Global Compact, a collection of principles \nthat guide organizations in promoting gender equality and the empowerment of women \nin the workplace, the market and the community. In line with international standards \non labour and human rights, the WEPs are based on the recognition of the role and"), Document(id='10a2ea9b-20c4-4ec6-9aa6-75ca187040f6', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 191, 'page_label': '190'}, page_content='CONTENT INDEX OF THE TEN PRINCIPLES\nOF THE UNITED NATIONS GLOBAL COMPACT \nAs a member of the UN Global Compact, Amplifon reports, in this Sustainability Report, the \nmain activities and progress made for the implementation and compliance with the Ten Prin-\nciples of the UNGC. Therefore, with a view to transparency and sharing with all stakeholders, \nthe table below illustrates, for each Principle, in which part of the document the main activities'), Document(id='a0026abd-c35d-47a4-a24f-0ab156e90b95', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 75, 'page_label': '74'}, page_content='WELL-BEING AND INTERNAL ENGAGEMENT \nIn line with the UN Global Compact principles, the Universal Declaration of Human Rights, \nand in compliance with the International Labor Organization Conventions on Fundamental \nHuman Rights, Amplifon is committed to complying with the fundamental human rights \nand labor rights in all the countries where we operate , both in business activities and \nunder the scope of relations with third parties, renouncing to all forms of exploitative for -')], 'answer': 'Amplifon does not specifically mention endorsing the UN Guiding Principles (UNGPs) in the provided context.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="inlineStr">
-        <is>
-          <t>Does the company endor the UN Guiding Principles, aslo called UNGPs?</t>
-        </is>
-      </c>
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>ALERION.pdf</t>
-        </is>
-      </c>
-      <c r="C163" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company endor the UN Guiding Principles, aslo called UNGPs?', 'context': [Document(id='8d2915a9-edec-472d-8bde-baa6034447b2', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 2, 'page_label': '3'}, page_content='Principles 2021 edition (“GBP”). The GBP core components are described as follow: \n1) Use of Proceeds \n2) Process for Project Evaluation and Selection \n3) Management of Proceeds \n4) Reporting \n5) External Review – Annual assurance report \n2.1- “ALERION GREEN BOND 2021 – 2027”- USE OF PROCEEDS \n \nAlerion intends to use the proceeds of the Green Bond 2021 – 2027 as follows: \n \n- the early redemption of the “Euro 150 million Alerion Clean Power \nS.p.A. 2018-2024” bond (ISIN IT0005333627);'), Document(id='649a691d-f955-4d58-a784-64b1a0ddf657', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 4, 'page_label': '5'}, page_content='by Alerion’s Green Bond Committee on the meeting held on March 09, 2023.  \n \n1 The above -listed indicators are subject to the availability of information and baseline data, and are based on \nmethodologies that will be made publicly available.'), Document(id='1603dfa0-95cf-4193-b970-a97988e35cc1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 1, 'page_label': '2'}, page_content='further in Europe, both in \nwind and solar sector. \n Alerion’s exclusive focus \non renewable energy \nimplies that sustainability \nis strictly embedded in our \nbusiness model. Our \noperations contribute \ndirectly to the reduction of \ngreenhouse gas (GHG) \nemissions and to the \npromotion of a system for \nsustainable territorial \ndevelopment. To this end, \nwe have in place a strong \nintegrated system for the \nassessment and \nmanagement of our')], 'answer': 'Alerion does not specifically mention endorsing the UN Guiding Principles (UNGPs) in the provided context.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>Does the company endor the European Convention for the Protection of Human Rights and Fundamental Freedoms?</t>
-        </is>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>ANTARES VISION.pdf</t>
-        </is>
-      </c>
-      <c r="C164" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company endor the European Convention for the Protection of Human Rights and Fundamental Freedoms?', 'context': [Document(id='ebb08d4c-7962-44e5-ad11-1acca0c46725', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content='Human Rights and the Convention on the Rights of the Child of the United Nations, Fundamental Conventions of the \nInternational Labour Organization (ILO), Declaration of Principles and Fundamental Rights at Work, European Convention for \nthe Protection of Human Rights and Fundamental Freedoms (ECHR), as well as in compliance with the internal policies and \nprocedures of the Antares Vision Group.'), Document(id='a5d4344c-bcff-442c-b0c1-8d73418a53a6', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="on 31 Jan uary 2023. This choice intends to reaffirm the importance of respect for human rights and strengthen the AV \nGroup's commitment to safeguarding them, in every country in which it operates. \n \nThe policy, available on the Antares Vision Group website  (Company Documents | Group Policies), has been developed in \naccordance with the main international human rights conventions, standards and recommendations (International Bill of"), Document(id='75c5dbc0-d6b8-4368-927a-395136c411fc', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 91, 'page_label': '92'}, page_content='Vision Group as well as in compliance with the main international conventions, standards a nd recommendations on the \nsubject, namely, on the reference framework defined by the International Charter of Human Rights, by the Declaration of the \nInternational Labor Organization (ILO) on principles and rights in the workplace and by the eight core conventions of the ILO \n(No. 29, 87, 98, 100, 105, 111, 138, 182), and by the principles defined by the United Nations Global Compact in collaboration')], 'answer': 'Antares Vision Group endorses the European Convention for the Protection of Human Rights and Fundamental Freedoms (ECHR).'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t>Does the company endor the European Convention for the Protection of Human Rights and Fundamental Freedoms?</t>
-        </is>
-      </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>AMPLIFON.pdf</t>
-        </is>
-      </c>
-      <c r="C165" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company endor the European Convention for the Protection of Human Rights and Fundamental Freedoms?', 'context': [Document(id='a0026abd-c35d-47a4-a24f-0ab156e90b95', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 75, 'page_label': '74'}, page_content='WELL-BEING AND INTERNAL ENGAGEMENT \nIn line with the UN Global Compact principles, the Universal Declaration of Human Rights, \nand in compliance with the International Labor Organization Conventions on Fundamental \nHuman Rights, Amplifon is committed to complying with the fundamental human rights \nand labor rights in all the countries where we operate , both in business activities and \nunder the scope of relations with third parties, renouncing to all forms of exploitative for -'), Document(id='25ec72d4-687e-40b4-a28b-466ed546d279', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 127, 'page_label': '126'}, page_content='practices (both direct or via third parties), illegal favors, collusive behavior and procuring \nadvantages.\n ■ the management of human resources , including the fight against any form of \ndiscrimination, rejecting exploitation of child labor, safeguarding the principle of equal \nopportunities for all aspects of the working relationship, preserving a healthy, safe work \nenvironment, protecting the environment, the fight against any form of a harassment in \nthe workplace and responsibility for assets.'), Document(id='1ac9a44a-4757-4315-9432-a7ca6eb63415', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 175, 'page_label': '174'}, page_content="suppliers, in accordance with the principles and values set out in the Group's Code of \nEthics and Sustainability Policy and in full compliance with the Universal Declaration of \nHuman Rights and the International Labor Organization Conventions on fundamental \nhuman rights, as well as in line with the Principles of the UN Global Compact;\n ■ In light of the specific business model and the lack of any type of production activity,")], 'answer': 'Amplifon does not specifically mention endorsing the European Convention for the Protection of Human Rights and Fundamental Freedoms. The company aligns its practices with the UN Global Compact, the Universal Declaration of Human Rights, and the International Labor Organization Conventions.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t>Does the company endor the European Convention for the Protection of Human Rights and Fundamental Freedoms?</t>
-        </is>
-      </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>ALERION.pdf</t>
-        </is>
-      </c>
-      <c r="C166" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company endor the European Convention for the Protection of Human Rights and Fundamental Freedoms?', 'context': [Document(id='1603dfa0-95cf-4193-b970-a97988e35cc1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 1, 'page_label': '2'}, page_content='further in Europe, both in \nwind and solar sector. \n Alerion’s exclusive focus \non renewable energy \nimplies that sustainability \nis strictly embedded in our \nbusiness model. Our \noperations contribute \ndirectly to the reduction of \ngreenhouse gas (GHG) \nemissions and to the \npromotion of a system for \nsustainable territorial \ndevelopment. To this end, \nwe have in place a strong \nintegrated system for the \nassessment and \nmanagement of our'), Document(id='6fef9802-f6ae-42bc-b253-3b10fc4c909f', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 5, 'page_label': '6'}, page_content='The Eligible Green Projects will be constructed according to Eur opean Union \nand national legislation that requires specific environmental screening before \nreceiving the building permit. \n  \n200\n100% ALLOCATED\nAlerion Green Bond 2021 \n -\n 2027 \nProceeds\nProceeds Allocated\n Proceeds not yet allocated\n100% of the proceeds \nof the Alerion Green \nBond 2021 – 2027 (Eur \n200 mln) were \nallocated. \n88,3% of the proceeds \nof the Alerion Green \nBond 2021 – 2027 (Eur \n176,5 mln) were \nallocated in 2021.'), Document(id='225f1439-813f-45a4-9043-28eea423ba61', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Pagina | 3  \n \nThe acquisition of operating wind farms and/or solar farms includes both the acquisition \nof operating assets as well as the acquisition of companies owning authorized and / or \noperating assets. Eligible Green Projects will be located in Europe, in particular in Italy, \nRomania and Spain and are expected to be constructed or acquired during the 24 \nmonths following the issuance of the Green Bond. \n \nThe Eligible Green Projects will be constructed according to European Union and national')], 'answer': 'Alerion: The context provided does not specify whether the company endorses the European Convention for the Protection of Human Rights and Fundamental Freedoms.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>Does the company endor the European Convention for the Protection of Human Rights and Fundamental Freedoms?</t>
-        </is>
-      </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>ANTARES VISION.pdf</t>
-        </is>
-      </c>
-      <c r="C167" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company endor the European Convention for the Protection of Human Rights and Fundamental Freedoms?', 'context': [Document(id='ebb08d4c-7962-44e5-ad11-1acca0c46725', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content='Human Rights and the Convention on the Rights of the Child of the United Nations, Fundamental Conventions of the \nInternational Labour Organization (ILO), Declaration of Principles and Fundamental Rights at Work, European Convention for \nthe Protection of Human Rights and Fundamental Freedoms (ECHR), as well as in compliance with the internal policies and \nprocedures of the Antares Vision Group.'), Document(id='a5d4344c-bcff-442c-b0c1-8d73418a53a6', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 47, 'page_label': '48'}, page_content="on 31 Jan uary 2023. This choice intends to reaffirm the importance of respect for human rights and strengthen the AV \nGroup's commitment to safeguarding them, in every country in which it operates. \n \nThe policy, available on the Antares Vision Group website  (Company Documents | Group Policies), has been developed in \naccordance with the main international human rights conventions, standards and recommendations (International Bill of"), Document(id='75c5dbc0-d6b8-4368-927a-395136c411fc', metadata={'producer': 'Microsoft® Word per Microsoft 365', 'creator': 'Microsoft® Word per Microsoft 365', 'creationdate': '2023-03-31T10:43:12+02:00', 'author': 'Adriana Buccomino', 'moddate': '2023-03-31T10:46:51+02:00', 'source': 'uploaded_files\\ANTARES VISION.pdf', 'total_pages': 123, 'page': 91, 'page_label': '92'}, page_content='Vision Group as well as in compliance with the main international conventions, standards a nd recommendations on the \nsubject, namely, on the reference framework defined by the International Charter of Human Rights, by the Declaration of the \nInternational Labor Organization (ILO) on principles and rights in the workplace and by the eight core conventions of the ILO \n(No. 29, 87, 98, 100, 105, 111, 138, 182), and by the principles defined by the United Nations Global Compact in collaboration')], 'answer': 'Antares Vision Group endorses the European Convention for the Protection of Human Rights and Fundamental Freedoms.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>Does the company endor the European Convention for the Protection of Human Rights and Fundamental Freedoms?</t>
-        </is>
-      </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>AMPLIFON.pdf</t>
-        </is>
-      </c>
-      <c r="C168" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company endor the European Convention for the Protection of Human Rights and Fundamental Freedoms?', 'context': [Document(id='a0026abd-c35d-47a4-a24f-0ab156e90b95', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 75, 'page_label': '74'}, page_content='WELL-BEING AND INTERNAL ENGAGEMENT \nIn line with the UN Global Compact principles, the Universal Declaration of Human Rights, \nand in compliance with the International Labor Organization Conventions on Fundamental \nHuman Rights, Amplifon is committed to complying with the fundamental human rights \nand labor rights in all the countries where we operate , both in business activities and \nunder the scope of relations with third parties, renouncing to all forms of exploitative for -'), Document(id='25ec72d4-687e-40b4-a28b-466ed546d279', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 127, 'page_label': '126'}, page_content='practices (both direct or via third parties), illegal favors, collusive behavior and procuring \nadvantages.\n ■ the management of human resources , including the fight against any form of \ndiscrimination, rejecting exploitation of child labor, safeguarding the principle of equal \nopportunities for all aspects of the working relationship, preserving a healthy, safe work \nenvironment, protecting the environment, the fight against any form of a harassment in \nthe workplace and responsibility for assets.'), Document(id='1ac9a44a-4757-4315-9432-a7ca6eb63415', metadata={'producer': 'Adobe PDF Library 17.0', 'creator': 'Adobe InDesign 18.1 (Macintosh)', 'creationdate': '2023-03-15T08:44:57+00:00', 'moddate': '2023-03-15T14:36:27+00:00', 'trapped': '/false', 'source': 'uploaded_files\\AMPLIFON.pdf', 'total_pages': 198, 'page': 175, 'page_label': '174'}, page_content="suppliers, in accordance with the principles and values set out in the Group's Code of \nEthics and Sustainability Policy and in full compliance with the Universal Declaration of \nHuman Rights and the International Labor Organization Conventions on fundamental \nhuman rights, as well as in line with the Principles of the UN Global Compact;\n ■ In light of the specific business model and the lack of any type of production activity,")], 'answer': 'Amplifon does not specifically mention endorsing the European Convention for the Protection of Human Rights and Fundamental Freedoms in the provided context. The company does endorse the UN Global Compact principles, the Universal Declaration of Human Rights, and International Labor Organization Conventions on Fundamental Human Rights.'}</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>Does the company endor the European Convention for the Protection of Human Rights and Fundamental Freedoms?</t>
-        </is>
-      </c>
-      <c r="B169" t="inlineStr">
-        <is>
-          <t>ALERION.pdf</t>
-        </is>
-      </c>
-      <c r="C169" t="inlineStr">
-        <is>
-          <t>{'input': 'Does the company endor the European Convention for the Protection of Human Rights and Fundamental Freedoms?', 'context': [Document(id='1603dfa0-95cf-4193-b970-a97988e35cc1', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 1, 'page_label': '2'}, page_content='further in Europe, both in \nwind and solar sector. \n Alerion’s exclusive focus \non renewable energy \nimplies that sustainability \nis strictly embedded in our \nbusiness model. Our \noperations contribute \ndirectly to the reduction of \ngreenhouse gas (GHG) \nemissions and to the \npromotion of a system for \nsustainable territorial \ndevelopment. To this end, \nwe have in place a strong \nintegrated system for the \nassessment and \nmanagement of our'), Document(id='6fef9802-f6ae-42bc-b253-3b10fc4c909f', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 5, 'page_label': '6'}, page_content='The Eligible Green Projects will be constructed according to Eur opean Union \nand national legislation that requires specific environmental screening before \nreceiving the building permit. \n  \n200\n100% ALLOCATED\nAlerion Green Bond 2021 \n -\n 2027 \nProceeds\nProceeds Allocated\n Proceeds not yet allocated\n100% of the proceeds \nof the Alerion Green \nBond 2021 – 2027 (Eur \n200 mln) were \nallocated. \n88,3% of the proceeds \nof the Alerion Green \nBond 2021 – 2027 (Eur \n176,5 mln) were \nallocated in 2021.'), Document(id='225f1439-813f-45a4-9043-28eea423ba61', metadata={'producer': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creator': 'Adobe Acrobat Pro (32-bit) 23.1.20093', 'creationdate': '2023-04-05T10:52:00+02:00', 'author': 'Alerion', 'moddate': '2023-04-05T12:53:03+02:00', 'subject': 'Use of Proceeds', 'title': 'Annual Report 2022 - Use of proceeds', 'source': 'uploaded_files\\ALERION.pdf', 'total_pages': 11, 'page': 3, 'page_label': '4'}, page_content='Pagina | 3  \n \nThe acquisition of operating wind farms and/or solar farms includes both the acquisition \nof operating assets as well as the acquisition of companies owning authorized and / or \noperating assets. Eligible Green Projects will be located in Europe, in particular in Italy, \nRomania and Spain and are expected to be constructed or acquired during the 24 \nmonths following the issuance of the Green Bond. \n \nThe Eligible Green Projects will be constructed according to European Union and national')], 'answer': "Alerion does not explicitly mention endorsing the European Convention for the Protection of Human Rights and Fundamental Freedoms in the provided context. Their focus is primarily on renewable energy and sustainability. I don't know if they endorse this convention based on the given information."}</t>
+          <t>Question: Does the company endorse the European Convention for the Protection of Human Rights and Fundamental Freedoms?
+Answer: Yes
+Evidence: "European Convention for the Protection of Human Rights and Fundamental Freedoms (ECHR), as well as in compliance with the internal policies and procedures of the Antares Vision Group."
+Location: Sustainability Report, not specified</t>
         </is>
       </c>
     </row>

</xml_diff>